<commit_message>
docs: record published tiger motion and 75 qualified symbol packs
</commit_message>
<xml_diff>
--- a/doc_web_interne/docs/suivi-symboles/suivi-240-symboles-6-langues.xlsx
+++ b/doc_web_interne/docs/suivi-symboles/suivi-240-symboles-6-langues.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Suivi symboles" sheetId="1" r:id="Ra5b4bd929bec4c98"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Suivi symboles" sheetId="1" r:id="R18faf94eba7249f6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -899,14 +899,14 @@
       </x:c>
       <x:c r="B5" s="9" t="n">
         <x:f>COUNTIF(W11:W250,"6/6 actuelles")</x:f>
-        <x:v>74</x:v>
+        <x:v>75</x:v>
       </x:c>
       <x:c r="C5" s="3" t="str">
         <x:v>QA 2560 px</x:v>
       </x:c>
       <x:c r="D5" s="9" t="n">
         <x:f>COUNTIF(X11:X250,"6/6 actuelles")</x:f>
-        <x:v>74</x:v>
+        <x:v>75</x:v>
       </x:c>
       <x:c r="E5" s="3" t="str">
         <x:v>Accord Thanh</x:v>
@@ -980,7 +980,7 @@
     </x:row>
     <x:row r="7" ht="20" customHeight="1">
       <x:c r="A7" s="7" t="str">
-        <x:v>74 packs standards et Tigre. Commun = cadre partagé sans pack complet. Les contrôles PR474 restent historiques.</x:v>
+        <x:v>75 packs sur le moteur commun. Commun = cadre partagé sans pack complet. Les contrôles PR474 restent historiques.</x:v>
       </x:c>
       <x:c r="B7" s="7"/>
       <x:c r="C7" s="7"/>
@@ -1013,7 +1013,7 @@
     </x:row>
     <x:row r="8" ht="20" customHeight="1">
       <x:c r="A8" s="7" t="str">
-        <x:v>Source : rapport canonique du 20/10/2026, empreinte 7f469489c44ab0eb. Révision : 1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>Source : rapport canonique du 20/10/2026, empreinte 182353099e1c6ce6. Révision : 76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="B8" s="7"/>
       <x:c r="C8" s="7"/>
@@ -1234,10 +1234,10 @@
         <x:v>Atlas</x:v>
       </x:c>
       <x:c r="W11" s="24" t="str">
-        <x:v>À corriger</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="X11" s="24" t="str">
-        <x:v>À corriger</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="Y11" s="24" t="str">
         <x:v>Historique</x:v>
@@ -1246,10 +1246,10 @@
         <x:v>Publié 6/6</x:v>
       </x:c>
       <x:c r="AA11" s="23" t="str">
-        <x:v>Animer la plaque et les trois vignettes dans six langues. Consigner la QA actuelle des six langues. Consigner l’accord de Thanh. Requalifier les preuves historiques</x:v>
+        <x:v>Consigner l’accord de Thanh. Requalifier les preuves historiques</x:v>
       </x:c>
       <x:c r="AB11" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC11" s="21" t="str">
         <x:v>En cours</x:v>
@@ -1340,7 +1340,7 @@
         <x:v>Consigner l’accord de Thanh. Requalifier les preuves historiques</x:v>
       </x:c>
       <x:c r="AB12" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC12" s="21" t="str">
         <x:v>En cours</x:v>
@@ -1431,7 +1431,7 @@
         <x:v>Consigner l’accord de Thanh. Requalifier les preuves historiques</x:v>
       </x:c>
       <x:c r="AB13" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC13" s="21" t="str">
         <x:v>En cours</x:v>
@@ -1522,7 +1522,7 @@
         <x:v>Consigner l’accord de Thanh. Requalifier les preuves historiques</x:v>
       </x:c>
       <x:c r="AB14" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC14" s="21" t="str">
         <x:v>En cours</x:v>
@@ -1613,7 +1613,7 @@
         <x:v>Consigner l’accord de Thanh. Requalifier les preuves historiques</x:v>
       </x:c>
       <x:c r="AB15" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC15" s="21" t="str">
         <x:v>En cours</x:v>
@@ -1704,7 +1704,7 @@
         <x:v>Consigner l’accord de Thanh. Requalifier les preuves historiques</x:v>
       </x:c>
       <x:c r="AB16" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC16" s="21" t="str">
         <x:v>En cours</x:v>
@@ -1795,7 +1795,7 @@
         <x:v>Consigner l’accord de Thanh. Requalifier les preuves historiques</x:v>
       </x:c>
       <x:c r="AB17" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC17" s="21" t="str">
         <x:v>En cours</x:v>
@@ -1886,7 +1886,7 @@
         <x:v>Consigner l’accord de Thanh. Requalifier les preuves historiques</x:v>
       </x:c>
       <x:c r="AB18" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC18" s="21" t="str">
         <x:v>En cours</x:v>
@@ -1977,7 +1977,7 @@
         <x:v>Consigner l’accord de Thanh. Requalifier les preuves historiques</x:v>
       </x:c>
       <x:c r="AB19" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC19" s="21" t="str">
         <x:v>En cours</x:v>
@@ -2068,7 +2068,7 @@
         <x:v>Consigner l’accord de Thanh. Requalifier les preuves historiques</x:v>
       </x:c>
       <x:c r="AB20" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC20" s="21" t="str">
         <x:v>En cours</x:v>
@@ -2159,7 +2159,7 @@
         <x:v>Consigner l’accord de Thanh. Requalifier les preuves historiques</x:v>
       </x:c>
       <x:c r="AB21" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC21" s="21" t="str">
         <x:v>En cours</x:v>
@@ -2250,7 +2250,7 @@
         <x:v>Consigner l’accord de Thanh. Requalifier les preuves historiques</x:v>
       </x:c>
       <x:c r="AB22" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC22" s="21" t="str">
         <x:v>En cours</x:v>
@@ -2341,7 +2341,7 @@
         <x:v>Consigner l’accord de Thanh. Requalifier les preuves historiques</x:v>
       </x:c>
       <x:c r="AB23" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC23" s="21" t="str">
         <x:v>En cours</x:v>
@@ -2432,7 +2432,7 @@
         <x:v>Consigner l’accord de Thanh. Requalifier les preuves historiques</x:v>
       </x:c>
       <x:c r="AB24" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC24" s="21" t="str">
         <x:v>En cours</x:v>
@@ -2523,7 +2523,7 @@
         <x:v>Consigner l’accord de Thanh. Requalifier les preuves historiques</x:v>
       </x:c>
       <x:c r="AB25" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC25" s="21" t="str">
         <x:v>En cours</x:v>
@@ -2614,7 +2614,7 @@
         <x:v>Consigner l’accord de Thanh. Requalifier les preuves historiques</x:v>
       </x:c>
       <x:c r="AB26" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC26" s="21" t="str">
         <x:v>En cours</x:v>
@@ -2705,7 +2705,7 @@
         <x:v>Consigner l’accord de Thanh. Requalifier les preuves historiques</x:v>
       </x:c>
       <x:c r="AB27" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC27" s="21" t="str">
         <x:v>En cours</x:v>
@@ -2796,7 +2796,7 @@
         <x:v>Consigner l’accord de Thanh. Requalifier les preuves historiques</x:v>
       </x:c>
       <x:c r="AB28" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC28" s="21" t="str">
         <x:v>En cours</x:v>
@@ -2887,7 +2887,7 @@
         <x:v>Consigner l’accord de Thanh. Requalifier les preuves historiques</x:v>
       </x:c>
       <x:c r="AB29" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC29" s="21" t="str">
         <x:v>En cours</x:v>
@@ -2978,7 +2978,7 @@
         <x:v>Consigner l’accord de Thanh. Requalifier les preuves historiques</x:v>
       </x:c>
       <x:c r="AB30" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC30" s="21" t="str">
         <x:v>En cours</x:v>
@@ -3069,7 +3069,7 @@
         <x:v>Consigner l’accord de Thanh. Requalifier les preuves historiques</x:v>
       </x:c>
       <x:c r="AB31" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC31" s="21" t="str">
         <x:v>En cours</x:v>
@@ -3160,7 +3160,7 @@
         <x:v>Consigner l’accord de Thanh. Requalifier les preuves historiques</x:v>
       </x:c>
       <x:c r="AB32" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC32" s="21" t="str">
         <x:v>En cours</x:v>
@@ -3251,7 +3251,7 @@
         <x:v>Consigner l’accord de Thanh. Requalifier les preuves historiques</x:v>
       </x:c>
       <x:c r="AB33" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC33" s="21" t="str">
         <x:v>En cours</x:v>
@@ -3342,7 +3342,7 @@
         <x:v>Consigner l’accord de Thanh. Requalifier les preuves historiques</x:v>
       </x:c>
       <x:c r="AB34" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC34" s="21" t="str">
         <x:v>En cours</x:v>
@@ -3433,7 +3433,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB35" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC35" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -3524,7 +3524,7 @@
         <x:v>Consigner l’accord de Thanh. Requalifier les preuves historiques</x:v>
       </x:c>
       <x:c r="AB36" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC36" s="21" t="str">
         <x:v>En cours</x:v>
@@ -3615,7 +3615,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB37" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC37" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -3706,7 +3706,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB38" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC38" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -3797,7 +3797,7 @@
         <x:v>Consigner l’accord de Thanh. Requalifier les preuves historiques</x:v>
       </x:c>
       <x:c r="AB39" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC39" s="21" t="str">
         <x:v>En cours</x:v>
@@ -3888,7 +3888,7 @@
         <x:v>Consigner l’accord de Thanh. Requalifier les preuves historiques</x:v>
       </x:c>
       <x:c r="AB40" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC40" s="21" t="str">
         <x:v>En cours</x:v>
@@ -3979,7 +3979,7 @@
         <x:v>Consigner l’accord de Thanh. Requalifier les preuves historiques</x:v>
       </x:c>
       <x:c r="AB41" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC41" s="21" t="str">
         <x:v>En cours</x:v>
@@ -4070,7 +4070,7 @@
         <x:v>Consigner l’accord de Thanh. Requalifier les preuves historiques</x:v>
       </x:c>
       <x:c r="AB42" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC42" s="21" t="str">
         <x:v>En cours</x:v>
@@ -4161,7 +4161,7 @@
         <x:v>Consigner l’accord de Thanh. Requalifier les preuves historiques</x:v>
       </x:c>
       <x:c r="AB43" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC43" s="21" t="str">
         <x:v>En cours</x:v>
@@ -4252,7 +4252,7 @@
         <x:v>Consigner l’accord de Thanh. Requalifier les preuves historiques</x:v>
       </x:c>
       <x:c r="AB44" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC44" s="21" t="str">
         <x:v>En cours</x:v>
@@ -4343,7 +4343,7 @@
         <x:v>Consigner l’accord de Thanh. Requalifier les preuves historiques</x:v>
       </x:c>
       <x:c r="AB45" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC45" s="21" t="str">
         <x:v>En cours</x:v>
@@ -4434,7 +4434,7 @@
         <x:v>Consigner l’accord de Thanh. Requalifier les preuves historiques</x:v>
       </x:c>
       <x:c r="AB46" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC46" s="21" t="str">
         <x:v>En cours</x:v>
@@ -4525,7 +4525,7 @@
         <x:v>Consigner l’accord de Thanh. Requalifier les preuves historiques</x:v>
       </x:c>
       <x:c r="AB47" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC47" s="21" t="str">
         <x:v>En cours</x:v>
@@ -4616,7 +4616,7 @@
         <x:v>Consigner l’accord de Thanh. Requalifier les preuves historiques</x:v>
       </x:c>
       <x:c r="AB48" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC48" s="21" t="str">
         <x:v>En cours</x:v>
@@ -4707,7 +4707,7 @@
         <x:v>Consigner l’accord de Thanh. Requalifier les preuves historiques</x:v>
       </x:c>
       <x:c r="AB49" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC49" s="21" t="str">
         <x:v>En cours</x:v>
@@ -4798,7 +4798,7 @@
         <x:v>Consigner l’accord de Thanh. Requalifier les preuves historiques</x:v>
       </x:c>
       <x:c r="AB50" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC50" s="21" t="str">
         <x:v>En cours</x:v>
@@ -4889,7 +4889,7 @@
         <x:v>Consigner l’accord de Thanh</x:v>
       </x:c>
       <x:c r="AB51" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC51" s="21" t="str">
         <x:v>En cours</x:v>
@@ -4980,7 +4980,7 @@
         <x:v>Consigner l’accord de Thanh</x:v>
       </x:c>
       <x:c r="AB52" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC52" s="21" t="str">
         <x:v>En cours</x:v>
@@ -5071,7 +5071,7 @@
         <x:v>Consigner l’accord de Thanh</x:v>
       </x:c>
       <x:c r="AB53" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC53" s="21" t="str">
         <x:v>En cours</x:v>
@@ -5162,7 +5162,7 @@
         <x:v>Consigner l’accord de Thanh</x:v>
       </x:c>
       <x:c r="AB54" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC54" s="21" t="str">
         <x:v>En cours</x:v>
@@ -5253,7 +5253,7 @@
         <x:v>Consigner l’accord de Thanh</x:v>
       </x:c>
       <x:c r="AB55" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC55" s="21" t="str">
         <x:v>En cours</x:v>
@@ -5344,7 +5344,7 @@
         <x:v>Consigner l’accord de Thanh</x:v>
       </x:c>
       <x:c r="AB56" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC56" s="21" t="str">
         <x:v>En cours</x:v>
@@ -5435,7 +5435,7 @@
         <x:v>Consigner l’accord de Thanh</x:v>
       </x:c>
       <x:c r="AB57" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC57" s="21" t="str">
         <x:v>En cours</x:v>
@@ -5526,7 +5526,7 @@
         <x:v>Consigner l’accord de Thanh</x:v>
       </x:c>
       <x:c r="AB58" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC58" s="21" t="str">
         <x:v>En cours</x:v>
@@ -5617,7 +5617,7 @@
         <x:v>Consigner l’accord de Thanh</x:v>
       </x:c>
       <x:c r="AB59" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC59" s="21" t="str">
         <x:v>En cours</x:v>
@@ -5708,7 +5708,7 @@
         <x:v>Consigner l’accord de Thanh</x:v>
       </x:c>
       <x:c r="AB60" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC60" s="21" t="str">
         <x:v>En cours</x:v>
@@ -5799,7 +5799,7 @@
         <x:v>Consigner l’accord de Thanh</x:v>
       </x:c>
       <x:c r="AB61" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC61" s="21" t="str">
         <x:v>En cours</x:v>
@@ -5890,7 +5890,7 @@
         <x:v>Consigner l’accord de Thanh</x:v>
       </x:c>
       <x:c r="AB62" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC62" s="21" t="str">
         <x:v>En cours</x:v>
@@ -5981,7 +5981,7 @@
         <x:v>Consigner l’accord de Thanh</x:v>
       </x:c>
       <x:c r="AB63" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC63" s="21" t="str">
         <x:v>En cours</x:v>
@@ -6072,7 +6072,7 @@
         <x:v>Consigner l’accord de Thanh</x:v>
       </x:c>
       <x:c r="AB64" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC64" s="21" t="str">
         <x:v>En cours</x:v>
@@ -6163,7 +6163,7 @@
         <x:v>Consigner l’accord de Thanh</x:v>
       </x:c>
       <x:c r="AB65" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC65" s="21" t="str">
         <x:v>En cours</x:v>
@@ -6254,7 +6254,7 @@
         <x:v>Consigner l’accord de Thanh</x:v>
       </x:c>
       <x:c r="AB66" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC66" s="21" t="str">
         <x:v>En cours</x:v>
@@ -6345,7 +6345,7 @@
         <x:v>Consigner l’accord de Thanh</x:v>
       </x:c>
       <x:c r="AB67" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC67" s="21" t="str">
         <x:v>En cours</x:v>
@@ -6436,7 +6436,7 @@
         <x:v>Consigner l’accord de Thanh</x:v>
       </x:c>
       <x:c r="AB68" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC68" s="21" t="str">
         <x:v>En cours</x:v>
@@ -6527,7 +6527,7 @@
         <x:v>Consigner l’accord de Thanh</x:v>
       </x:c>
       <x:c r="AB69" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC69" s="21" t="str">
         <x:v>En cours</x:v>
@@ -6618,7 +6618,7 @@
         <x:v>Consigner l’accord de Thanh</x:v>
       </x:c>
       <x:c r="AB70" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC70" s="21" t="str">
         <x:v>En cours</x:v>
@@ -6709,7 +6709,7 @@
         <x:v>Consigner l’accord de Thanh</x:v>
       </x:c>
       <x:c r="AB71" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC71" s="21" t="str">
         <x:v>En cours</x:v>
@@ -6800,7 +6800,7 @@
         <x:v>Consigner l’accord de Thanh</x:v>
       </x:c>
       <x:c r="AB72" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC72" s="21" t="str">
         <x:v>En cours</x:v>
@@ -6891,7 +6891,7 @@
         <x:v>Consigner l’accord de Thanh</x:v>
       </x:c>
       <x:c r="AB73" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC73" s="21" t="str">
         <x:v>En cours</x:v>
@@ -6982,7 +6982,7 @@
         <x:v>Consigner l’accord de Thanh</x:v>
       </x:c>
       <x:c r="AB74" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC74" s="21" t="str">
         <x:v>En cours</x:v>
@@ -7073,7 +7073,7 @@
         <x:v>Consigner l’accord de Thanh</x:v>
       </x:c>
       <x:c r="AB75" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC75" s="21" t="str">
         <x:v>En cours</x:v>
@@ -7164,7 +7164,7 @@
         <x:v>Consigner l’accord de Thanh</x:v>
       </x:c>
       <x:c r="AB76" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC76" s="21" t="str">
         <x:v>En cours</x:v>
@@ -7255,7 +7255,7 @@
         <x:v>Consigner l’accord de Thanh</x:v>
       </x:c>
       <x:c r="AB77" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC77" s="21" t="str">
         <x:v>En cours</x:v>
@@ -7346,7 +7346,7 @@
         <x:v>Consigner l’accord de Thanh</x:v>
       </x:c>
       <x:c r="AB78" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC78" s="21" t="str">
         <x:v>En cours</x:v>
@@ -7437,7 +7437,7 @@
         <x:v>Consigner l’accord de Thanh</x:v>
       </x:c>
       <x:c r="AB79" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC79" s="21" t="str">
         <x:v>En cours</x:v>
@@ -7528,7 +7528,7 @@
         <x:v>Consigner l’accord de Thanh</x:v>
       </x:c>
       <x:c r="AB80" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC80" s="21" t="str">
         <x:v>En cours</x:v>
@@ -7619,7 +7619,7 @@
         <x:v>Consigner l’accord de Thanh</x:v>
       </x:c>
       <x:c r="AB81" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC81" s="21" t="str">
         <x:v>En cours</x:v>
@@ -7710,7 +7710,7 @@
         <x:v>Consigner l’accord de Thanh</x:v>
       </x:c>
       <x:c r="AB82" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC82" s="21" t="str">
         <x:v>En cours</x:v>
@@ -7801,7 +7801,7 @@
         <x:v>Consigner l’accord de Thanh</x:v>
       </x:c>
       <x:c r="AB83" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC83" s="21" t="str">
         <x:v>En cours</x:v>
@@ -7892,7 +7892,7 @@
         <x:v>Consigner l’accord de Thanh</x:v>
       </x:c>
       <x:c r="AB84" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC84" s="21" t="str">
         <x:v>En cours</x:v>
@@ -7983,7 +7983,7 @@
         <x:v>Consigner l’accord de Thanh</x:v>
       </x:c>
       <x:c r="AB85" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC85" s="21" t="str">
         <x:v>En cours</x:v>
@@ -8074,7 +8074,7 @@
         <x:v>Consigner l’accord de Thanh</x:v>
       </x:c>
       <x:c r="AB86" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC86" s="21" t="str">
         <x:v>En cours</x:v>
@@ -8165,7 +8165,7 @@
         <x:v>Consigner l’accord de Thanh</x:v>
       </x:c>
       <x:c r="AB87" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC87" s="21" t="str">
         <x:v>En cours</x:v>
@@ -8256,7 +8256,7 @@
         <x:v>Consigner l’accord de Thanh</x:v>
       </x:c>
       <x:c r="AB88" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC88" s="21" t="str">
         <x:v>En cours</x:v>
@@ -8347,7 +8347,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB89" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC89" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -8438,7 +8438,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB90" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC90" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -8529,7 +8529,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB91" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC91" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -8620,7 +8620,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB92" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC92" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -8711,7 +8711,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB93" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC93" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -8802,7 +8802,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB94" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC94" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -8893,7 +8893,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB95" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC95" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -8984,7 +8984,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB96" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC96" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -9075,7 +9075,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB97" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC97" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -9166,7 +9166,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB98" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC98" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -9257,7 +9257,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB99" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC99" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -9348,7 +9348,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB100" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC100" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -9439,7 +9439,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB101" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC101" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -9530,7 +9530,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB102" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC102" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -9621,7 +9621,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB103" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC103" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -9712,7 +9712,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB104" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC104" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -9803,7 +9803,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB105" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC105" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -9894,7 +9894,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB106" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC106" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -9985,7 +9985,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB107" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC107" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -10076,7 +10076,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB108" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC108" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -10167,7 +10167,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB109" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC109" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -10258,7 +10258,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB110" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC110" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -10349,7 +10349,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB111" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC111" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -10440,7 +10440,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB112" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC112" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -10531,7 +10531,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB113" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC113" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -10622,7 +10622,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB114" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC114" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -10713,7 +10713,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB115" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC115" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -10804,7 +10804,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB116" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC116" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -10895,7 +10895,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB117" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC117" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -10986,7 +10986,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB118" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC118" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -11077,7 +11077,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB119" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC119" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -11168,7 +11168,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB120" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC120" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -11259,7 +11259,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB121" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC121" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -11350,7 +11350,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB122" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC122" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -11441,7 +11441,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB123" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC123" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -11532,7 +11532,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB124" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC124" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -11623,7 +11623,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB125" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC125" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -11714,7 +11714,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB126" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC126" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -11805,7 +11805,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB127" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC127" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -11896,7 +11896,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB128" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC128" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -11987,7 +11987,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB129" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC129" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -12078,7 +12078,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB130" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC130" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -12169,7 +12169,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB131" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC131" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -12260,7 +12260,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB132" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC132" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -12351,7 +12351,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB133" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC133" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -12442,7 +12442,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB134" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC134" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -12533,7 +12533,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB135" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC135" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -12624,7 +12624,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB136" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC136" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -12715,7 +12715,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB137" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC137" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -12806,7 +12806,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB138" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC138" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -12897,7 +12897,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB139" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC139" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -12988,7 +12988,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB140" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC140" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -13079,7 +13079,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB141" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC141" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -13170,7 +13170,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB142" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC142" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -13261,7 +13261,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB143" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC143" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -13352,7 +13352,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB144" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC144" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -13443,7 +13443,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB145" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC145" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -13534,7 +13534,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB146" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC146" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -13625,7 +13625,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB147" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC147" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -13716,7 +13716,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB148" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC148" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -13807,7 +13807,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB149" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC149" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -13898,7 +13898,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB150" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC150" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -13989,7 +13989,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB151" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC151" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -14080,7 +14080,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB152" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC152" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -14171,7 +14171,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB153" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC153" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -14262,7 +14262,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB154" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC154" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -14353,7 +14353,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB155" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC155" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -14444,7 +14444,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB156" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC156" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -14535,7 +14535,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB157" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC157" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -14626,7 +14626,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB158" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC158" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -14717,7 +14717,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB159" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC159" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -14808,7 +14808,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB160" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC160" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -14899,7 +14899,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB161" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC161" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -14990,7 +14990,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB162" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC162" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -15081,7 +15081,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB163" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC163" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -15172,7 +15172,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB164" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC164" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -15263,7 +15263,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB165" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC165" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -15354,7 +15354,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB166" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC166" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -15445,7 +15445,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB167" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC167" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -15536,7 +15536,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB168" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC168" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -15627,7 +15627,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB169" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC169" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -15718,7 +15718,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB170" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC170" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -15809,7 +15809,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB171" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC171" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -15900,7 +15900,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB172" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC172" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -15991,7 +15991,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB173" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC173" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -16082,7 +16082,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB174" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC174" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -16173,7 +16173,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB175" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC175" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -16264,7 +16264,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB176" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC176" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -16355,7 +16355,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB177" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC177" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -16446,7 +16446,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB178" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC178" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -16537,7 +16537,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB179" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC179" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -16628,7 +16628,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB180" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC180" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -16719,7 +16719,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB181" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC181" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -16810,7 +16810,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB182" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC182" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -16901,7 +16901,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB183" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC183" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -16992,7 +16992,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB184" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC184" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -17083,7 +17083,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB185" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC185" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -17174,7 +17174,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB186" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC186" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -17265,7 +17265,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB187" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC187" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -17356,7 +17356,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB188" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC188" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -17447,7 +17447,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB189" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC189" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -17538,7 +17538,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB190" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC190" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -17629,7 +17629,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB191" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC191" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -17720,7 +17720,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB192" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC192" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -17811,7 +17811,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB193" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC193" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -17902,7 +17902,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB194" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC194" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -17993,7 +17993,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB195" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC195" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -18084,7 +18084,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB196" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC196" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -18175,7 +18175,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB197" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC197" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -18266,7 +18266,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB198" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC198" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -18357,7 +18357,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB199" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC199" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -18448,7 +18448,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB200" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC200" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -18539,7 +18539,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB201" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC201" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -18630,7 +18630,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB202" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC202" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -18721,7 +18721,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB203" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC203" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -18812,7 +18812,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB204" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC204" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -18903,7 +18903,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB205" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC205" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -18994,7 +18994,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB206" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC206" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -19085,7 +19085,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB207" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC207" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -19176,7 +19176,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB208" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC208" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -19267,7 +19267,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB209" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC209" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -19358,7 +19358,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB210" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC210" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -19449,7 +19449,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB211" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC211" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -19540,7 +19540,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB212" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC212" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -19631,7 +19631,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB213" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC213" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -19722,7 +19722,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB214" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC214" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -19813,7 +19813,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB215" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC215" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -19904,7 +19904,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB216" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC216" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -19995,7 +19995,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB217" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC217" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -20086,7 +20086,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB218" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC218" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -20177,7 +20177,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB219" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC219" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -20268,7 +20268,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB220" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC220" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -20359,7 +20359,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB221" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC221" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -20450,7 +20450,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB222" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC222" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -20541,7 +20541,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB223" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC223" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -20632,7 +20632,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB224" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC224" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -20723,7 +20723,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB225" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC225" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -20814,7 +20814,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB226" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC226" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -20905,7 +20905,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB227" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC227" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -20996,7 +20996,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB228" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC228" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -21087,7 +21087,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB229" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC229" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -21178,7 +21178,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB230" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC230" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -21269,7 +21269,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB231" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC231" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -21360,7 +21360,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB232" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC232" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -21451,7 +21451,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB233" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC233" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -21542,7 +21542,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB234" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC234" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -21633,7 +21633,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB235" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC235" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -21724,7 +21724,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB236" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC236" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -21815,7 +21815,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB237" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC237" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -21906,7 +21906,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB238" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC238" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -21997,7 +21997,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB239" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC239" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -22088,7 +22088,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB240" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC240" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -22179,7 +22179,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB241" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC241" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -22270,7 +22270,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB242" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC242" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -22361,7 +22361,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB243" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC243" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -22452,7 +22452,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB244" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC244" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -22543,7 +22543,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB245" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC245" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -22634,7 +22634,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB246" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC246" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -22725,7 +22725,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB247" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC247" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -22816,7 +22816,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB248" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC248" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -22907,7 +22907,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB249" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC249" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -22998,7 +22998,7 @@
         <x:v>Choisir trois scènes. Préparer les huit sources. Intégrer le pack dans les six langues</x:v>
       </x:c>
       <x:c r="AB250" s="21" t="str">
-        <x:v>1a63ecf787bc8d20e322314e1ba17987c83b1198</x:v>
+        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC250" s="21" t="str">
         <x:v>Pack à compléter</x:v>
@@ -23094,7 +23094,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0abd3bf23be1423e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5c91631952f5408a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Record 29 qualified symbol packs and refresh Excel CSV handoff
</commit_message>
<xml_diff>
--- a/doc_web_interne/docs/suivi-symboles/suivi-240-symboles-6-langues.xlsx
+++ b/doc_web_interne/docs/suivi-symboles/suivi-240-symboles-6-langues.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Suivi symboles" sheetId="1" r:id="R7d7186195bc74f82"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Suivi symboles" sheetId="1" r:id="R5b4ca2c0133c4438"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -811,7 +811,7 @@
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="7" t="str">
-        <x:v>Lot 08 en branche : 30 couvertures conservées, 210 nouveaux PNG. Les preuves périmées restent historiques.</x:v>
+        <x:v>Lot 10 en branche : 29 couvertures conservées, 203 nouveaux PNG. Les QA inchangées du lot 08 restent actuelles.</x:v>
       </x:c>
       <x:c r="B3" s="7"/>
       <x:c r="C3" s="7"/>
@@ -848,21 +848,21 @@
       </x:c>
       <x:c r="B4" s="9" t="n">
         <x:f>COUNTIF(F11:F250,"Intégré")</x:f>
-        <x:v>105</x:v>
+        <x:v>140</x:v>
       </x:c>
       <x:c r="C4" s="3" t="str">
         <x:v>Packs à terminer</x:v>
       </x:c>
       <x:c r="D4" s="9" t="n">
         <x:f>COUNTA(B11:B250)-B4</x:f>
-        <x:v>135</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="E4" s="3" t="str">
         <x:v>Pages avec pack</x:v>
       </x:c>
       <x:c r="F4" s="9" t="n">
         <x:f>COUNTIF(Q11:V250,"Atlas")</x:f>
-        <x:v>630</x:v>
+        <x:v>840</x:v>
       </x:c>
       <x:c r="G4" s="3" t="str">
         <x:v>Pages web</x:v>
@@ -899,14 +899,14 @@
       </x:c>
       <x:c r="B5" s="9" t="n">
         <x:f>COUNTIF(W11:W250,"6/6 actuelles")</x:f>
-        <x:v>30</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="C5" s="3" t="str">
         <x:v>QA 2560 px</x:v>
       </x:c>
       <x:c r="D5" s="9" t="n">
         <x:f>COUNTIF(X11:X250,"6/6 actuelles")</x:f>
-        <x:v>30</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="E5" s="3" t="str">
         <x:v>Accord Thanh</x:v>
@@ -980,7 +980,7 @@
     </x:row>
     <x:row r="7" ht="20" customHeight="1">
       <x:c r="A7" s="7" t="str">
-        <x:v>105 packs ; 135 à compléter. Cadre commun : 1 440 pages. Publication antérieure conservée dans les reçus.</x:v>
+        <x:v>140 packs ; 100 à compléter. Cadre commun : 1 440 pages. Publication antérieure conservée dans les reçus.</x:v>
       </x:c>
       <x:c r="B7" s="7"/>
       <x:c r="C7" s="7"/>
@@ -1013,7 +1013,7 @@
     </x:row>
     <x:row r="8" ht="20" customHeight="1">
       <x:c r="A8" s="7" t="str">
-        <x:v>Source : rapport canonique du 20/10/2026, empreinte e9cf4eb1696b8cda. Révision : 9184f780a23f21687350020fa3448d58e4e0aadd</x:v>
+        <x:v>Source : rapport canonique du 20/10/2026, empreinte fe68cf7fc49c16e1. Révision : fc0d47528b092ffae3e49cc020fbc27e902dc01b</x:v>
       </x:c>
       <x:c r="B8" s="7"/>
       <x:c r="C8" s="7"/>
@@ -1240,13 +1240,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="Y11" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="Z11" s="24" t="str">
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA11" s="23" t="str">
-        <x:v>Requalifier QA et publication du candidat ; accord non consigné.</x:v>
+        <x:v>Requalifier QA ; accord et publication non consignés.</x:v>
       </x:c>
       <x:c r="AB11" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -1331,13 +1331,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="Y12" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="Z12" s="24" t="str">
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA12" s="23" t="str">
-        <x:v>Requalifier QA et publication du candidat ; accord non consigné.</x:v>
+        <x:v>Requalifier QA ; accord et publication non consignés.</x:v>
       </x:c>
       <x:c r="AB12" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -1422,13 +1422,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="Y13" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="Z13" s="24" t="str">
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA13" s="23" t="str">
-        <x:v>Requalifier QA et publication du candidat ; accord non consigné.</x:v>
+        <x:v>Requalifier QA ; accord et publication non consignés.</x:v>
       </x:c>
       <x:c r="AB13" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -1513,13 +1513,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="Y14" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="Z14" s="24" t="str">
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA14" s="23" t="str">
-        <x:v>Requalifier QA et publication du candidat ; accord non consigné.</x:v>
+        <x:v>Requalifier QA ; accord et publication non consignés.</x:v>
       </x:c>
       <x:c r="AB14" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -1604,13 +1604,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="Y15" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="Z15" s="24" t="str">
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA15" s="23" t="str">
-        <x:v>Requalifier QA et publication du candidat ; accord non consigné.</x:v>
+        <x:v>Requalifier QA ; accord et publication non consignés.</x:v>
       </x:c>
       <x:c r="AB15" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -1695,13 +1695,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="Y16" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="Z16" s="24" t="str">
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA16" s="23" t="str">
-        <x:v>Requalifier QA et publication du candidat ; accord non consigné.</x:v>
+        <x:v>Requalifier QA ; accord et publication non consignés.</x:v>
       </x:c>
       <x:c r="AB16" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -1786,13 +1786,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="Y17" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="Z17" s="24" t="str">
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA17" s="23" t="str">
-        <x:v>Requalifier QA et publication du candidat ; accord non consigné.</x:v>
+        <x:v>Requalifier QA ; accord et publication non consignés.</x:v>
       </x:c>
       <x:c r="AB17" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -1877,13 +1877,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="Y18" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="Z18" s="24" t="str">
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA18" s="23" t="str">
-        <x:v>Requalifier QA et publication du candidat ; accord non consigné.</x:v>
+        <x:v>Requalifier QA ; accord et publication non consignés.</x:v>
       </x:c>
       <x:c r="AB18" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -1968,13 +1968,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="Y19" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="Z19" s="24" t="str">
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA19" s="23" t="str">
-        <x:v>Requalifier QA et publication du candidat ; accord non consigné.</x:v>
+        <x:v>Requalifier QA ; accord et publication non consignés.</x:v>
       </x:c>
       <x:c r="AB19" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -2059,13 +2059,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="Y20" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="Z20" s="24" t="str">
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA20" s="23" t="str">
-        <x:v>Requalifier QA et publication du candidat ; accord non consigné.</x:v>
+        <x:v>Requalifier QA ; accord et publication non consignés.</x:v>
       </x:c>
       <x:c r="AB20" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -2150,13 +2150,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="Y21" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="Z21" s="24" t="str">
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA21" s="23" t="str">
-        <x:v>Requalifier QA et publication du candidat ; accord non consigné.</x:v>
+        <x:v>Requalifier QA ; accord et publication non consignés.</x:v>
       </x:c>
       <x:c r="AB21" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -2241,13 +2241,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="Y22" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="Z22" s="24" t="str">
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA22" s="23" t="str">
-        <x:v>Requalifier QA et publication du candidat ; accord non consigné.</x:v>
+        <x:v>Requalifier QA ; accord et publication non consignés.</x:v>
       </x:c>
       <x:c r="AB22" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -2332,13 +2332,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="Y23" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="Z23" s="24" t="str">
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA23" s="23" t="str">
-        <x:v>Requalifier QA et publication du candidat ; accord non consigné.</x:v>
+        <x:v>Requalifier QA ; accord et publication non consignés.</x:v>
       </x:c>
       <x:c r="AB23" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -2423,13 +2423,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="Y24" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="Z24" s="24" t="str">
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA24" s="23" t="str">
-        <x:v>Requalifier QA et publication du candidat ; accord non consigné.</x:v>
+        <x:v>Requalifier QA ; accord et publication non consignés.</x:v>
       </x:c>
       <x:c r="AB24" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -2514,13 +2514,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="Y25" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="Z25" s="24" t="str">
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA25" s="23" t="str">
-        <x:v>Requalifier QA et publication du candidat ; accord non consigné.</x:v>
+        <x:v>Requalifier QA ; accord et publication non consignés.</x:v>
       </x:c>
       <x:c r="AB25" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -2605,13 +2605,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="Y26" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="Z26" s="24" t="str">
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA26" s="23" t="str">
-        <x:v>Requalifier QA et publication du candidat ; accord non consigné.</x:v>
+        <x:v>Requalifier QA ; accord et publication non consignés.</x:v>
       </x:c>
       <x:c r="AB26" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -2696,13 +2696,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="Y27" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="Z27" s="24" t="str">
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA27" s="23" t="str">
-        <x:v>Requalifier QA et publication du candidat ; accord non consigné.</x:v>
+        <x:v>Requalifier QA ; accord et publication non consignés.</x:v>
       </x:c>
       <x:c r="AB27" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -2787,13 +2787,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="Y28" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="Z28" s="24" t="str">
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA28" s="23" t="str">
-        <x:v>Requalifier QA et publication du candidat ; accord non consigné.</x:v>
+        <x:v>Requalifier QA ; accord et publication non consignés.</x:v>
       </x:c>
       <x:c r="AB28" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -2878,13 +2878,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="Y29" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="Z29" s="24" t="str">
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA29" s="23" t="str">
-        <x:v>Requalifier QA et publication du candidat ; accord non consigné.</x:v>
+        <x:v>Requalifier QA ; accord et publication non consignés.</x:v>
       </x:c>
       <x:c r="AB29" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -2969,13 +2969,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="Y30" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="Z30" s="24" t="str">
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA30" s="23" t="str">
-        <x:v>Requalifier QA et publication du candidat ; accord non consigné.</x:v>
+        <x:v>Requalifier QA ; accord et publication non consignés.</x:v>
       </x:c>
       <x:c r="AB30" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -3060,13 +3060,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="Y31" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="Z31" s="24" t="str">
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA31" s="23" t="str">
-        <x:v>Requalifier QA et publication du candidat ; accord non consigné.</x:v>
+        <x:v>Requalifier QA ; accord et publication non consignés.</x:v>
       </x:c>
       <x:c r="AB31" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -3151,13 +3151,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="Y32" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="Z32" s="24" t="str">
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA32" s="23" t="str">
-        <x:v>Requalifier QA et publication du candidat ; accord non consigné.</x:v>
+        <x:v>Requalifier QA ; accord et publication non consignés.</x:v>
       </x:c>
       <x:c r="AB32" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -3242,13 +3242,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="Y33" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="Z33" s="24" t="str">
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA33" s="23" t="str">
-        <x:v>Requalifier QA et publication du candidat ; accord non consigné.</x:v>
+        <x:v>Requalifier QA ; accord et publication non consignés.</x:v>
       </x:c>
       <x:c r="AB33" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -3333,13 +3333,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="Y34" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="Z34" s="24" t="str">
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA34" s="23" t="str">
-        <x:v>Requalifier QA et publication du candidat ; accord non consigné.</x:v>
+        <x:v>Requalifier QA ; accord et publication non consignés.</x:v>
       </x:c>
       <x:c r="AB34" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -3515,13 +3515,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="Y36" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="Z36" s="24" t="str">
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA36" s="23" t="str">
-        <x:v>Requalifier QA et publication du candidat ; accord non consigné.</x:v>
+        <x:v>Requalifier QA ; accord et publication non consignés.</x:v>
       </x:c>
       <x:c r="AB36" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -3703,7 +3703,7 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA38" s="23" t="str">
-        <x:v>Accord et publication du lot non consignés.</x:v>
+        <x:v>QA actuelle ; accord et publication non consignés.</x:v>
       </x:c>
       <x:c r="AB38" s="21" t="str">
         <x:v>9184f780a23f21687350020fa3448d58e4e0aadd</x:v>
@@ -3788,13 +3788,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="Y39" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="Z39" s="24" t="str">
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA39" s="23" t="str">
-        <x:v>Requalifier QA et publication du candidat ; accord non consigné.</x:v>
+        <x:v>Requalifier QA ; accord et publication non consignés.</x:v>
       </x:c>
       <x:c r="AB39" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -3879,13 +3879,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="Y40" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="Z40" s="24" t="str">
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA40" s="23" t="str">
-        <x:v>Requalifier QA et publication du candidat ; accord non consigné.</x:v>
+        <x:v>Requalifier QA ; accord et publication non consignés.</x:v>
       </x:c>
       <x:c r="AB40" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -3970,13 +3970,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="Y41" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="Z41" s="24" t="str">
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA41" s="23" t="str">
-        <x:v>Requalifier QA et publication du candidat ; accord non consigné.</x:v>
+        <x:v>Requalifier QA ; accord et publication non consignés.</x:v>
       </x:c>
       <x:c r="AB41" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -4061,13 +4061,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="Y42" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="Z42" s="24" t="str">
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA42" s="23" t="str">
-        <x:v>Requalifier QA et publication du candidat ; accord non consigné.</x:v>
+        <x:v>Requalifier QA ; accord et publication non consignés.</x:v>
       </x:c>
       <x:c r="AB42" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -4152,13 +4152,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="Y43" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="Z43" s="24" t="str">
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA43" s="23" t="str">
-        <x:v>Requalifier QA et publication du candidat ; accord non consigné.</x:v>
+        <x:v>Requalifier QA ; accord et publication non consignés.</x:v>
       </x:c>
       <x:c r="AB43" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -4243,13 +4243,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="Y44" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="Z44" s="24" t="str">
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA44" s="23" t="str">
-        <x:v>Requalifier QA et publication du candidat ; accord non consigné.</x:v>
+        <x:v>Requalifier QA ; accord et publication non consignés.</x:v>
       </x:c>
       <x:c r="AB44" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -4334,13 +4334,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="Y45" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="Z45" s="24" t="str">
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA45" s="23" t="str">
-        <x:v>Requalifier QA et publication du candidat ; accord non consigné.</x:v>
+        <x:v>Requalifier QA ; accord et publication non consignés.</x:v>
       </x:c>
       <x:c r="AB45" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -4425,13 +4425,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="Y46" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="Z46" s="24" t="str">
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA46" s="23" t="str">
-        <x:v>Requalifier QA et publication du candidat ; accord non consigné.</x:v>
+        <x:v>Requalifier QA ; accord et publication non consignés.</x:v>
       </x:c>
       <x:c r="AB46" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -4516,13 +4516,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="Y47" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="Z47" s="24" t="str">
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA47" s="23" t="str">
-        <x:v>Requalifier QA et publication du candidat ; accord non consigné.</x:v>
+        <x:v>Requalifier QA ; accord et publication non consignés.</x:v>
       </x:c>
       <x:c r="AB47" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -4607,13 +4607,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="Y48" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="Z48" s="24" t="str">
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA48" s="23" t="str">
-        <x:v>Requalifier QA et publication du candidat ; accord non consigné.</x:v>
+        <x:v>Requalifier QA ; accord et publication non consignés.</x:v>
       </x:c>
       <x:c r="AB48" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -4698,13 +4698,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="Y49" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="Z49" s="24" t="str">
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA49" s="23" t="str">
-        <x:v>Requalifier QA et publication du candidat ; accord non consigné.</x:v>
+        <x:v>Requalifier QA ; accord et publication non consignés.</x:v>
       </x:c>
       <x:c r="AB49" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -4789,13 +4789,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="Y50" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="Z50" s="24" t="str">
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA50" s="23" t="str">
-        <x:v>Requalifier QA et publication du candidat ; accord non consigné.</x:v>
+        <x:v>Requalifier QA ; accord et publication non consignés.</x:v>
       </x:c>
       <x:c r="AB50" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -4886,7 +4886,7 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA51" s="23" t="str">
-        <x:v>Requalifier QA et publication du candidat ; accord non consigné.</x:v>
+        <x:v>Requalifier QA ; accord et publication non consignés.</x:v>
       </x:c>
       <x:c r="AB51" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -4977,7 +4977,7 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA52" s="23" t="str">
-        <x:v>Requalifier QA et publication du candidat ; accord non consigné.</x:v>
+        <x:v>Requalifier QA ; accord et publication non consignés.</x:v>
       </x:c>
       <x:c r="AB52" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -5068,7 +5068,7 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA53" s="23" t="str">
-        <x:v>Requalifier QA et publication du candidat ; accord non consigné.</x:v>
+        <x:v>Requalifier QA ; accord et publication non consignés.</x:v>
       </x:c>
       <x:c r="AB53" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -5159,7 +5159,7 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA54" s="23" t="str">
-        <x:v>Requalifier QA et publication du candidat ; accord non consigné.</x:v>
+        <x:v>Requalifier QA ; accord et publication non consignés.</x:v>
       </x:c>
       <x:c r="AB54" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -5250,7 +5250,7 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA55" s="23" t="str">
-        <x:v>Requalifier QA et publication du candidat ; accord non consigné.</x:v>
+        <x:v>Requalifier QA ; accord et publication non consignés.</x:v>
       </x:c>
       <x:c r="AB55" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -5341,7 +5341,7 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA56" s="23" t="str">
-        <x:v>Requalifier QA et publication du candidat ; accord non consigné.</x:v>
+        <x:v>Requalifier QA ; accord et publication non consignés.</x:v>
       </x:c>
       <x:c r="AB56" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -5432,7 +5432,7 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA57" s="23" t="str">
-        <x:v>Requalifier QA et publication du candidat ; accord non consigné.</x:v>
+        <x:v>Requalifier QA ; accord et publication non consignés.</x:v>
       </x:c>
       <x:c r="AB57" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -5523,7 +5523,7 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA58" s="23" t="str">
-        <x:v>Requalifier QA et publication du candidat ; accord non consigné.</x:v>
+        <x:v>Requalifier QA ; accord et publication non consignés.</x:v>
       </x:c>
       <x:c r="AB58" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -5614,7 +5614,7 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA59" s="23" t="str">
-        <x:v>Requalifier QA et publication du candidat ; accord non consigné.</x:v>
+        <x:v>Requalifier QA ; accord et publication non consignés.</x:v>
       </x:c>
       <x:c r="AB59" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -5705,7 +5705,7 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA60" s="23" t="str">
-        <x:v>Requalifier QA et publication du candidat ; accord non consigné.</x:v>
+        <x:v>Requalifier QA ; accord et publication non consignés.</x:v>
       </x:c>
       <x:c r="AB60" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -5796,7 +5796,7 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA61" s="23" t="str">
-        <x:v>Requalifier QA et publication du candidat ; accord non consigné.</x:v>
+        <x:v>Requalifier QA ; accord et publication non consignés.</x:v>
       </x:c>
       <x:c r="AB61" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -5887,7 +5887,7 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA62" s="23" t="str">
-        <x:v>Requalifier QA et publication du candidat ; accord non consigné.</x:v>
+        <x:v>Requalifier QA ; accord et publication non consignés.</x:v>
       </x:c>
       <x:c r="AB62" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -5978,7 +5978,7 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA63" s="23" t="str">
-        <x:v>Requalifier QA et publication du candidat ; accord non consigné.</x:v>
+        <x:v>Requalifier QA ; accord et publication non consignés.</x:v>
       </x:c>
       <x:c r="AB63" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -6069,7 +6069,7 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA64" s="23" t="str">
-        <x:v>Requalifier QA et publication du candidat ; accord non consigné.</x:v>
+        <x:v>Requalifier QA ; accord et publication non consignés.</x:v>
       </x:c>
       <x:c r="AB64" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -6160,7 +6160,7 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA65" s="23" t="str">
-        <x:v>Requalifier QA et publication du candidat ; accord non consigné.</x:v>
+        <x:v>Requalifier QA ; accord et publication non consignés.</x:v>
       </x:c>
       <x:c r="AB65" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -6251,7 +6251,7 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA66" s="23" t="str">
-        <x:v>Requalifier QA et publication du candidat ; accord non consigné.</x:v>
+        <x:v>Requalifier QA ; accord et publication non consignés.</x:v>
       </x:c>
       <x:c r="AB66" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -6342,7 +6342,7 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA67" s="23" t="str">
-        <x:v>Requalifier QA et publication du candidat ; accord non consigné.</x:v>
+        <x:v>Requalifier QA ; accord et publication non consignés.</x:v>
       </x:c>
       <x:c r="AB67" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -6433,7 +6433,7 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA68" s="23" t="str">
-        <x:v>Requalifier QA et publication du candidat ; accord non consigné.</x:v>
+        <x:v>Requalifier QA ; accord et publication non consignés.</x:v>
       </x:c>
       <x:c r="AB68" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -6524,7 +6524,7 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA69" s="23" t="str">
-        <x:v>Requalifier QA et publication du candidat ; accord non consigné.</x:v>
+        <x:v>Requalifier QA ; accord et publication non consignés.</x:v>
       </x:c>
       <x:c r="AB69" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -6615,7 +6615,7 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA70" s="23" t="str">
-        <x:v>Requalifier QA et publication du candidat ; accord non consigné.</x:v>
+        <x:v>Requalifier QA ; accord et publication non consignés.</x:v>
       </x:c>
       <x:c r="AB70" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -6706,7 +6706,7 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA71" s="23" t="str">
-        <x:v>Requalifier QA et publication du candidat ; accord non consigné.</x:v>
+        <x:v>Requalifier QA ; accord et publication non consignés.</x:v>
       </x:c>
       <x:c r="AB71" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -6797,7 +6797,7 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA72" s="23" t="str">
-        <x:v>Requalifier QA et publication du candidat ; accord non consigné.</x:v>
+        <x:v>Requalifier QA ; accord et publication non consignés.</x:v>
       </x:c>
       <x:c r="AB72" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -6888,7 +6888,7 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA73" s="23" t="str">
-        <x:v>Requalifier QA et publication du candidat ; accord non consigné.</x:v>
+        <x:v>Requalifier QA ; accord et publication non consignés.</x:v>
       </x:c>
       <x:c r="AB73" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -6979,7 +6979,7 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA74" s="23" t="str">
-        <x:v>Requalifier QA et publication du candidat ; accord non consigné.</x:v>
+        <x:v>Requalifier QA ; accord et publication non consignés.</x:v>
       </x:c>
       <x:c r="AB74" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -7070,7 +7070,7 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA75" s="23" t="str">
-        <x:v>Requalifier QA et publication du candidat ; accord non consigné.</x:v>
+        <x:v>Requalifier QA ; accord et publication non consignés.</x:v>
       </x:c>
       <x:c r="AB75" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -7161,7 +7161,7 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA76" s="23" t="str">
-        <x:v>Requalifier QA et publication du candidat ; accord non consigné.</x:v>
+        <x:v>Requalifier QA ; accord et publication non consignés.</x:v>
       </x:c>
       <x:c r="AB76" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -7252,7 +7252,7 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA77" s="23" t="str">
-        <x:v>Requalifier QA et publication du candidat ; accord non consigné.</x:v>
+        <x:v>Requalifier QA ; accord et publication non consignés.</x:v>
       </x:c>
       <x:c r="AB77" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -7343,7 +7343,7 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA78" s="23" t="str">
-        <x:v>Requalifier QA et publication du candidat ; accord non consigné.</x:v>
+        <x:v>Requalifier QA ; accord et publication non consignés.</x:v>
       </x:c>
       <x:c r="AB78" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -7434,7 +7434,7 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA79" s="23" t="str">
-        <x:v>Requalifier QA et publication du candidat ; accord non consigné.</x:v>
+        <x:v>Requalifier QA ; accord et publication non consignés.</x:v>
       </x:c>
       <x:c r="AB79" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -7525,7 +7525,7 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA80" s="23" t="str">
-        <x:v>Requalifier QA et publication du candidat ; accord non consigné.</x:v>
+        <x:v>Requalifier QA ; accord et publication non consignés.</x:v>
       </x:c>
       <x:c r="AB80" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -7616,7 +7616,7 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA81" s="23" t="str">
-        <x:v>Requalifier QA et publication du candidat ; accord non consigné.</x:v>
+        <x:v>Requalifier QA ; accord et publication non consignés.</x:v>
       </x:c>
       <x:c r="AB81" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -7707,7 +7707,7 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA82" s="23" t="str">
-        <x:v>Requalifier QA et publication du candidat ; accord non consigné.</x:v>
+        <x:v>Requalifier QA ; accord et publication non consignés.</x:v>
       </x:c>
       <x:c r="AB82" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -7798,7 +7798,7 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA83" s="23" t="str">
-        <x:v>Requalifier QA et publication du candidat ; accord non consigné.</x:v>
+        <x:v>Requalifier QA ; accord et publication non consignés.</x:v>
       </x:c>
       <x:c r="AB83" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -7889,7 +7889,7 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA84" s="23" t="str">
-        <x:v>Requalifier QA et publication du candidat ; accord non consigné.</x:v>
+        <x:v>Requalifier QA ; accord et publication non consignés.</x:v>
       </x:c>
       <x:c r="AB84" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -7980,7 +7980,7 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA85" s="23" t="str">
-        <x:v>Requalifier QA et publication du candidat ; accord non consigné.</x:v>
+        <x:v>Requalifier QA ; accord et publication non consignés.</x:v>
       </x:c>
       <x:c r="AB85" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -8071,7 +8071,7 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA86" s="23" t="str">
-        <x:v>Requalifier QA et publication du candidat ; accord non consigné.</x:v>
+        <x:v>Requalifier QA ; accord et publication non consignés.</x:v>
       </x:c>
       <x:c r="AB86" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -8162,7 +8162,7 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA87" s="23" t="str">
-        <x:v>Requalifier QA et publication du candidat ; accord non consigné.</x:v>
+        <x:v>Requalifier QA ; accord et publication non consignés.</x:v>
       </x:c>
       <x:c r="AB87" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -8253,7 +8253,7 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA88" s="23" t="str">
-        <x:v>Requalifier QA et publication du candidat ; accord non consigné.</x:v>
+        <x:v>Requalifier QA ; accord et publication non consignés.</x:v>
       </x:c>
       <x:c r="AB88" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -8273,69 +8273,69 @@
         <x:v>79</x:v>
       </x:c>
       <x:c r="D89" s="24" t="str">
-        <x:v>À planifier</x:v>
+        <x:v>Lot 10</x:v>
       </x:c>
       <x:c r="E89" s="25" t="str">
         <x:v>Actions</x:v>
       </x:c>
       <x:c r="F89" s="24" t="str">
         <x:f>IF(AND(G89=8,COUNTIF(Q89:V89,"Atlas")=6),"Intégré","À faire")</x:f>
-        <x:v>À faire</x:v>
+        <x:v>Intégré</x:v>
       </x:c>
       <x:c r="G89" s="27" t="n">
         <x:f>COUNTIF(I89:P89,"Présent")</x:f>
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H89" s="24" t="str">
-        <x:v>À assembler</x:v>
+        <x:v>Archivé Drive</x:v>
       </x:c>
       <x:c r="I89" s="24" t="str">
-        <x:v>Référence</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="J89" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="K89" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="L89" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="M89" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="N89" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="O89" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="P89" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="Q89" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="R89" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="S89" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="T89" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="U89" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="V89" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="W89" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="X89" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="Y89" s="24" t="str">
         <x:v>Non consignée</x:v>
@@ -8344,13 +8344,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA89" s="23" t="str">
-        <x:v>Compléter le pack ; consigner QA, accord et publication.</x:v>
+        <x:v>Accord et publication du lot non consignés.</x:v>
       </x:c>
       <x:c r="AB89" s="21" t="str">
-        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
+        <x:v>fc0d47528b092ffae3e49cc020fbc27e902dc01b</x:v>
       </x:c>
       <x:c r="AC89" s="21" t="str">
-        <x:v>À intégrer</x:v>
+        <x:v>En cours</x:v>
       </x:c>
     </x:row>
     <x:row r="90" ht="40" customHeight="1">
@@ -8455,69 +8455,69 @@
         <x:v>81</x:v>
       </x:c>
       <x:c r="D91" s="24" t="str">
-        <x:v>À planifier</x:v>
+        <x:v>Lot 10</x:v>
       </x:c>
       <x:c r="E91" s="25" t="str">
         <x:v>Actions</x:v>
       </x:c>
       <x:c r="F91" s="24" t="str">
         <x:f>IF(AND(G91=8,COUNTIF(Q91:V91,"Atlas")=6),"Intégré","À faire")</x:f>
-        <x:v>À faire</x:v>
+        <x:v>Intégré</x:v>
       </x:c>
       <x:c r="G91" s="27" t="n">
         <x:f>COUNTIF(I91:P91,"Présent")</x:f>
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H91" s="24" t="str">
-        <x:v>À assembler</x:v>
+        <x:v>Archivé Drive</x:v>
       </x:c>
       <x:c r="I91" s="24" t="str">
-        <x:v>Référence</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="J91" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="K91" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="L91" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="M91" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="N91" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="O91" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="P91" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="Q91" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="R91" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="S91" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="T91" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="U91" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="V91" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="W91" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="X91" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="Y91" s="24" t="str">
         <x:v>Non consignée</x:v>
@@ -8526,13 +8526,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA91" s="23" t="str">
-        <x:v>Compléter le pack ; consigner QA, accord et publication.</x:v>
+        <x:v>Accord et publication du lot non consignés.</x:v>
       </x:c>
       <x:c r="AB91" s="21" t="str">
-        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
+        <x:v>fc0d47528b092ffae3e49cc020fbc27e902dc01b</x:v>
       </x:c>
       <x:c r="AC91" s="21" t="str">
-        <x:v>À intégrer</x:v>
+        <x:v>En cours</x:v>
       </x:c>
     </x:row>
     <x:row r="92" ht="40" customHeight="1">
@@ -8546,69 +8546,69 @@
         <x:v>82</x:v>
       </x:c>
       <x:c r="D92" s="24" t="str">
-        <x:v>À planifier</x:v>
+        <x:v>Lot 10</x:v>
       </x:c>
       <x:c r="E92" s="25" t="str">
         <x:v>Lieux</x:v>
       </x:c>
       <x:c r="F92" s="24" t="str">
         <x:f>IF(AND(G92=8,COUNTIF(Q92:V92,"Atlas")=6),"Intégré","À faire")</x:f>
-        <x:v>À faire</x:v>
+        <x:v>Intégré</x:v>
       </x:c>
       <x:c r="G92" s="27" t="n">
         <x:f>COUNTIF(I92:P92,"Présent")</x:f>
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H92" s="24" t="str">
-        <x:v>À assembler</x:v>
+        <x:v>Archivé Drive</x:v>
       </x:c>
       <x:c r="I92" s="24" t="str">
-        <x:v>Référence</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="J92" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="K92" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="L92" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="M92" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="N92" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="O92" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="P92" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="Q92" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="R92" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="S92" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="T92" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="U92" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="V92" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="W92" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="X92" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="Y92" s="24" t="str">
         <x:v>Non consignée</x:v>
@@ -8617,13 +8617,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA92" s="23" t="str">
-        <x:v>Compléter le pack ; consigner QA, accord et publication.</x:v>
+        <x:v>Accord et publication du lot non consignés.</x:v>
       </x:c>
       <x:c r="AB92" s="21" t="str">
-        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
+        <x:v>fc0d47528b092ffae3e49cc020fbc27e902dc01b</x:v>
       </x:c>
       <x:c r="AC92" s="21" t="str">
-        <x:v>À intégrer</x:v>
+        <x:v>En cours</x:v>
       </x:c>
     </x:row>
     <x:row r="93" ht="40" customHeight="1">
@@ -8728,69 +8728,69 @@
         <x:v>84</x:v>
       </x:c>
       <x:c r="D94" s="24" t="str">
-        <x:v>À planifier</x:v>
+        <x:v>Lot 10</x:v>
       </x:c>
       <x:c r="E94" s="25" t="str">
         <x:v>Personnes</x:v>
       </x:c>
       <x:c r="F94" s="24" t="str">
         <x:f>IF(AND(G94=8,COUNTIF(Q94:V94,"Atlas")=6),"Intégré","À faire")</x:f>
-        <x:v>À faire</x:v>
+        <x:v>Intégré</x:v>
       </x:c>
       <x:c r="G94" s="27" t="n">
         <x:f>COUNTIF(I94:P94,"Présent")</x:f>
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H94" s="24" t="str">
-        <x:v>À assembler</x:v>
+        <x:v>Archivé Drive</x:v>
       </x:c>
       <x:c r="I94" s="24" t="str">
-        <x:v>Référence</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="J94" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="K94" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="L94" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="M94" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="N94" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="O94" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="P94" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="Q94" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="R94" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="S94" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="T94" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="U94" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="V94" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="W94" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="X94" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="Y94" s="24" t="str">
         <x:v>Non consignée</x:v>
@@ -8799,13 +8799,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA94" s="23" t="str">
-        <x:v>Compléter le pack ; consigner QA, accord et publication.</x:v>
+        <x:v>Accord et publication du lot non consignés.</x:v>
       </x:c>
       <x:c r="AB94" s="21" t="str">
-        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
+        <x:v>fc0d47528b092ffae3e49cc020fbc27e902dc01b</x:v>
       </x:c>
       <x:c r="AC94" s="21" t="str">
-        <x:v>À intégrer</x:v>
+        <x:v>En cours</x:v>
       </x:c>
     </x:row>
     <x:row r="95" ht="40" customHeight="1">
@@ -8819,69 +8819,69 @@
         <x:v>85</x:v>
       </x:c>
       <x:c r="D95" s="24" t="str">
-        <x:v>À planifier</x:v>
+        <x:v>Lot 10</x:v>
       </x:c>
       <x:c r="E95" s="25" t="str">
         <x:v>Ciel</x:v>
       </x:c>
       <x:c r="F95" s="24" t="str">
         <x:f>IF(AND(G95=8,COUNTIF(Q95:V95,"Atlas")=6),"Intégré","À faire")</x:f>
-        <x:v>À faire</x:v>
+        <x:v>Intégré</x:v>
       </x:c>
       <x:c r="G95" s="27" t="n">
         <x:f>COUNTIF(I95:P95,"Présent")</x:f>
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H95" s="24" t="str">
-        <x:v>À assembler</x:v>
+        <x:v>Archivé Drive</x:v>
       </x:c>
       <x:c r="I95" s="24" t="str">
-        <x:v>Référence</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="J95" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="K95" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="L95" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="M95" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="N95" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="O95" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="P95" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="Q95" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="R95" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="S95" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="T95" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="U95" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="V95" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="W95" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="X95" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="Y95" s="24" t="str">
         <x:v>Non consignée</x:v>
@@ -8890,13 +8890,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA95" s="23" t="str">
-        <x:v>Compléter le pack ; consigner QA, accord et publication.</x:v>
+        <x:v>Accord et publication du lot non consignés.</x:v>
       </x:c>
       <x:c r="AB95" s="21" t="str">
-        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
+        <x:v>fc0d47528b092ffae3e49cc020fbc27e902dc01b</x:v>
       </x:c>
       <x:c r="AC95" s="21" t="str">
-        <x:v>À intégrer</x:v>
+        <x:v>En cours</x:v>
       </x:c>
     </x:row>
     <x:row r="96" ht="40" customHeight="1">
@@ -8910,69 +8910,69 @@
         <x:v>86</x:v>
       </x:c>
       <x:c r="D96" s="24" t="str">
-        <x:v>À planifier</x:v>
+        <x:v>Lot 10</x:v>
       </x:c>
       <x:c r="E96" s="25" t="str">
         <x:v>Nature</x:v>
       </x:c>
       <x:c r="F96" s="24" t="str">
         <x:f>IF(AND(G96=8,COUNTIF(Q96:V96,"Atlas")=6),"Intégré","À faire")</x:f>
-        <x:v>À faire</x:v>
+        <x:v>Intégré</x:v>
       </x:c>
       <x:c r="G96" s="27" t="n">
         <x:f>COUNTIF(I96:P96,"Présent")</x:f>
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H96" s="24" t="str">
-        <x:v>À assembler</x:v>
+        <x:v>Archivé Drive</x:v>
       </x:c>
       <x:c r="I96" s="24" t="str">
-        <x:v>Référence</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="J96" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="K96" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="L96" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="M96" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="N96" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="O96" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="P96" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="Q96" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="R96" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="S96" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="T96" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="U96" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="V96" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="W96" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="X96" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="Y96" s="24" t="str">
         <x:v>Non consignée</x:v>
@@ -8981,13 +8981,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA96" s="23" t="str">
-        <x:v>Compléter le pack ; consigner QA, accord et publication.</x:v>
+        <x:v>Accord et publication du lot non consignés.</x:v>
       </x:c>
       <x:c r="AB96" s="21" t="str">
-        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
+        <x:v>fc0d47528b092ffae3e49cc020fbc27e902dc01b</x:v>
       </x:c>
       <x:c r="AC96" s="21" t="str">
-        <x:v>À intégrer</x:v>
+        <x:v>En cours</x:v>
       </x:c>
     </x:row>
     <x:row r="97" ht="40" customHeight="1">
@@ -9072,7 +9072,7 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA97" s="23" t="str">
-        <x:v>Accord et publication du lot non consignés.</x:v>
+        <x:v>QA actuelle ; accord et publication non consignés.</x:v>
       </x:c>
       <x:c r="AB97" s="21" t="str">
         <x:v>9184f780a23f21687350020fa3448d58e4e0aadd</x:v>
@@ -9163,7 +9163,7 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA98" s="23" t="str">
-        <x:v>Accord et publication du lot non consignés.</x:v>
+        <x:v>QA actuelle ; accord et publication non consignés.</x:v>
       </x:c>
       <x:c r="AB98" s="21" t="str">
         <x:v>9184f780a23f21687350020fa3448d58e4e0aadd</x:v>
@@ -9254,7 +9254,7 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA99" s="23" t="str">
-        <x:v>Accord et publication du lot non consignés.</x:v>
+        <x:v>QA actuelle ; accord et publication non consignés.</x:v>
       </x:c>
       <x:c r="AB99" s="21" t="str">
         <x:v>9184f780a23f21687350020fa3448d58e4e0aadd</x:v>
@@ -9345,7 +9345,7 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA100" s="23" t="str">
-        <x:v>Accord et publication du lot non consignés.</x:v>
+        <x:v>QA actuelle ; accord et publication non consignés.</x:v>
       </x:c>
       <x:c r="AB100" s="21" t="str">
         <x:v>9184f780a23f21687350020fa3448d58e4e0aadd</x:v>
@@ -9527,7 +9527,7 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA102" s="23" t="str">
-        <x:v>Accord et publication du lot non consignés.</x:v>
+        <x:v>QA actuelle ; accord et publication non consignés.</x:v>
       </x:c>
       <x:c r="AB102" s="21" t="str">
         <x:v>9184f780a23f21687350020fa3448d58e4e0aadd</x:v>
@@ -9638,63 +9638,63 @@
         <x:v>94</x:v>
       </x:c>
       <x:c r="D104" s="24" t="str">
-        <x:v>À planifier</x:v>
+        <x:v>Lot 09</x:v>
       </x:c>
       <x:c r="E104" s="25" t="str">
         <x:v>Animaux</x:v>
       </x:c>
       <x:c r="F104" s="24" t="str">
         <x:f>IF(AND(G104=8,COUNTIF(Q104:V104,"Atlas")=6),"Intégré","À faire")</x:f>
-        <x:v>À faire</x:v>
+        <x:v>Intégré</x:v>
       </x:c>
       <x:c r="G104" s="27" t="n">
         <x:f>COUNTIF(I104:P104,"Présent")</x:f>
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H104" s="24" t="str">
-        <x:v>À assembler</x:v>
+        <x:v>Archivé local</x:v>
       </x:c>
       <x:c r="I104" s="24" t="str">
-        <x:v>Référence</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="J104" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="K104" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="L104" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="M104" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="N104" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="O104" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="P104" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="Q104" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="R104" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="S104" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="T104" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="U104" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="V104" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="W104" s="24" t="str">
         <x:v>Non consignée</x:v>
@@ -9709,13 +9709,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA104" s="23" t="str">
-        <x:v>Compléter le pack ; consigner QA, accord et publication.</x:v>
+        <x:v>Requalifier QA ; accord et publication non consignés.</x:v>
       </x:c>
       <x:c r="AB104" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC104" s="21" t="str">
-        <x:v>À intégrer</x:v>
+        <x:v>En cours</x:v>
       </x:c>
     </x:row>
     <x:row r="105" ht="40" customHeight="1">
@@ -9729,63 +9729,63 @@
         <x:v>95</x:v>
       </x:c>
       <x:c r="D105" s="24" t="str">
-        <x:v>À planifier</x:v>
+        <x:v>Lot 09</x:v>
       </x:c>
       <x:c r="E105" s="25" t="str">
         <x:v>Objets</x:v>
       </x:c>
       <x:c r="F105" s="24" t="str">
         <x:f>IF(AND(G105=8,COUNTIF(Q105:V105,"Atlas")=6),"Intégré","À faire")</x:f>
-        <x:v>À faire</x:v>
+        <x:v>Intégré</x:v>
       </x:c>
       <x:c r="G105" s="27" t="n">
         <x:f>COUNTIF(I105:P105,"Présent")</x:f>
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H105" s="24" t="str">
-        <x:v>À assembler</x:v>
+        <x:v>Archivé local</x:v>
       </x:c>
       <x:c r="I105" s="24" t="str">
-        <x:v>Référence</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="J105" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="K105" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="L105" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="M105" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="N105" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="O105" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="P105" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="Q105" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="R105" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="S105" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="T105" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="U105" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="V105" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="W105" s="24" t="str">
         <x:v>Non consignée</x:v>
@@ -9800,13 +9800,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA105" s="23" t="str">
-        <x:v>Compléter le pack ; consigner QA, accord et publication.</x:v>
+        <x:v>Requalifier QA ; accord et publication non consignés.</x:v>
       </x:c>
       <x:c r="AB105" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC105" s="21" t="str">
-        <x:v>À intégrer</x:v>
+        <x:v>En cours</x:v>
       </x:c>
     </x:row>
     <x:row r="106" ht="40" customHeight="1">
@@ -9891,7 +9891,7 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA106" s="23" t="str">
-        <x:v>Accord et publication du lot non consignés.</x:v>
+        <x:v>QA actuelle ; accord et publication non consignés.</x:v>
       </x:c>
       <x:c r="AB106" s="21" t="str">
         <x:v>9184f780a23f21687350020fa3448d58e4e0aadd</x:v>
@@ -9911,69 +9911,69 @@
         <x:v>97</x:v>
       </x:c>
       <x:c r="D107" s="24" t="str">
-        <x:v>À planifier</x:v>
+        <x:v>Lot 10</x:v>
       </x:c>
       <x:c r="E107" s="25" t="str">
         <x:v>Objets</x:v>
       </x:c>
       <x:c r="F107" s="24" t="str">
         <x:f>IF(AND(G107=8,COUNTIF(Q107:V107,"Atlas")=6),"Intégré","À faire")</x:f>
-        <x:v>À faire</x:v>
+        <x:v>Intégré</x:v>
       </x:c>
       <x:c r="G107" s="27" t="n">
         <x:f>COUNTIF(I107:P107,"Présent")</x:f>
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H107" s="24" t="str">
-        <x:v>À assembler</x:v>
+        <x:v>Archivé Drive</x:v>
       </x:c>
       <x:c r="I107" s="24" t="str">
-        <x:v>Référence</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="J107" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="K107" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="L107" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="M107" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="N107" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="O107" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="P107" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="Q107" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="R107" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="S107" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="T107" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="U107" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="V107" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="W107" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="X107" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="Y107" s="24" t="str">
         <x:v>Non consignée</x:v>
@@ -9982,13 +9982,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA107" s="23" t="str">
-        <x:v>Compléter le pack ; consigner QA, accord et publication.</x:v>
+        <x:v>Accord et publication du lot non consignés.</x:v>
       </x:c>
       <x:c r="AB107" s="21" t="str">
-        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
+        <x:v>fc0d47528b092ffae3e49cc020fbc27e902dc01b</x:v>
       </x:c>
       <x:c r="AC107" s="21" t="str">
-        <x:v>À intégrer</x:v>
+        <x:v>En cours</x:v>
       </x:c>
     </x:row>
     <x:row r="108" ht="40" customHeight="1">
@@ -10639,69 +10639,69 @@
         <x:v>105</x:v>
       </x:c>
       <x:c r="D115" s="24" t="str">
-        <x:v>À planifier</x:v>
+        <x:v>Lot 10</x:v>
       </x:c>
       <x:c r="E115" s="25" t="str">
         <x:v>Lieux</x:v>
       </x:c>
       <x:c r="F115" s="24" t="str">
         <x:f>IF(AND(G115=8,COUNTIF(Q115:V115,"Atlas")=6),"Intégré","À faire")</x:f>
-        <x:v>À faire</x:v>
+        <x:v>Intégré</x:v>
       </x:c>
       <x:c r="G115" s="27" t="n">
         <x:f>COUNTIF(I115:P115,"Présent")</x:f>
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H115" s="24" t="str">
-        <x:v>À assembler</x:v>
+        <x:v>Archivé Drive</x:v>
       </x:c>
       <x:c r="I115" s="24" t="str">
-        <x:v>Référence</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="J115" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="K115" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="L115" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="M115" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="N115" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="O115" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="P115" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="Q115" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="R115" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="S115" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="T115" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="U115" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="V115" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="W115" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="X115" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="Y115" s="24" t="str">
         <x:v>Non consignée</x:v>
@@ -10710,13 +10710,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA115" s="23" t="str">
-        <x:v>Compléter le pack ; consigner QA, accord et publication.</x:v>
+        <x:v>Accord et publication du lot non consignés.</x:v>
       </x:c>
       <x:c r="AB115" s="21" t="str">
-        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
+        <x:v>fc0d47528b092ffae3e49cc020fbc27e902dc01b</x:v>
       </x:c>
       <x:c r="AC115" s="21" t="str">
-        <x:v>À intégrer</x:v>
+        <x:v>En cours</x:v>
       </x:c>
     </x:row>
     <x:row r="116" ht="40" customHeight="1">
@@ -10983,7 +10983,7 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA118" s="23" t="str">
-        <x:v>Accord et publication du lot non consignés.</x:v>
+        <x:v>QA actuelle ; accord et publication non consignés.</x:v>
       </x:c>
       <x:c r="AB118" s="21" t="str">
         <x:v>9184f780a23f21687350020fa3448d58e4e0aadd</x:v>
@@ -11640,69 +11640,69 @@
         <x:v>116</x:v>
       </x:c>
       <x:c r="D126" s="24" t="str">
-        <x:v>À planifier</x:v>
+        <x:v>Lot 10</x:v>
       </x:c>
       <x:c r="E126" s="25" t="str">
         <x:v>Personnes</x:v>
       </x:c>
       <x:c r="F126" s="24" t="str">
         <x:f>IF(AND(G126=8,COUNTIF(Q126:V126,"Atlas")=6),"Intégré","À faire")</x:f>
-        <x:v>À faire</x:v>
+        <x:v>Intégré</x:v>
       </x:c>
       <x:c r="G126" s="27" t="n">
         <x:f>COUNTIF(I126:P126,"Présent")</x:f>
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H126" s="24" t="str">
-        <x:v>À assembler</x:v>
+        <x:v>Archivé Drive</x:v>
       </x:c>
       <x:c r="I126" s="24" t="str">
-        <x:v>Référence</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="J126" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="K126" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="L126" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="M126" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="N126" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="O126" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="P126" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="Q126" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="R126" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="S126" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="T126" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="U126" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="V126" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="W126" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="X126" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="Y126" s="24" t="str">
         <x:v>Non consignée</x:v>
@@ -11711,13 +11711,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA126" s="23" t="str">
-        <x:v>Compléter le pack ; consigner QA, accord et publication.</x:v>
+        <x:v>Accord et publication du lot non consignés.</x:v>
       </x:c>
       <x:c r="AB126" s="21" t="str">
-        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
+        <x:v>fc0d47528b092ffae3e49cc020fbc27e902dc01b</x:v>
       </x:c>
       <x:c r="AC126" s="21" t="str">
-        <x:v>À intégrer</x:v>
+        <x:v>En cours</x:v>
       </x:c>
     </x:row>
     <x:row r="127" ht="40" customHeight="1">
@@ -11893,7 +11893,7 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA128" s="23" t="str">
-        <x:v>Accord et publication du lot non consignés.</x:v>
+        <x:v>QA actuelle ; accord et publication non consignés.</x:v>
       </x:c>
       <x:c r="AB128" s="21" t="str">
         <x:v>9184f780a23f21687350020fa3448d58e4e0aadd</x:v>
@@ -12277,69 +12277,69 @@
         <x:v>123</x:v>
       </x:c>
       <x:c r="D133" s="24" t="str">
-        <x:v>À planifier</x:v>
+        <x:v>Lot 10</x:v>
       </x:c>
       <x:c r="E133" s="25" t="str">
         <x:v>Lieux</x:v>
       </x:c>
       <x:c r="F133" s="24" t="str">
         <x:f>IF(AND(G133=8,COUNTIF(Q133:V133,"Atlas")=6),"Intégré","À faire")</x:f>
-        <x:v>À faire</x:v>
+        <x:v>Intégré</x:v>
       </x:c>
       <x:c r="G133" s="27" t="n">
         <x:f>COUNTIF(I133:P133,"Présent")</x:f>
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H133" s="24" t="str">
-        <x:v>À assembler</x:v>
+        <x:v>Archivé Drive</x:v>
       </x:c>
       <x:c r="I133" s="24" t="str">
-        <x:v>Référence</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="J133" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="K133" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="L133" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="M133" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="N133" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="O133" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="P133" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="Q133" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="R133" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="S133" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="T133" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="U133" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="V133" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="W133" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="X133" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="Y133" s="24" t="str">
         <x:v>Non consignée</x:v>
@@ -12348,13 +12348,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA133" s="23" t="str">
-        <x:v>Compléter le pack ; consigner QA, accord et publication.</x:v>
+        <x:v>Accord et publication du lot non consignés.</x:v>
       </x:c>
       <x:c r="AB133" s="21" t="str">
-        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
+        <x:v>fc0d47528b092ffae3e49cc020fbc27e902dc01b</x:v>
       </x:c>
       <x:c r="AC133" s="21" t="str">
-        <x:v>À intégrer</x:v>
+        <x:v>En cours</x:v>
       </x:c>
     </x:row>
     <x:row r="134" ht="40" customHeight="1">
@@ -12530,7 +12530,7 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA135" s="23" t="str">
-        <x:v>Accord et publication du lot non consignés.</x:v>
+        <x:v>QA actuelle ; accord et publication non consignés.</x:v>
       </x:c>
       <x:c r="AB135" s="21" t="str">
         <x:v>9184f780a23f21687350020fa3448d58e4e0aadd</x:v>
@@ -12823,69 +12823,69 @@
         <x:v>129</x:v>
       </x:c>
       <x:c r="D139" s="24" t="str">
-        <x:v>À planifier</x:v>
+        <x:v>Lot 10</x:v>
       </x:c>
       <x:c r="E139" s="25" t="str">
         <x:v>Actions</x:v>
       </x:c>
       <x:c r="F139" s="24" t="str">
         <x:f>IF(AND(G139=8,COUNTIF(Q139:V139,"Atlas")=6),"Intégré","À faire")</x:f>
-        <x:v>À faire</x:v>
+        <x:v>Intégré</x:v>
       </x:c>
       <x:c r="G139" s="27" t="n">
         <x:f>COUNTIF(I139:P139,"Présent")</x:f>
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H139" s="24" t="str">
-        <x:v>À assembler</x:v>
+        <x:v>Archivé Drive</x:v>
       </x:c>
       <x:c r="I139" s="24" t="str">
-        <x:v>Référence</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="J139" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="K139" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="L139" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="M139" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="N139" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="O139" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="P139" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="Q139" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="R139" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="S139" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="T139" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="U139" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="V139" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="W139" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="X139" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="Y139" s="24" t="str">
         <x:v>Non consignée</x:v>
@@ -12894,13 +12894,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA139" s="23" t="str">
-        <x:v>Compléter le pack ; consigner QA, accord et publication.</x:v>
+        <x:v>Accord et publication du lot non consignés.</x:v>
       </x:c>
       <x:c r="AB139" s="21" t="str">
-        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
+        <x:v>fc0d47528b092ffae3e49cc020fbc27e902dc01b</x:v>
       </x:c>
       <x:c r="AC139" s="21" t="str">
-        <x:v>À intégrer</x:v>
+        <x:v>En cours</x:v>
       </x:c>
     </x:row>
     <x:row r="140" ht="40" customHeight="1">
@@ -12914,63 +12914,63 @@
         <x:v>130</x:v>
       </x:c>
       <x:c r="D140" s="24" t="str">
-        <x:v>À planifier</x:v>
+        <x:v>Lot 09</x:v>
       </x:c>
       <x:c r="E140" s="25" t="str">
         <x:v>Nature</x:v>
       </x:c>
       <x:c r="F140" s="24" t="str">
         <x:f>IF(AND(G140=8,COUNTIF(Q140:V140,"Atlas")=6),"Intégré","À faire")</x:f>
-        <x:v>À faire</x:v>
+        <x:v>Intégré</x:v>
       </x:c>
       <x:c r="G140" s="27" t="n">
         <x:f>COUNTIF(I140:P140,"Présent")</x:f>
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H140" s="24" t="str">
-        <x:v>À assembler</x:v>
+        <x:v>Archivé local</x:v>
       </x:c>
       <x:c r="I140" s="24" t="str">
-        <x:v>Référence</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="J140" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="K140" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="L140" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="M140" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="N140" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="O140" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="P140" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="Q140" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="R140" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="S140" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="T140" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="U140" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="V140" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="W140" s="24" t="str">
         <x:v>Non consignée</x:v>
@@ -12985,13 +12985,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA140" s="23" t="str">
-        <x:v>Compléter le pack ; consigner QA, accord et publication.</x:v>
+        <x:v>Requalifier QA ; accord et publication non consignés.</x:v>
       </x:c>
       <x:c r="AB140" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC140" s="21" t="str">
-        <x:v>À intégrer</x:v>
+        <x:v>En cours</x:v>
       </x:c>
     </x:row>
     <x:row r="141" ht="40" customHeight="1">
@@ -13076,7 +13076,7 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA141" s="23" t="str">
-        <x:v>Accord et publication du lot non consignés.</x:v>
+        <x:v>QA actuelle ; accord et publication non consignés.</x:v>
       </x:c>
       <x:c r="AB141" s="21" t="str">
         <x:v>9184f780a23f21687350020fa3448d58e4e0aadd</x:v>
@@ -13440,7 +13440,7 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA145" s="23" t="str">
-        <x:v>Accord et publication du lot non consignés.</x:v>
+        <x:v>QA actuelle ; accord et publication non consignés.</x:v>
       </x:c>
       <x:c r="AB145" s="21" t="str">
         <x:v>9184f780a23f21687350020fa3448d58e4e0aadd</x:v>
@@ -13551,69 +13551,69 @@
         <x:v>137</x:v>
       </x:c>
       <x:c r="D147" s="24" t="str">
-        <x:v>À planifier</x:v>
+        <x:v>Lot 10</x:v>
       </x:c>
       <x:c r="E147" s="25" t="str">
         <x:v>Actions</x:v>
       </x:c>
       <x:c r="F147" s="24" t="str">
         <x:f>IF(AND(G147=8,COUNTIF(Q147:V147,"Atlas")=6),"Intégré","À faire")</x:f>
-        <x:v>À faire</x:v>
+        <x:v>Intégré</x:v>
       </x:c>
       <x:c r="G147" s="27" t="n">
         <x:f>COUNTIF(I147:P147,"Présent")</x:f>
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H147" s="24" t="str">
-        <x:v>À assembler</x:v>
+        <x:v>Archivé Drive</x:v>
       </x:c>
       <x:c r="I147" s="24" t="str">
-        <x:v>Référence</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="J147" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="K147" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="L147" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="M147" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="N147" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="O147" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="P147" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="Q147" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="R147" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="S147" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="T147" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="U147" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="V147" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="W147" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="X147" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="Y147" s="24" t="str">
         <x:v>Non consignée</x:v>
@@ -13622,13 +13622,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA147" s="23" t="str">
-        <x:v>Compléter le pack ; consigner QA, accord et publication.</x:v>
+        <x:v>Accord et publication du lot non consignés.</x:v>
       </x:c>
       <x:c r="AB147" s="21" t="str">
-        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
+        <x:v>fc0d47528b092ffae3e49cc020fbc27e902dc01b</x:v>
       </x:c>
       <x:c r="AC147" s="21" t="str">
-        <x:v>À intégrer</x:v>
+        <x:v>En cours</x:v>
       </x:c>
     </x:row>
     <x:row r="148" ht="40" customHeight="1">
@@ -13895,7 +13895,7 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA150" s="23" t="str">
-        <x:v>Accord et publication du lot non consignés.</x:v>
+        <x:v>QA actuelle ; accord et publication non consignés.</x:v>
       </x:c>
       <x:c r="AB150" s="21" t="str">
         <x:v>9184f780a23f21687350020fa3448d58e4e0aadd</x:v>
@@ -13986,7 +13986,7 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA151" s="23" t="str">
-        <x:v>Accord et publication du lot non consignés.</x:v>
+        <x:v>QA actuelle ; accord et publication non consignés.</x:v>
       </x:c>
       <x:c r="AB151" s="21" t="str">
         <x:v>9184f780a23f21687350020fa3448d58e4e0aadd</x:v>
@@ -14077,7 +14077,7 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA152" s="23" t="str">
-        <x:v>Accord et publication du lot non consignés.</x:v>
+        <x:v>QA actuelle ; accord et publication non consignés.</x:v>
       </x:c>
       <x:c r="AB152" s="21" t="str">
         <x:v>9184f780a23f21687350020fa3448d58e4e0aadd</x:v>
@@ -14259,7 +14259,7 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA154" s="23" t="str">
-        <x:v>Accord et publication du lot non consignés.</x:v>
+        <x:v>QA actuelle ; accord et publication non consignés.</x:v>
       </x:c>
       <x:c r="AB154" s="21" t="str">
         <x:v>9184f780a23f21687350020fa3448d58e4e0aadd</x:v>
@@ -14461,69 +14461,69 @@
         <x:v>147</x:v>
       </x:c>
       <x:c r="D157" s="24" t="str">
-        <x:v>À planifier</x:v>
+        <x:v>Lot 10</x:v>
       </x:c>
       <x:c r="E157" s="25" t="str">
         <x:v>Personnes</x:v>
       </x:c>
       <x:c r="F157" s="24" t="str">
         <x:f>IF(AND(G157=8,COUNTIF(Q157:V157,"Atlas")=6),"Intégré","À faire")</x:f>
-        <x:v>À faire</x:v>
+        <x:v>Intégré</x:v>
       </x:c>
       <x:c r="G157" s="27" t="n">
         <x:f>COUNTIF(I157:P157,"Présent")</x:f>
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H157" s="24" t="str">
-        <x:v>À assembler</x:v>
+        <x:v>Archivé Drive</x:v>
       </x:c>
       <x:c r="I157" s="24" t="str">
-        <x:v>Référence</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="J157" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="K157" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="L157" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="M157" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="N157" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="O157" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="P157" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="Q157" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="R157" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="S157" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="T157" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="U157" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="V157" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="W157" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="X157" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="Y157" s="24" t="str">
         <x:v>Non consignée</x:v>
@@ -14532,13 +14532,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA157" s="23" t="str">
-        <x:v>Compléter le pack ; consigner QA, accord et publication.</x:v>
+        <x:v>Accord et publication du lot non consignés.</x:v>
       </x:c>
       <x:c r="AB157" s="21" t="str">
-        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
+        <x:v>fc0d47528b092ffae3e49cc020fbc27e902dc01b</x:v>
       </x:c>
       <x:c r="AC157" s="21" t="str">
-        <x:v>À intégrer</x:v>
+        <x:v>En cours</x:v>
       </x:c>
     </x:row>
     <x:row r="158" ht="40" customHeight="1">
@@ -14552,69 +14552,69 @@
         <x:v>148</x:v>
       </x:c>
       <x:c r="D158" s="24" t="str">
-        <x:v>À planifier</x:v>
+        <x:v>Lot 10</x:v>
       </x:c>
       <x:c r="E158" s="25" t="str">
         <x:v>Personnes</x:v>
       </x:c>
       <x:c r="F158" s="24" t="str">
         <x:f>IF(AND(G158=8,COUNTIF(Q158:V158,"Atlas")=6),"Intégré","À faire")</x:f>
-        <x:v>À faire</x:v>
+        <x:v>Intégré</x:v>
       </x:c>
       <x:c r="G158" s="27" t="n">
         <x:f>COUNTIF(I158:P158,"Présent")</x:f>
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H158" s="24" t="str">
-        <x:v>À assembler</x:v>
+        <x:v>Archivé Drive</x:v>
       </x:c>
       <x:c r="I158" s="24" t="str">
-        <x:v>Référence</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="J158" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="K158" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="L158" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="M158" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="N158" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="O158" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="P158" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="Q158" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="R158" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="S158" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="T158" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="U158" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="V158" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="W158" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="X158" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="Y158" s="24" t="str">
         <x:v>Non consignée</x:v>
@@ -14623,13 +14623,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA158" s="23" t="str">
-        <x:v>Compléter le pack ; consigner QA, accord et publication.</x:v>
+        <x:v>Accord et publication du lot non consignés.</x:v>
       </x:c>
       <x:c r="AB158" s="21" t="str">
-        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
+        <x:v>fc0d47528b092ffae3e49cc020fbc27e902dc01b</x:v>
       </x:c>
       <x:c r="AC158" s="21" t="str">
-        <x:v>À intégrer</x:v>
+        <x:v>En cours</x:v>
       </x:c>
     </x:row>
     <x:row r="159" ht="40" customHeight="1">
@@ -14643,69 +14643,69 @@
         <x:v>149</x:v>
       </x:c>
       <x:c r="D159" s="24" t="str">
-        <x:v>À planifier</x:v>
+        <x:v>Lot 10</x:v>
       </x:c>
       <x:c r="E159" s="25" t="str">
         <x:v>Personnes</x:v>
       </x:c>
       <x:c r="F159" s="24" t="str">
         <x:f>IF(AND(G159=8,COUNTIF(Q159:V159,"Atlas")=6),"Intégré","À faire")</x:f>
-        <x:v>À faire</x:v>
+        <x:v>Intégré</x:v>
       </x:c>
       <x:c r="G159" s="27" t="n">
         <x:f>COUNTIF(I159:P159,"Présent")</x:f>
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H159" s="24" t="str">
-        <x:v>À assembler</x:v>
+        <x:v>Archivé Drive</x:v>
       </x:c>
       <x:c r="I159" s="24" t="str">
-        <x:v>Référence</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="J159" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="K159" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="L159" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="M159" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="N159" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="O159" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="P159" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="Q159" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="R159" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="S159" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="T159" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="U159" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="V159" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="W159" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="X159" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="Y159" s="24" t="str">
         <x:v>Non consignée</x:v>
@@ -14714,13 +14714,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA159" s="23" t="str">
-        <x:v>Compléter le pack ; consigner QA, accord et publication.</x:v>
+        <x:v>Accord et publication du lot non consignés.</x:v>
       </x:c>
       <x:c r="AB159" s="21" t="str">
-        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
+        <x:v>fc0d47528b092ffae3e49cc020fbc27e902dc01b</x:v>
       </x:c>
       <x:c r="AC159" s="21" t="str">
-        <x:v>À intégrer</x:v>
+        <x:v>En cours</x:v>
       </x:c>
     </x:row>
     <x:row r="160" ht="40" customHeight="1">
@@ -14987,7 +14987,7 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA162" s="23" t="str">
-        <x:v>Accord et publication du lot non consignés.</x:v>
+        <x:v>QA actuelle ; accord et publication non consignés.</x:v>
       </x:c>
       <x:c r="AB162" s="21" t="str">
         <x:v>9184f780a23f21687350020fa3448d58e4e0aadd</x:v>
@@ -15007,63 +15007,63 @@
         <x:v>153</x:v>
       </x:c>
       <x:c r="D163" s="24" t="str">
-        <x:v>À planifier</x:v>
+        <x:v>Lot 09</x:v>
       </x:c>
       <x:c r="E163" s="25" t="str">
         <x:v>Lieux</x:v>
       </x:c>
       <x:c r="F163" s="24" t="str">
         <x:f>IF(AND(G163=8,COUNTIF(Q163:V163,"Atlas")=6),"Intégré","À faire")</x:f>
-        <x:v>À faire</x:v>
+        <x:v>Intégré</x:v>
       </x:c>
       <x:c r="G163" s="27" t="n">
         <x:f>COUNTIF(I163:P163,"Présent")</x:f>
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H163" s="24" t="str">
-        <x:v>À assembler</x:v>
+        <x:v>Archivé local</x:v>
       </x:c>
       <x:c r="I163" s="24" t="str">
-        <x:v>Référence</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="J163" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="K163" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="L163" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="M163" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="N163" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="O163" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="P163" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="Q163" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="R163" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="S163" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="T163" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="U163" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="V163" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="W163" s="24" t="str">
         <x:v>Non consignée</x:v>
@@ -15078,13 +15078,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA163" s="23" t="str">
-        <x:v>Compléter le pack ; consigner QA, accord et publication.</x:v>
+        <x:v>Requalifier QA ; accord et publication non consignés.</x:v>
       </x:c>
       <x:c r="AB163" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC163" s="21" t="str">
-        <x:v>À intégrer</x:v>
+        <x:v>En cours</x:v>
       </x:c>
     </x:row>
     <x:row r="164" ht="40" customHeight="1">
@@ -15280,63 +15280,63 @@
         <x:v>156</x:v>
       </x:c>
       <x:c r="D166" s="24" t="str">
-        <x:v>À planifier</x:v>
+        <x:v>Lot 09</x:v>
       </x:c>
       <x:c r="E166" s="25" t="str">
         <x:v>Animaux</x:v>
       </x:c>
       <x:c r="F166" s="24" t="str">
         <x:f>IF(AND(G166=8,COUNTIF(Q166:V166,"Atlas")=6),"Intégré","À faire")</x:f>
-        <x:v>À faire</x:v>
+        <x:v>Intégré</x:v>
       </x:c>
       <x:c r="G166" s="27" t="n">
         <x:f>COUNTIF(I166:P166,"Présent")</x:f>
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H166" s="24" t="str">
-        <x:v>À assembler</x:v>
+        <x:v>Archivé local</x:v>
       </x:c>
       <x:c r="I166" s="24" t="str">
-        <x:v>Référence</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="J166" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="K166" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="L166" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="M166" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="N166" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="O166" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="P166" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="Q166" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="R166" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="S166" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="T166" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="U166" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="V166" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="W166" s="24" t="str">
         <x:v>Non consignée</x:v>
@@ -15351,13 +15351,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA166" s="23" t="str">
-        <x:v>Compléter le pack ; consigner QA, accord et publication.</x:v>
+        <x:v>Requalifier QA ; accord et publication non consignés.</x:v>
       </x:c>
       <x:c r="AB166" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC166" s="21" t="str">
-        <x:v>À intégrer</x:v>
+        <x:v>En cours</x:v>
       </x:c>
     </x:row>
     <x:row r="167" ht="40" customHeight="1">
@@ -15442,7 +15442,7 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA167" s="23" t="str">
-        <x:v>Accord et publication du lot non consignés.</x:v>
+        <x:v>QA actuelle ; accord et publication non consignés.</x:v>
       </x:c>
       <x:c r="AB167" s="21" t="str">
         <x:v>9184f780a23f21687350020fa3448d58e4e0aadd</x:v>
@@ -15735,69 +15735,69 @@
         <x:v>161</x:v>
       </x:c>
       <x:c r="D171" s="24" t="str">
-        <x:v>À planifier</x:v>
+        <x:v>Lot 10</x:v>
       </x:c>
       <x:c r="E171" s="25" t="str">
         <x:v>Personnes</x:v>
       </x:c>
       <x:c r="F171" s="24" t="str">
         <x:f>IF(AND(G171=8,COUNTIF(Q171:V171,"Atlas")=6),"Intégré","À faire")</x:f>
-        <x:v>À faire</x:v>
+        <x:v>Intégré</x:v>
       </x:c>
       <x:c r="G171" s="27" t="n">
         <x:f>COUNTIF(I171:P171,"Présent")</x:f>
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H171" s="24" t="str">
-        <x:v>À assembler</x:v>
+        <x:v>Archivé Drive</x:v>
       </x:c>
       <x:c r="I171" s="24" t="str">
-        <x:v>Référence</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="J171" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="K171" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="L171" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="M171" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="N171" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="O171" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="P171" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="Q171" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="R171" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="S171" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="T171" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="U171" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="V171" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="W171" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="X171" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="Y171" s="24" t="str">
         <x:v>Non consignée</x:v>
@@ -15806,13 +15806,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA171" s="23" t="str">
-        <x:v>Compléter le pack ; consigner QA, accord et publication.</x:v>
+        <x:v>Accord et publication du lot non consignés.</x:v>
       </x:c>
       <x:c r="AB171" s="21" t="str">
-        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
+        <x:v>fc0d47528b092ffae3e49cc020fbc27e902dc01b</x:v>
       </x:c>
       <x:c r="AC171" s="21" t="str">
-        <x:v>À intégrer</x:v>
+        <x:v>En cours</x:v>
       </x:c>
     </x:row>
     <x:row r="172" ht="40" customHeight="1">
@@ -15988,7 +15988,7 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA173" s="23" t="str">
-        <x:v>Accord et publication du lot non consignés.</x:v>
+        <x:v>QA actuelle ; accord et publication non consignés.</x:v>
       </x:c>
       <x:c r="AB173" s="21" t="str">
         <x:v>9184f780a23f21687350020fa3448d58e4e0aadd</x:v>
@@ -16463,69 +16463,69 @@
         <x:v>169</x:v>
       </x:c>
       <x:c r="D179" s="24" t="str">
-        <x:v>À planifier</x:v>
+        <x:v>Lot 10</x:v>
       </x:c>
       <x:c r="E179" s="25" t="str">
         <x:v>Lieux</x:v>
       </x:c>
       <x:c r="F179" s="24" t="str">
         <x:f>IF(AND(G179=8,COUNTIF(Q179:V179,"Atlas")=6),"Intégré","À faire")</x:f>
-        <x:v>À faire</x:v>
+        <x:v>Intégré</x:v>
       </x:c>
       <x:c r="G179" s="27" t="n">
         <x:f>COUNTIF(I179:P179,"Présent")</x:f>
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H179" s="24" t="str">
-        <x:v>À assembler</x:v>
+        <x:v>Archivé Drive</x:v>
       </x:c>
       <x:c r="I179" s="24" t="str">
-        <x:v>Référence</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="J179" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="K179" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="L179" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="M179" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="N179" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="O179" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="P179" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="Q179" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="R179" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="S179" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="T179" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="U179" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="V179" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="W179" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="X179" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="Y179" s="24" t="str">
         <x:v>Non consignée</x:v>
@@ -16534,13 +16534,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA179" s="23" t="str">
-        <x:v>Compléter le pack ; consigner QA, accord et publication.</x:v>
+        <x:v>Accord et publication du lot non consignés.</x:v>
       </x:c>
       <x:c r="AB179" s="21" t="str">
-        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
+        <x:v>fc0d47528b092ffae3e49cc020fbc27e902dc01b</x:v>
       </x:c>
       <x:c r="AC179" s="21" t="str">
-        <x:v>À intégrer</x:v>
+        <x:v>En cours</x:v>
       </x:c>
     </x:row>
     <x:row r="180" ht="40" customHeight="1">
@@ -16625,7 +16625,7 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA180" s="23" t="str">
-        <x:v>Accord et publication du lot non consignés.</x:v>
+        <x:v>QA actuelle ; accord et publication non consignés.</x:v>
       </x:c>
       <x:c r="AB180" s="21" t="str">
         <x:v>9184f780a23f21687350020fa3448d58e4e0aadd</x:v>
@@ -16989,7 +16989,7 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA184" s="23" t="str">
-        <x:v>Accord et publication du lot non consignés.</x:v>
+        <x:v>QA actuelle ; accord et publication non consignés.</x:v>
       </x:c>
       <x:c r="AB184" s="21" t="str">
         <x:v>9184f780a23f21687350020fa3448d58e4e0aadd</x:v>
@@ -17100,69 +17100,69 @@
         <x:v>176</x:v>
       </x:c>
       <x:c r="D186" s="24" t="str">
-        <x:v>À planifier</x:v>
+        <x:v>Lot 10</x:v>
       </x:c>
       <x:c r="E186" s="25" t="str">
         <x:v>Personnes</x:v>
       </x:c>
       <x:c r="F186" s="24" t="str">
         <x:f>IF(AND(G186=8,COUNTIF(Q186:V186,"Atlas")=6),"Intégré","À faire")</x:f>
-        <x:v>À faire</x:v>
+        <x:v>Intégré</x:v>
       </x:c>
       <x:c r="G186" s="27" t="n">
         <x:f>COUNTIF(I186:P186,"Présent")</x:f>
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H186" s="24" t="str">
-        <x:v>À assembler</x:v>
+        <x:v>Archivé Drive</x:v>
       </x:c>
       <x:c r="I186" s="24" t="str">
-        <x:v>Référence</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="J186" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="K186" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="L186" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="M186" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="N186" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="O186" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="P186" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="Q186" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="R186" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="S186" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="T186" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="U186" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="V186" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="W186" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="X186" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="Y186" s="24" t="str">
         <x:v>Non consignée</x:v>
@@ -17171,13 +17171,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA186" s="23" t="str">
-        <x:v>Compléter le pack ; consigner QA, accord et publication.</x:v>
+        <x:v>Accord et publication du lot non consignés.</x:v>
       </x:c>
       <x:c r="AB186" s="21" t="str">
-        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
+        <x:v>fc0d47528b092ffae3e49cc020fbc27e902dc01b</x:v>
       </x:c>
       <x:c r="AC186" s="21" t="str">
-        <x:v>À intégrer</x:v>
+        <x:v>En cours</x:v>
       </x:c>
     </x:row>
     <x:row r="187" ht="40" customHeight="1">
@@ -17191,69 +17191,69 @@
         <x:v>177</x:v>
       </x:c>
       <x:c r="D187" s="24" t="str">
-        <x:v>À planifier</x:v>
+        <x:v>Lot 10</x:v>
       </x:c>
       <x:c r="E187" s="25" t="str">
         <x:v>Personnes</x:v>
       </x:c>
       <x:c r="F187" s="24" t="str">
         <x:f>IF(AND(G187=8,COUNTIF(Q187:V187,"Atlas")=6),"Intégré","À faire")</x:f>
-        <x:v>À faire</x:v>
+        <x:v>Intégré</x:v>
       </x:c>
       <x:c r="G187" s="27" t="n">
         <x:f>COUNTIF(I187:P187,"Présent")</x:f>
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H187" s="24" t="str">
-        <x:v>À assembler</x:v>
+        <x:v>Archivé Drive</x:v>
       </x:c>
       <x:c r="I187" s="24" t="str">
-        <x:v>Référence</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="J187" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="K187" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="L187" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="M187" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="N187" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="O187" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="P187" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="Q187" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="R187" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="S187" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="T187" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="U187" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="V187" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="W187" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="X187" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="Y187" s="24" t="str">
         <x:v>Non consignée</x:v>
@@ -17262,13 +17262,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA187" s="23" t="str">
-        <x:v>Compléter le pack ; consigner QA, accord et publication.</x:v>
+        <x:v>Accord et publication du lot non consignés.</x:v>
       </x:c>
       <x:c r="AB187" s="21" t="str">
-        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
+        <x:v>fc0d47528b092ffae3e49cc020fbc27e902dc01b</x:v>
       </x:c>
       <x:c r="AC187" s="21" t="str">
-        <x:v>À intégrer</x:v>
+        <x:v>En cours</x:v>
       </x:c>
     </x:row>
     <x:row r="188" ht="40" customHeight="1">
@@ -17535,7 +17535,7 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA190" s="23" t="str">
-        <x:v>Accord et publication du lot non consignés.</x:v>
+        <x:v>QA actuelle ; accord et publication non consignés.</x:v>
       </x:c>
       <x:c r="AB190" s="21" t="str">
         <x:v>9184f780a23f21687350020fa3448d58e4e0aadd</x:v>
@@ -17626,7 +17626,7 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA191" s="23" t="str">
-        <x:v>Accord et publication du lot non consignés.</x:v>
+        <x:v>QA actuelle ; accord et publication non consignés.</x:v>
       </x:c>
       <x:c r="AB191" s="21" t="str">
         <x:v>9184f780a23f21687350020fa3448d58e4e0aadd</x:v>
@@ -17646,69 +17646,69 @@
         <x:v>182</x:v>
       </x:c>
       <x:c r="D192" s="24" t="str">
-        <x:v>À planifier</x:v>
+        <x:v>Lot 10</x:v>
       </x:c>
       <x:c r="E192" s="25" t="str">
         <x:v>Actions</x:v>
       </x:c>
       <x:c r="F192" s="24" t="str">
         <x:f>IF(AND(G192=8,COUNTIF(Q192:V192,"Atlas")=6),"Intégré","À faire")</x:f>
-        <x:v>À faire</x:v>
+        <x:v>Intégré</x:v>
       </x:c>
       <x:c r="G192" s="27" t="n">
         <x:f>COUNTIF(I192:P192,"Présent")</x:f>
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H192" s="24" t="str">
-        <x:v>À assembler</x:v>
+        <x:v>Archivé Drive</x:v>
       </x:c>
       <x:c r="I192" s="24" t="str">
-        <x:v>Référence</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="J192" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="K192" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="L192" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="M192" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="N192" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="O192" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="P192" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="Q192" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="R192" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="S192" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="T192" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="U192" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="V192" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="W192" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="X192" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="Y192" s="24" t="str">
         <x:v>Non consignée</x:v>
@@ -17717,13 +17717,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA192" s="23" t="str">
-        <x:v>Compléter le pack ; consigner QA, accord et publication.</x:v>
+        <x:v>Accord et publication du lot non consignés.</x:v>
       </x:c>
       <x:c r="AB192" s="21" t="str">
-        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
+        <x:v>fc0d47528b092ffae3e49cc020fbc27e902dc01b</x:v>
       </x:c>
       <x:c r="AC192" s="21" t="str">
-        <x:v>À intégrer</x:v>
+        <x:v>En cours</x:v>
       </x:c>
     </x:row>
     <x:row r="193" ht="40" customHeight="1">
@@ -17899,7 +17899,7 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA194" s="23" t="str">
-        <x:v>Accord et publication du lot non consignés.</x:v>
+        <x:v>QA actuelle ; accord et publication non consignés.</x:v>
       </x:c>
       <x:c r="AB194" s="21" t="str">
         <x:v>9184f780a23f21687350020fa3448d58e4e0aadd</x:v>
@@ -17990,7 +17990,7 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA195" s="23" t="str">
-        <x:v>Accord et publication du lot non consignés.</x:v>
+        <x:v>QA actuelle ; accord et publication non consignés.</x:v>
       </x:c>
       <x:c r="AB195" s="21" t="str">
         <x:v>9184f780a23f21687350020fa3448d58e4e0aadd</x:v>
@@ -18374,69 +18374,69 @@
         <x:v>190</x:v>
       </x:c>
       <x:c r="D200" s="24" t="str">
-        <x:v>À planifier</x:v>
+        <x:v>Lot 10</x:v>
       </x:c>
       <x:c r="E200" s="25" t="str">
         <x:v>Personnes</x:v>
       </x:c>
       <x:c r="F200" s="24" t="str">
         <x:f>IF(AND(G200=8,COUNTIF(Q200:V200,"Atlas")=6),"Intégré","À faire")</x:f>
-        <x:v>À faire</x:v>
+        <x:v>Intégré</x:v>
       </x:c>
       <x:c r="G200" s="27" t="n">
         <x:f>COUNTIF(I200:P200,"Présent")</x:f>
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H200" s="24" t="str">
-        <x:v>À assembler</x:v>
+        <x:v>Archivé Drive</x:v>
       </x:c>
       <x:c r="I200" s="24" t="str">
-        <x:v>Référence</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="J200" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="K200" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="L200" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="M200" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="N200" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="O200" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="P200" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="Q200" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="R200" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="S200" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="T200" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="U200" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="V200" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="W200" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="X200" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="Y200" s="24" t="str">
         <x:v>Non consignée</x:v>
@@ -18445,13 +18445,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA200" s="23" t="str">
-        <x:v>Compléter le pack ; consigner QA, accord et publication.</x:v>
+        <x:v>Accord et publication du lot non consignés.</x:v>
       </x:c>
       <x:c r="AB200" s="21" t="str">
-        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
+        <x:v>fc0d47528b092ffae3e49cc020fbc27e902dc01b</x:v>
       </x:c>
       <x:c r="AC200" s="21" t="str">
-        <x:v>À intégrer</x:v>
+        <x:v>En cours</x:v>
       </x:c>
     </x:row>
     <x:row r="201" ht="40" customHeight="1">
@@ -18647,69 +18647,69 @@
         <x:v>193</x:v>
       </x:c>
       <x:c r="D203" s="24" t="str">
-        <x:v>À planifier</x:v>
+        <x:v>Lot 10</x:v>
       </x:c>
       <x:c r="E203" s="25" t="str">
         <x:v>Personnes</x:v>
       </x:c>
       <x:c r="F203" s="24" t="str">
         <x:f>IF(AND(G203=8,COUNTIF(Q203:V203,"Atlas")=6),"Intégré","À faire")</x:f>
-        <x:v>À faire</x:v>
+        <x:v>Intégré</x:v>
       </x:c>
       <x:c r="G203" s="27" t="n">
         <x:f>COUNTIF(I203:P203,"Présent")</x:f>
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H203" s="24" t="str">
-        <x:v>À assembler</x:v>
+        <x:v>Archivé Drive</x:v>
       </x:c>
       <x:c r="I203" s="24" t="str">
-        <x:v>Référence</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="J203" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="K203" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="L203" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="M203" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="N203" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="O203" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="P203" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="Q203" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="R203" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="S203" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="T203" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="U203" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="V203" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="W203" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="X203" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="Y203" s="24" t="str">
         <x:v>Non consignée</x:v>
@@ -18718,13 +18718,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA203" s="23" t="str">
-        <x:v>Compléter le pack ; consigner QA, accord et publication.</x:v>
+        <x:v>Accord et publication du lot non consignés.</x:v>
       </x:c>
       <x:c r="AB203" s="21" t="str">
-        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
+        <x:v>fc0d47528b092ffae3e49cc020fbc27e902dc01b</x:v>
       </x:c>
       <x:c r="AC203" s="21" t="str">
-        <x:v>À intégrer</x:v>
+        <x:v>En cours</x:v>
       </x:c>
     </x:row>
     <x:row r="204" ht="40" customHeight="1">
@@ -19173,7 +19173,7 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA208" s="23" t="str">
-        <x:v>Accord et publication du lot non consignés.</x:v>
+        <x:v>QA actuelle ; accord et publication non consignés.</x:v>
       </x:c>
       <x:c r="AB208" s="21" t="str">
         <x:v>9184f780a23f21687350020fa3448d58e4e0aadd</x:v>
@@ -19284,69 +19284,69 @@
         <x:v>200</x:v>
       </x:c>
       <x:c r="D210" s="24" t="str">
-        <x:v>À planifier</x:v>
+        <x:v>Lot 10</x:v>
       </x:c>
       <x:c r="E210" s="25" t="str">
         <x:v>Personnes</x:v>
       </x:c>
       <x:c r="F210" s="24" t="str">
         <x:f>IF(AND(G210=8,COUNTIF(Q210:V210,"Atlas")=6),"Intégré","À faire")</x:f>
-        <x:v>À faire</x:v>
+        <x:v>Intégré</x:v>
       </x:c>
       <x:c r="G210" s="27" t="n">
         <x:f>COUNTIF(I210:P210,"Présent")</x:f>
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H210" s="24" t="str">
-        <x:v>À assembler</x:v>
+        <x:v>Archivé Drive</x:v>
       </x:c>
       <x:c r="I210" s="24" t="str">
-        <x:v>Référence</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="J210" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="K210" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="L210" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="M210" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="N210" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="O210" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="P210" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="Q210" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="R210" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="S210" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="T210" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="U210" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="V210" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="W210" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="X210" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="Y210" s="24" t="str">
         <x:v>Non consignée</x:v>
@@ -19355,13 +19355,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA210" s="23" t="str">
-        <x:v>Compléter le pack ; consigner QA, accord et publication.</x:v>
+        <x:v>Accord et publication du lot non consignés.</x:v>
       </x:c>
       <x:c r="AB210" s="21" t="str">
-        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
+        <x:v>fc0d47528b092ffae3e49cc020fbc27e902dc01b</x:v>
       </x:c>
       <x:c r="AC210" s="21" t="str">
-        <x:v>À intégrer</x:v>
+        <x:v>En cours</x:v>
       </x:c>
     </x:row>
     <x:row r="211" ht="40" customHeight="1">
@@ -19628,7 +19628,7 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA213" s="23" t="str">
-        <x:v>Accord et publication du lot non consignés.</x:v>
+        <x:v>QA actuelle ; accord et publication non consignés.</x:v>
       </x:c>
       <x:c r="AB213" s="21" t="str">
         <x:v>9184f780a23f21687350020fa3448d58e4e0aadd</x:v>
@@ -19830,69 +19830,69 @@
         <x:v>206</x:v>
       </x:c>
       <x:c r="D216" s="24" t="str">
-        <x:v>À planifier</x:v>
+        <x:v>Lot 10</x:v>
       </x:c>
       <x:c r="E216" s="25" t="str">
         <x:v>Personnes</x:v>
       </x:c>
       <x:c r="F216" s="24" t="str">
         <x:f>IF(AND(G216=8,COUNTIF(Q216:V216,"Atlas")=6),"Intégré","À faire")</x:f>
-        <x:v>À faire</x:v>
+        <x:v>Intégré</x:v>
       </x:c>
       <x:c r="G216" s="27" t="n">
         <x:f>COUNTIF(I216:P216,"Présent")</x:f>
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H216" s="24" t="str">
-        <x:v>À assembler</x:v>
+        <x:v>Archivé Drive</x:v>
       </x:c>
       <x:c r="I216" s="24" t="str">
-        <x:v>Référence</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="J216" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="K216" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="L216" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="M216" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="N216" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="O216" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="P216" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="Q216" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="R216" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="S216" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="T216" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="U216" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="V216" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="W216" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="X216" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="Y216" s="24" t="str">
         <x:v>Non consignée</x:v>
@@ -19901,13 +19901,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA216" s="23" t="str">
-        <x:v>Compléter le pack ; consigner QA, accord et publication.</x:v>
+        <x:v>Accord et publication du lot non consignés.</x:v>
       </x:c>
       <x:c r="AB216" s="21" t="str">
-        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
+        <x:v>fc0d47528b092ffae3e49cc020fbc27e902dc01b</x:v>
       </x:c>
       <x:c r="AC216" s="21" t="str">
-        <x:v>À intégrer</x:v>
+        <x:v>En cours</x:v>
       </x:c>
     </x:row>
     <x:row r="217" ht="40" customHeight="1">
@@ -20285,63 +20285,63 @@
         <x:v>211</x:v>
       </x:c>
       <x:c r="D221" s="24" t="str">
-        <x:v>À planifier</x:v>
+        <x:v>Lot 09</x:v>
       </x:c>
       <x:c r="E221" s="25" t="str">
         <x:v>Nature</x:v>
       </x:c>
       <x:c r="F221" s="24" t="str">
         <x:f>IF(AND(G221=8,COUNTIF(Q221:V221,"Atlas")=6),"Intégré","À faire")</x:f>
-        <x:v>À faire</x:v>
+        <x:v>Intégré</x:v>
       </x:c>
       <x:c r="G221" s="27" t="n">
         <x:f>COUNTIF(I221:P221,"Présent")</x:f>
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H221" s="24" t="str">
-        <x:v>À assembler</x:v>
+        <x:v>Archivé local</x:v>
       </x:c>
       <x:c r="I221" s="24" t="str">
-        <x:v>Référence</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="J221" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="K221" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="L221" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="M221" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="N221" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="O221" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="P221" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="Q221" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="R221" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="S221" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="T221" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="U221" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="V221" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="W221" s="24" t="str">
         <x:v>Non consignée</x:v>
@@ -20356,13 +20356,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA221" s="23" t="str">
-        <x:v>Compléter le pack ; consigner QA, accord et publication.</x:v>
+        <x:v>Requalifier QA ; accord et publication non consignés.</x:v>
       </x:c>
       <x:c r="AB221" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
       </x:c>
       <x:c r="AC221" s="21" t="str">
-        <x:v>À intégrer</x:v>
+        <x:v>En cours</x:v>
       </x:c>
     </x:row>
     <x:row r="222" ht="40" customHeight="1">
@@ -20376,69 +20376,69 @@
         <x:v>212</x:v>
       </x:c>
       <x:c r="D222" s="24" t="str">
-        <x:v>À planifier</x:v>
+        <x:v>Lot 10</x:v>
       </x:c>
       <x:c r="E222" s="25" t="str">
         <x:v>Lieux</x:v>
       </x:c>
       <x:c r="F222" s="24" t="str">
         <x:f>IF(AND(G222=8,COUNTIF(Q222:V222,"Atlas")=6),"Intégré","À faire")</x:f>
-        <x:v>À faire</x:v>
+        <x:v>Intégré</x:v>
       </x:c>
       <x:c r="G222" s="27" t="n">
         <x:f>COUNTIF(I222:P222,"Présent")</x:f>
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H222" s="24" t="str">
-        <x:v>À assembler</x:v>
+        <x:v>Archivé Drive</x:v>
       </x:c>
       <x:c r="I222" s="24" t="str">
-        <x:v>Référence</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="J222" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="K222" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="L222" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="M222" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="N222" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="O222" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="P222" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="Q222" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="R222" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="S222" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="T222" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="U222" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="V222" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="W222" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="X222" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="Y222" s="24" t="str">
         <x:v>Non consignée</x:v>
@@ -20447,13 +20447,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA222" s="23" t="str">
-        <x:v>Compléter le pack ; consigner QA, accord et publication.</x:v>
+        <x:v>Accord et publication du lot non consignés.</x:v>
       </x:c>
       <x:c r="AB222" s="21" t="str">
-        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
+        <x:v>fc0d47528b092ffae3e49cc020fbc27e902dc01b</x:v>
       </x:c>
       <x:c r="AC222" s="21" t="str">
-        <x:v>À intégrer</x:v>
+        <x:v>En cours</x:v>
       </x:c>
     </x:row>
     <x:row r="223" ht="40" customHeight="1">
@@ -20558,69 +20558,69 @@
         <x:v>214</x:v>
       </x:c>
       <x:c r="D224" s="24" t="str">
-        <x:v>À planifier</x:v>
+        <x:v>Lot 10</x:v>
       </x:c>
       <x:c r="E224" s="25" t="str">
         <x:v>Lieux</x:v>
       </x:c>
       <x:c r="F224" s="24" t="str">
         <x:f>IF(AND(G224=8,COUNTIF(Q224:V224,"Atlas")=6),"Intégré","À faire")</x:f>
-        <x:v>À faire</x:v>
+        <x:v>Intégré</x:v>
       </x:c>
       <x:c r="G224" s="27" t="n">
         <x:f>COUNTIF(I224:P224,"Présent")</x:f>
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H224" s="24" t="str">
-        <x:v>À assembler</x:v>
+        <x:v>Archivé Drive</x:v>
       </x:c>
       <x:c r="I224" s="24" t="str">
-        <x:v>Référence</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="J224" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="K224" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="L224" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="M224" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="N224" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="O224" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="P224" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="Q224" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="R224" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="S224" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="T224" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="U224" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="V224" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="W224" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="X224" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="Y224" s="24" t="str">
         <x:v>Non consignée</x:v>
@@ -20629,13 +20629,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA224" s="23" t="str">
-        <x:v>Compléter le pack ; consigner QA, accord et publication.</x:v>
+        <x:v>Accord et publication du lot non consignés.</x:v>
       </x:c>
       <x:c r="AB224" s="21" t="str">
-        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
+        <x:v>fc0d47528b092ffae3e49cc020fbc27e902dc01b</x:v>
       </x:c>
       <x:c r="AC224" s="21" t="str">
-        <x:v>À intégrer</x:v>
+        <x:v>En cours</x:v>
       </x:c>
     </x:row>
     <x:row r="225" ht="40" customHeight="1">
@@ -20649,69 +20649,69 @@
         <x:v>215</x:v>
       </x:c>
       <x:c r="D225" s="24" t="str">
-        <x:v>À planifier</x:v>
+        <x:v>Lot 10</x:v>
       </x:c>
       <x:c r="E225" s="25" t="str">
         <x:v>Lieux</x:v>
       </x:c>
       <x:c r="F225" s="24" t="str">
         <x:f>IF(AND(G225=8,COUNTIF(Q225:V225,"Atlas")=6),"Intégré","À faire")</x:f>
-        <x:v>À faire</x:v>
+        <x:v>Intégré</x:v>
       </x:c>
       <x:c r="G225" s="27" t="n">
         <x:f>COUNTIF(I225:P225,"Présent")</x:f>
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H225" s="24" t="str">
-        <x:v>À assembler</x:v>
+        <x:v>Archivé Drive</x:v>
       </x:c>
       <x:c r="I225" s="24" t="str">
-        <x:v>Référence</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="J225" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="K225" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="L225" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="M225" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="N225" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="O225" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="P225" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="Q225" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="R225" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="S225" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="T225" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="U225" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="V225" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="W225" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="X225" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="Y225" s="24" t="str">
         <x:v>Non consignée</x:v>
@@ -20720,13 +20720,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA225" s="23" t="str">
-        <x:v>Compléter le pack ; consigner QA, accord et publication.</x:v>
+        <x:v>Accord et publication du lot non consignés.</x:v>
       </x:c>
       <x:c r="AB225" s="21" t="str">
-        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
+        <x:v>fc0d47528b092ffae3e49cc020fbc27e902dc01b</x:v>
       </x:c>
       <x:c r="AC225" s="21" t="str">
-        <x:v>À intégrer</x:v>
+        <x:v>En cours</x:v>
       </x:c>
     </x:row>
     <x:row r="226" ht="40" customHeight="1">
@@ -20811,7 +20811,7 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA226" s="23" t="str">
-        <x:v>Accord et publication du lot non consignés.</x:v>
+        <x:v>QA actuelle ; accord et publication non consignés.</x:v>
       </x:c>
       <x:c r="AB226" s="21" t="str">
         <x:v>9184f780a23f21687350020fa3448d58e4e0aadd</x:v>
@@ -21357,7 +21357,7 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA232" s="23" t="str">
-        <x:v>Accord et publication du lot non consignés.</x:v>
+        <x:v>QA actuelle ; accord et publication non consignés.</x:v>
       </x:c>
       <x:c r="AB232" s="21" t="str">
         <x:v>9184f780a23f21687350020fa3448d58e4e0aadd</x:v>
@@ -21721,7 +21721,7 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA236" s="23" t="str">
-        <x:v>Accord et publication du lot non consignés.</x:v>
+        <x:v>QA actuelle ; accord et publication non consignés.</x:v>
       </x:c>
       <x:c r="AB236" s="21" t="str">
         <x:v>9184f780a23f21687350020fa3448d58e4e0aadd</x:v>
@@ -22378,69 +22378,69 @@
         <x:v>234</x:v>
       </x:c>
       <x:c r="D244" s="24" t="str">
-        <x:v>À planifier</x:v>
+        <x:v>Lot 10</x:v>
       </x:c>
       <x:c r="E244" s="25" t="str">
         <x:v>Objets</x:v>
       </x:c>
       <x:c r="F244" s="24" t="str">
         <x:f>IF(AND(G244=8,COUNTIF(Q244:V244,"Atlas")=6),"Intégré","À faire")</x:f>
-        <x:v>À faire</x:v>
+        <x:v>Intégré</x:v>
       </x:c>
       <x:c r="G244" s="27" t="n">
         <x:f>COUNTIF(I244:P244,"Présent")</x:f>
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H244" s="24" t="str">
-        <x:v>À assembler</x:v>
+        <x:v>Archivé Drive</x:v>
       </x:c>
       <x:c r="I244" s="24" t="str">
-        <x:v>Référence</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="J244" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="K244" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="L244" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="M244" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="N244" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="O244" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="P244" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="Q244" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="R244" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="S244" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="T244" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="U244" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="V244" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="W244" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="X244" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="Y244" s="24" t="str">
         <x:v>Non consignée</x:v>
@@ -22449,13 +22449,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA244" s="23" t="str">
-        <x:v>Compléter le pack ; consigner QA, accord et publication.</x:v>
+        <x:v>Accord et publication du lot non consignés.</x:v>
       </x:c>
       <x:c r="AB244" s="21" t="str">
-        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
+        <x:v>fc0d47528b092ffae3e49cc020fbc27e902dc01b</x:v>
       </x:c>
       <x:c r="AC244" s="21" t="str">
-        <x:v>À intégrer</x:v>
+        <x:v>En cours</x:v>
       </x:c>
     </x:row>
     <x:row r="245" ht="40" customHeight="1">
@@ -22469,69 +22469,69 @@
         <x:v>235</x:v>
       </x:c>
       <x:c r="D245" s="24" t="str">
-        <x:v>À planifier</x:v>
+        <x:v>Lot 10</x:v>
       </x:c>
       <x:c r="E245" s="25" t="str">
         <x:v>Objets</x:v>
       </x:c>
       <x:c r="F245" s="24" t="str">
         <x:f>IF(AND(G245=8,COUNTIF(Q245:V245,"Atlas")=6),"Intégré","À faire")</x:f>
-        <x:v>À faire</x:v>
+        <x:v>Intégré</x:v>
       </x:c>
       <x:c r="G245" s="27" t="n">
         <x:f>COUNTIF(I245:P245,"Présent")</x:f>
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H245" s="24" t="str">
-        <x:v>À assembler</x:v>
+        <x:v>Archivé Drive</x:v>
       </x:c>
       <x:c r="I245" s="24" t="str">
-        <x:v>Référence</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="J245" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="K245" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="L245" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="M245" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="N245" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="O245" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="P245" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="Q245" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="R245" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="S245" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="T245" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="U245" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="V245" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="W245" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="X245" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="Y245" s="24" t="str">
         <x:v>Non consignée</x:v>
@@ -22540,13 +22540,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA245" s="23" t="str">
-        <x:v>Compléter le pack ; consigner QA, accord et publication.</x:v>
+        <x:v>Accord et publication du lot non consignés.</x:v>
       </x:c>
       <x:c r="AB245" s="21" t="str">
-        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
+        <x:v>fc0d47528b092ffae3e49cc020fbc27e902dc01b</x:v>
       </x:c>
       <x:c r="AC245" s="21" t="str">
-        <x:v>À intégrer</x:v>
+        <x:v>En cours</x:v>
       </x:c>
     </x:row>
     <x:row r="246" ht="40" customHeight="1">
@@ -23094,7 +23094,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8a28178414e848ea"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0bd4b2fb564e4028"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs(symbols): record 175-pack layout qualification and refresh tracking
</commit_message>
<xml_diff>
--- a/doc_web_interne/docs/suivi-symboles/suivi-240-symboles-6-langues.xlsx
+++ b/doc_web_interne/docs/suivi-symboles/suivi-240-symboles-6-langues.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Suivi symboles" sheetId="1" r:id="Rcc11e5a5ad504ea8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Suivi symboles" sheetId="1" r:id="Reb337a6b48024bfa"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -811,7 +811,7 @@
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="7" t="str">
-        <x:v>Lot 11 en branche : 30 couvertures conservées, 210 nouveaux PNG. Preuves antérieures inchangées conservées.</x:v>
+        <x:v>Lot 11 en branche : 29 couvertures conservées, 203 nouveaux PNG. Preuves antérieures inchangées conservées.</x:v>
       </x:c>
       <x:c r="B3" s="7"/>
       <x:c r="C3" s="7"/>
@@ -848,21 +848,21 @@
       </x:c>
       <x:c r="B4" s="9" t="n">
         <x:f>COUNTIF(F11:F250,"Intégré")</x:f>
-        <x:v>170</x:v>
+        <x:v>175</x:v>
       </x:c>
       <x:c r="C4" s="3" t="str">
         <x:v>Packs à terminer</x:v>
       </x:c>
       <x:c r="D4" s="9" t="n">
         <x:f>COUNTA(B11:B250)-B4</x:f>
-        <x:v>70</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="E4" s="3" t="str">
         <x:v>Pages avec pack</x:v>
       </x:c>
       <x:c r="F4" s="9" t="n">
         <x:f>COUNTIF(Q11:V250,"Atlas")</x:f>
-        <x:v>1020</x:v>
+        <x:v>1050</x:v>
       </x:c>
       <x:c r="G4" s="3" t="str">
         <x:v>Pages web</x:v>
@@ -899,14 +899,14 @@
       </x:c>
       <x:c r="B5" s="9" t="n">
         <x:f>COUNTIF(W11:W250,"6/6 actuelles")</x:f>
-        <x:v>170</x:v>
+        <x:v>175</x:v>
       </x:c>
       <x:c r="C5" s="3" t="str">
         <x:v>QA 2560 px</x:v>
       </x:c>
       <x:c r="D5" s="9" t="n">
         <x:f>COUNTIF(X11:X250,"6/6 actuelles")</x:f>
-        <x:v>170</x:v>
+        <x:v>175</x:v>
       </x:c>
       <x:c r="E5" s="3" t="str">
         <x:v>Accord Thanh</x:v>
@@ -920,7 +920,7 @@
       </x:c>
       <x:c r="H5" s="9" t="n">
         <x:f>COUNTIF(Z11:Z250,"Publié 6/6")</x:f>
-        <x:v>177</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="I5" s="3"/>
       <x:c r="J5" s="3"/>
@@ -980,7 +980,7 @@
     </x:row>
     <x:row r="7" ht="20" customHeight="1">
       <x:c r="A7" s="7" t="str">
-        <x:v>170 packs ; 70 à compléter. Cadre commun : 1 440 pages. Publication antérieure conservée dans les reçus.</x:v>
+        <x:v>175 packs ; 65 à compléter. Cadre commun : 1 440 pages. Publication antérieure conservée dans les reçus.</x:v>
       </x:c>
       <x:c r="B7" s="7"/>
       <x:c r="C7" s="7"/>
@@ -1013,7 +1013,7 @@
     </x:row>
     <x:row r="8" ht="20" customHeight="1">
       <x:c r="A8" s="7" t="str">
-        <x:v>Source : rapport canonique du 20/10/2026, empreinte bc7774d8371f775b. Révision : 622dd61d9ef0f43f5a9090416fe6cf21e4224e20</x:v>
+        <x:v>Source : rapport canonique du 20/10/2026, empreinte 7721867ea6eecebc. Révision : 34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="B8" s="7"/>
       <x:c r="C8" s="7"/>
@@ -1243,13 +1243,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="Z11" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA11" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB11" s="21" t="str">
-        <x:v>1038406132baf06556f6abda8f1620ac4774984b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC11" s="21" t="str">
         <x:v>En cours</x:v>
@@ -1334,13 +1334,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="Z12" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA12" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB12" s="21" t="str">
-        <x:v>1038406132baf06556f6abda8f1620ac4774984b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC12" s="21" t="str">
         <x:v>En cours</x:v>
@@ -1425,13 +1425,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="Z13" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA13" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB13" s="21" t="str">
-        <x:v>1038406132baf06556f6abda8f1620ac4774984b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC13" s="21" t="str">
         <x:v>En cours</x:v>
@@ -1516,13 +1516,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="Z14" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA14" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB14" s="21" t="str">
-        <x:v>1038406132baf06556f6abda8f1620ac4774984b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC14" s="21" t="str">
         <x:v>En cours</x:v>
@@ -1607,13 +1607,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="Z15" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA15" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB15" s="21" t="str">
-        <x:v>1038406132baf06556f6abda8f1620ac4774984b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC15" s="21" t="str">
         <x:v>En cours</x:v>
@@ -1698,13 +1698,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="Z16" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA16" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB16" s="21" t="str">
-        <x:v>1038406132baf06556f6abda8f1620ac4774984b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC16" s="21" t="str">
         <x:v>En cours</x:v>
@@ -1789,13 +1789,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="Z17" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA17" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB17" s="21" t="str">
-        <x:v>1038406132baf06556f6abda8f1620ac4774984b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC17" s="21" t="str">
         <x:v>En cours</x:v>
@@ -1880,13 +1880,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="Z18" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA18" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB18" s="21" t="str">
-        <x:v>1038406132baf06556f6abda8f1620ac4774984b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC18" s="21" t="str">
         <x:v>En cours</x:v>
@@ -1971,13 +1971,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="Z19" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA19" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB19" s="21" t="str">
-        <x:v>1038406132baf06556f6abda8f1620ac4774984b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC19" s="21" t="str">
         <x:v>En cours</x:v>
@@ -2062,13 +2062,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="Z20" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA20" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB20" s="21" t="str">
-        <x:v>1038406132baf06556f6abda8f1620ac4774984b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC20" s="21" t="str">
         <x:v>En cours</x:v>
@@ -2153,13 +2153,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="Z21" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA21" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB21" s="21" t="str">
-        <x:v>1038406132baf06556f6abda8f1620ac4774984b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC21" s="21" t="str">
         <x:v>En cours</x:v>
@@ -2244,13 +2244,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="Z22" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA22" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB22" s="21" t="str">
-        <x:v>1038406132baf06556f6abda8f1620ac4774984b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC22" s="21" t="str">
         <x:v>En cours</x:v>
@@ -2335,13 +2335,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="Z23" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA23" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB23" s="21" t="str">
-        <x:v>1038406132baf06556f6abda8f1620ac4774984b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC23" s="21" t="str">
         <x:v>En cours</x:v>
@@ -2426,13 +2426,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="Z24" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA24" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB24" s="21" t="str">
-        <x:v>1038406132baf06556f6abda8f1620ac4774984b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC24" s="21" t="str">
         <x:v>En cours</x:v>
@@ -2517,13 +2517,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="Z25" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA25" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB25" s="21" t="str">
-        <x:v>1038406132baf06556f6abda8f1620ac4774984b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC25" s="21" t="str">
         <x:v>En cours</x:v>
@@ -2608,13 +2608,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="Z26" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA26" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB26" s="21" t="str">
-        <x:v>1038406132baf06556f6abda8f1620ac4774984b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC26" s="21" t="str">
         <x:v>En cours</x:v>
@@ -2699,13 +2699,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="Z27" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA27" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB27" s="21" t="str">
-        <x:v>1038406132baf06556f6abda8f1620ac4774984b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC27" s="21" t="str">
         <x:v>En cours</x:v>
@@ -2790,13 +2790,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="Z28" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA28" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB28" s="21" t="str">
-        <x:v>1038406132baf06556f6abda8f1620ac4774984b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC28" s="21" t="str">
         <x:v>En cours</x:v>
@@ -2881,13 +2881,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="Z29" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA29" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB29" s="21" t="str">
-        <x:v>1038406132baf06556f6abda8f1620ac4774984b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC29" s="21" t="str">
         <x:v>En cours</x:v>
@@ -2972,13 +2972,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="Z30" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA30" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB30" s="21" t="str">
-        <x:v>1038406132baf06556f6abda8f1620ac4774984b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC30" s="21" t="str">
         <x:v>En cours</x:v>
@@ -3063,13 +3063,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="Z31" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA31" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB31" s="21" t="str">
-        <x:v>1038406132baf06556f6abda8f1620ac4774984b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC31" s="21" t="str">
         <x:v>En cours</x:v>
@@ -3154,13 +3154,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="Z32" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA32" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB32" s="21" t="str">
-        <x:v>1038406132baf06556f6abda8f1620ac4774984b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC32" s="21" t="str">
         <x:v>En cours</x:v>
@@ -3245,13 +3245,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="Z33" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA33" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB33" s="21" t="str">
-        <x:v>1038406132baf06556f6abda8f1620ac4774984b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC33" s="21" t="str">
         <x:v>En cours</x:v>
@@ -3336,13 +3336,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="Z34" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA34" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB34" s="21" t="str">
-        <x:v>1038406132baf06556f6abda8f1620ac4774984b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC34" s="21" t="str">
         <x:v>En cours</x:v>
@@ -3427,10 +3427,10 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z35" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA35" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB35" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -3518,13 +3518,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="Z36" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA36" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB36" s="21" t="str">
-        <x:v>1038406132baf06556f6abda8f1620ac4774984b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC36" s="21" t="str">
         <x:v>En cours</x:v>
@@ -3541,84 +3541,84 @@
         <x:v>27</x:v>
       </x:c>
       <x:c r="D37" s="24" t="str">
-        <x:v>Lot 12 (prévu)</x:v>
+        <x:v>Lot 12 (master)</x:v>
       </x:c>
       <x:c r="E37" s="25" t="str">
         <x:v>Animaux</x:v>
       </x:c>
       <x:c r="F37" s="24" t="str">
         <x:f>IF(AND(G37=8,COUNTIF(Q37:V37,"Atlas")=6),"Intégré","À faire")</x:f>
-        <x:v>À faire</x:v>
+        <x:v>Intégré</x:v>
       </x:c>
       <x:c r="G37" s="27" t="n">
         <x:f>COUNTIF(I37:P37,"Présent")</x:f>
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H37" s="24" t="str">
-        <x:v>À assembler</x:v>
+        <x:v>Réutilisé master #509</x:v>
       </x:c>
       <x:c r="I37" s="24" t="str">
-        <x:v>Référence</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="J37" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="K37" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="L37" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="M37" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="N37" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="O37" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="P37" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="Q37" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="R37" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="S37" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="T37" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="U37" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="V37" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="W37" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="X37" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="Y37" s="24" t="str">
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z37" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA37" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB37" s="21" t="str">
-        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC37" s="21" t="str">
-        <x:v>À intégrer</x:v>
+        <x:v>En cours</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="40" customHeight="1">
@@ -3700,13 +3700,13 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z38" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA38" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB38" s="21" t="str">
-        <x:v>1038406132baf06556f6abda8f1620ac4774984b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC38" s="21" t="str">
         <x:v>En cours</x:v>
@@ -3791,13 +3791,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="Z39" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA39" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB39" s="21" t="str">
-        <x:v>1038406132baf06556f6abda8f1620ac4774984b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC39" s="21" t="str">
         <x:v>En cours</x:v>
@@ -3882,13 +3882,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="Z40" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA40" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB40" s="21" t="str">
-        <x:v>1038406132baf06556f6abda8f1620ac4774984b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC40" s="21" t="str">
         <x:v>En cours</x:v>
@@ -3973,13 +3973,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="Z41" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA41" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB41" s="21" t="str">
-        <x:v>1038406132baf06556f6abda8f1620ac4774984b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC41" s="21" t="str">
         <x:v>En cours</x:v>
@@ -4064,13 +4064,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="Z42" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA42" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB42" s="21" t="str">
-        <x:v>1038406132baf06556f6abda8f1620ac4774984b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC42" s="21" t="str">
         <x:v>En cours</x:v>
@@ -4155,13 +4155,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="Z43" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA43" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB43" s="21" t="str">
-        <x:v>1038406132baf06556f6abda8f1620ac4774984b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC43" s="21" t="str">
         <x:v>En cours</x:v>
@@ -4246,13 +4246,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="Z44" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA44" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB44" s="21" t="str">
-        <x:v>1038406132baf06556f6abda8f1620ac4774984b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC44" s="21" t="str">
         <x:v>En cours</x:v>
@@ -4337,13 +4337,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="Z45" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA45" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB45" s="21" t="str">
-        <x:v>1038406132baf06556f6abda8f1620ac4774984b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC45" s="21" t="str">
         <x:v>En cours</x:v>
@@ -4428,13 +4428,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="Z46" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA46" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB46" s="21" t="str">
-        <x:v>1038406132baf06556f6abda8f1620ac4774984b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC46" s="21" t="str">
         <x:v>En cours</x:v>
@@ -4519,13 +4519,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="Z47" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA47" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB47" s="21" t="str">
-        <x:v>1038406132baf06556f6abda8f1620ac4774984b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC47" s="21" t="str">
         <x:v>En cours</x:v>
@@ -4610,13 +4610,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="Z48" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA48" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB48" s="21" t="str">
-        <x:v>1038406132baf06556f6abda8f1620ac4774984b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC48" s="21" t="str">
         <x:v>En cours</x:v>
@@ -4701,13 +4701,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="Z49" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA49" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB49" s="21" t="str">
-        <x:v>1038406132baf06556f6abda8f1620ac4774984b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC49" s="21" t="str">
         <x:v>En cours</x:v>
@@ -4792,13 +4792,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="Z50" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA50" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB50" s="21" t="str">
-        <x:v>1038406132baf06556f6abda8f1620ac4774984b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC50" s="21" t="str">
         <x:v>En cours</x:v>
@@ -4883,13 +4883,13 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z51" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA51" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB51" s="21" t="str">
-        <x:v>1038406132baf06556f6abda8f1620ac4774984b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC51" s="21" t="str">
         <x:v>En cours</x:v>
@@ -4974,13 +4974,13 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z52" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA52" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB52" s="21" t="str">
-        <x:v>1038406132baf06556f6abda8f1620ac4774984b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC52" s="21" t="str">
         <x:v>En cours</x:v>
@@ -5065,13 +5065,13 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z53" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA53" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB53" s="21" t="str">
-        <x:v>1038406132baf06556f6abda8f1620ac4774984b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC53" s="21" t="str">
         <x:v>En cours</x:v>
@@ -5156,13 +5156,13 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z54" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA54" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB54" s="21" t="str">
-        <x:v>1038406132baf06556f6abda8f1620ac4774984b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC54" s="21" t="str">
         <x:v>En cours</x:v>
@@ -5247,13 +5247,13 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z55" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA55" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB55" s="21" t="str">
-        <x:v>1038406132baf06556f6abda8f1620ac4774984b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC55" s="21" t="str">
         <x:v>En cours</x:v>
@@ -5338,13 +5338,13 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z56" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA56" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB56" s="21" t="str">
-        <x:v>1038406132baf06556f6abda8f1620ac4774984b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC56" s="21" t="str">
         <x:v>En cours</x:v>
@@ -5429,13 +5429,13 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z57" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA57" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB57" s="21" t="str">
-        <x:v>1038406132baf06556f6abda8f1620ac4774984b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC57" s="21" t="str">
         <x:v>En cours</x:v>
@@ -5520,13 +5520,13 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z58" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA58" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB58" s="21" t="str">
-        <x:v>1038406132baf06556f6abda8f1620ac4774984b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC58" s="21" t="str">
         <x:v>En cours</x:v>
@@ -5611,13 +5611,13 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z59" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA59" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB59" s="21" t="str">
-        <x:v>1038406132baf06556f6abda8f1620ac4774984b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC59" s="21" t="str">
         <x:v>En cours</x:v>
@@ -5702,13 +5702,13 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z60" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA60" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB60" s="21" t="str">
-        <x:v>1038406132baf06556f6abda8f1620ac4774984b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC60" s="21" t="str">
         <x:v>En cours</x:v>
@@ -5793,13 +5793,13 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z61" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA61" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB61" s="21" t="str">
-        <x:v>1038406132baf06556f6abda8f1620ac4774984b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC61" s="21" t="str">
         <x:v>En cours</x:v>
@@ -5884,13 +5884,13 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z62" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA62" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB62" s="21" t="str">
-        <x:v>1038406132baf06556f6abda8f1620ac4774984b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC62" s="21" t="str">
         <x:v>En cours</x:v>
@@ -5975,13 +5975,13 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z63" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA63" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB63" s="21" t="str">
-        <x:v>1038406132baf06556f6abda8f1620ac4774984b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC63" s="21" t="str">
         <x:v>En cours</x:v>
@@ -6066,13 +6066,13 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z64" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA64" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB64" s="21" t="str">
-        <x:v>1038406132baf06556f6abda8f1620ac4774984b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC64" s="21" t="str">
         <x:v>En cours</x:v>
@@ -6157,13 +6157,13 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z65" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA65" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB65" s="21" t="str">
-        <x:v>1038406132baf06556f6abda8f1620ac4774984b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC65" s="21" t="str">
         <x:v>En cours</x:v>
@@ -6248,13 +6248,13 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z66" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA66" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB66" s="21" t="str">
-        <x:v>1038406132baf06556f6abda8f1620ac4774984b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC66" s="21" t="str">
         <x:v>En cours</x:v>
@@ -6339,13 +6339,13 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z67" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA67" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB67" s="21" t="str">
-        <x:v>1038406132baf06556f6abda8f1620ac4774984b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC67" s="21" t="str">
         <x:v>En cours</x:v>
@@ -6430,13 +6430,13 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z68" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA68" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB68" s="21" t="str">
-        <x:v>1038406132baf06556f6abda8f1620ac4774984b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC68" s="21" t="str">
         <x:v>En cours</x:v>
@@ -6521,13 +6521,13 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z69" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA69" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB69" s="21" t="str">
-        <x:v>1038406132baf06556f6abda8f1620ac4774984b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC69" s="21" t="str">
         <x:v>En cours</x:v>
@@ -6612,13 +6612,13 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z70" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA70" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB70" s="21" t="str">
-        <x:v>1038406132baf06556f6abda8f1620ac4774984b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC70" s="21" t="str">
         <x:v>En cours</x:v>
@@ -6703,13 +6703,13 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z71" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA71" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB71" s="21" t="str">
-        <x:v>1038406132baf06556f6abda8f1620ac4774984b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC71" s="21" t="str">
         <x:v>En cours</x:v>
@@ -6794,13 +6794,13 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z72" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA72" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB72" s="21" t="str">
-        <x:v>1038406132baf06556f6abda8f1620ac4774984b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC72" s="21" t="str">
         <x:v>En cours</x:v>
@@ -6885,13 +6885,13 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z73" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA73" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB73" s="21" t="str">
-        <x:v>1038406132baf06556f6abda8f1620ac4774984b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC73" s="21" t="str">
         <x:v>En cours</x:v>
@@ -6976,13 +6976,13 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z74" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA74" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB74" s="21" t="str">
-        <x:v>1038406132baf06556f6abda8f1620ac4774984b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC74" s="21" t="str">
         <x:v>En cours</x:v>
@@ -7067,13 +7067,13 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z75" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA75" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB75" s="21" t="str">
-        <x:v>1038406132baf06556f6abda8f1620ac4774984b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC75" s="21" t="str">
         <x:v>En cours</x:v>
@@ -7158,13 +7158,13 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z76" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA76" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB76" s="21" t="str">
-        <x:v>1038406132baf06556f6abda8f1620ac4774984b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC76" s="21" t="str">
         <x:v>En cours</x:v>
@@ -7249,13 +7249,13 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z77" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA77" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB77" s="21" t="str">
-        <x:v>1038406132baf06556f6abda8f1620ac4774984b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC77" s="21" t="str">
         <x:v>En cours</x:v>
@@ -7340,13 +7340,13 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z78" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA78" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB78" s="21" t="str">
-        <x:v>1038406132baf06556f6abda8f1620ac4774984b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC78" s="21" t="str">
         <x:v>En cours</x:v>
@@ -7431,13 +7431,13 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z79" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA79" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB79" s="21" t="str">
-        <x:v>1038406132baf06556f6abda8f1620ac4774984b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC79" s="21" t="str">
         <x:v>En cours</x:v>
@@ -7522,13 +7522,13 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z80" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA80" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB80" s="21" t="str">
-        <x:v>1038406132baf06556f6abda8f1620ac4774984b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC80" s="21" t="str">
         <x:v>En cours</x:v>
@@ -7613,13 +7613,13 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z81" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA81" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB81" s="21" t="str">
-        <x:v>1038406132baf06556f6abda8f1620ac4774984b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC81" s="21" t="str">
         <x:v>En cours</x:v>
@@ -7704,13 +7704,13 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z82" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA82" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB82" s="21" t="str">
-        <x:v>1038406132baf06556f6abda8f1620ac4774984b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC82" s="21" t="str">
         <x:v>En cours</x:v>
@@ -7795,13 +7795,13 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z83" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA83" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB83" s="21" t="str">
-        <x:v>1038406132baf06556f6abda8f1620ac4774984b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC83" s="21" t="str">
         <x:v>En cours</x:v>
@@ -7886,13 +7886,13 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z84" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA84" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB84" s="21" t="str">
-        <x:v>1038406132baf06556f6abda8f1620ac4774984b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC84" s="21" t="str">
         <x:v>En cours</x:v>
@@ -7977,13 +7977,13 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z85" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA85" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB85" s="21" t="str">
-        <x:v>1038406132baf06556f6abda8f1620ac4774984b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC85" s="21" t="str">
         <x:v>En cours</x:v>
@@ -8068,13 +8068,13 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z86" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA86" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB86" s="21" t="str">
-        <x:v>1038406132baf06556f6abda8f1620ac4774984b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC86" s="21" t="str">
         <x:v>En cours</x:v>
@@ -8159,13 +8159,13 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z87" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA87" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB87" s="21" t="str">
-        <x:v>1038406132baf06556f6abda8f1620ac4774984b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC87" s="21" t="str">
         <x:v>En cours</x:v>
@@ -8250,13 +8250,13 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z88" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA88" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB88" s="21" t="str">
-        <x:v>1038406132baf06556f6abda8f1620ac4774984b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC88" s="21" t="str">
         <x:v>En cours</x:v>
@@ -8347,7 +8347,7 @@
         <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB89" s="21" t="str">
-        <x:v>fc0d47528b092ffae3e49cc020fbc27e902dc01b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC89" s="21" t="str">
         <x:v>En cours</x:v>
@@ -8364,84 +8364,84 @@
         <x:v>80</x:v>
       </x:c>
       <x:c r="D90" s="24" t="str">
-        <x:v>Lot 12 (prévu)</x:v>
+        <x:v>Lot 12 (master)</x:v>
       </x:c>
       <x:c r="E90" s="25" t="str">
         <x:v>Animaux</x:v>
       </x:c>
       <x:c r="F90" s="24" t="str">
         <x:f>IF(AND(G90=8,COUNTIF(Q90:V90,"Atlas")=6),"Intégré","À faire")</x:f>
-        <x:v>À faire</x:v>
+        <x:v>Intégré</x:v>
       </x:c>
       <x:c r="G90" s="27" t="n">
         <x:f>COUNTIF(I90:P90,"Présent")</x:f>
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H90" s="24" t="str">
-        <x:v>À assembler</x:v>
+        <x:v>Réutilisé master #509</x:v>
       </x:c>
       <x:c r="I90" s="24" t="str">
-        <x:v>Référence</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="J90" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="K90" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="L90" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="M90" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="N90" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="O90" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="P90" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="Q90" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="R90" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="S90" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="T90" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="U90" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="V90" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="W90" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="X90" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="Y90" s="24" t="str">
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z90" s="24" t="str">
-        <x:v>Périmée (5/6)</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA90" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB90" s="21" t="str">
-        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC90" s="21" t="str">
-        <x:v>À intégrer</x:v>
+        <x:v>En cours</x:v>
       </x:c>
     </x:row>
     <x:row r="91" ht="40" customHeight="1">
@@ -8529,7 +8529,7 @@
         <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB91" s="21" t="str">
-        <x:v>fc0d47528b092ffae3e49cc020fbc27e902dc01b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC91" s="21" t="str">
         <x:v>En cours</x:v>
@@ -8620,7 +8620,7 @@
         <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB92" s="21" t="str">
-        <x:v>fc0d47528b092ffae3e49cc020fbc27e902dc01b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC92" s="21" t="str">
         <x:v>En cours</x:v>
@@ -8705,10 +8705,10 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z93" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA93" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB93" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -8802,7 +8802,7 @@
         <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB94" s="21" t="str">
-        <x:v>fc0d47528b092ffae3e49cc020fbc27e902dc01b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC94" s="21" t="str">
         <x:v>En cours</x:v>
@@ -8893,7 +8893,7 @@
         <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB95" s="21" t="str">
-        <x:v>fc0d47528b092ffae3e49cc020fbc27e902dc01b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC95" s="21" t="str">
         <x:v>En cours</x:v>
@@ -8984,7 +8984,7 @@
         <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB96" s="21" t="str">
-        <x:v>fc0d47528b092ffae3e49cc020fbc27e902dc01b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC96" s="21" t="str">
         <x:v>En cours</x:v>
@@ -9069,13 +9069,13 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z97" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA97" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB97" s="21" t="str">
-        <x:v>1038406132baf06556f6abda8f1620ac4774984b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC97" s="21" t="str">
         <x:v>En cours</x:v>
@@ -9160,13 +9160,13 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z98" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA98" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB98" s="21" t="str">
-        <x:v>1038406132baf06556f6abda8f1620ac4774984b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC98" s="21" t="str">
         <x:v>En cours</x:v>
@@ -9251,13 +9251,13 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z99" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA99" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB99" s="21" t="str">
-        <x:v>1038406132baf06556f6abda8f1620ac4774984b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC99" s="21" t="str">
         <x:v>En cours</x:v>
@@ -9342,13 +9342,13 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z100" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA100" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB100" s="21" t="str">
-        <x:v>1038406132baf06556f6abda8f1620ac4774984b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC100" s="21" t="str">
         <x:v>En cours</x:v>
@@ -9433,10 +9433,10 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z101" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA101" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB101" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -9524,13 +9524,13 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z102" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA102" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB102" s="21" t="str">
-        <x:v>1038406132baf06556f6abda8f1620ac4774984b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC102" s="21" t="str">
         <x:v>En cours</x:v>
@@ -9547,7 +9547,7 @@
         <x:v>93</x:v>
       </x:c>
       <x:c r="D103" s="24" t="str">
-        <x:v>Lot 11</x:v>
+        <x:v>Lot 11 (master)</x:v>
       </x:c>
       <x:c r="E103" s="25" t="str">
         <x:v>Objets</x:v>
@@ -9561,7 +9561,7 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="H103" s="24" t="str">
-        <x:v>Archivé Drive</x:v>
+        <x:v>Réutilisé master #509</x:v>
       </x:c>
       <x:c r="I103" s="24" t="str">
         <x:v>Présent</x:v>
@@ -9621,7 +9621,7 @@
         <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB103" s="21" t="str">
-        <x:v>622dd61d9ef0f43f5a9090416fe6cf21e4224e20</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC103" s="21" t="str">
         <x:v>En cours</x:v>
@@ -9706,13 +9706,13 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z104" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA104" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB104" s="21" t="str">
-        <x:v>1038406132baf06556f6abda8f1620ac4774984b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC104" s="21" t="str">
         <x:v>En cours</x:v>
@@ -9797,13 +9797,13 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z105" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA105" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB105" s="21" t="str">
-        <x:v>1038406132baf06556f6abda8f1620ac4774984b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC105" s="21" t="str">
         <x:v>En cours</x:v>
@@ -9888,13 +9888,13 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z106" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA106" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB106" s="21" t="str">
-        <x:v>1038406132baf06556f6abda8f1620ac4774984b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC106" s="21" t="str">
         <x:v>En cours</x:v>
@@ -9985,7 +9985,7 @@
         <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB107" s="21" t="str">
-        <x:v>fc0d47528b092ffae3e49cc020fbc27e902dc01b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC107" s="21" t="str">
         <x:v>En cours</x:v>
@@ -10070,10 +10070,10 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z108" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA108" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB108" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -10161,10 +10161,10 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z109" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA109" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB109" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -10184,84 +10184,84 @@
         <x:v>100</x:v>
       </x:c>
       <x:c r="D110" s="24" t="str">
-        <x:v>Lot 12 (prévu)</x:v>
+        <x:v>Lot 12 (master)</x:v>
       </x:c>
       <x:c r="E110" s="25" t="str">
         <x:v>Nature</x:v>
       </x:c>
       <x:c r="F110" s="24" t="str">
         <x:f>IF(AND(G110=8,COUNTIF(Q110:V110,"Atlas")=6),"Intégré","À faire")</x:f>
-        <x:v>À faire</x:v>
+        <x:v>Intégré</x:v>
       </x:c>
       <x:c r="G110" s="27" t="n">
         <x:f>COUNTIF(I110:P110,"Présent")</x:f>
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H110" s="24" t="str">
-        <x:v>À assembler</x:v>
+        <x:v>Réutilisé master #509</x:v>
       </x:c>
       <x:c r="I110" s="24" t="str">
-        <x:v>Référence</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="J110" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="K110" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="L110" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="M110" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="N110" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="O110" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="P110" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="Q110" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="R110" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="S110" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="T110" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="U110" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="V110" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="W110" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="X110" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="Y110" s="24" t="str">
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z110" s="24" t="str">
-        <x:v>Périmée (5/6)</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA110" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB110" s="21" t="str">
-        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC110" s="21" t="str">
-        <x:v>À intégrer</x:v>
+        <x:v>En cours</x:v>
       </x:c>
     </x:row>
     <x:row r="111" ht="40" customHeight="1">
@@ -10343,10 +10343,10 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z111" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA111" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB111" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -10434,10 +10434,10 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z112" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA112" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB112" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -10525,10 +10525,10 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z113" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA113" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB113" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -10616,10 +10616,10 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z114" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA114" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB114" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -10713,7 +10713,7 @@
         <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB115" s="21" t="str">
-        <x:v>fc0d47528b092ffae3e49cc020fbc27e902dc01b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC115" s="21" t="str">
         <x:v>En cours</x:v>
@@ -10798,10 +10798,10 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z116" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA116" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB116" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -10889,10 +10889,10 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z117" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA117" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB117" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -10980,13 +10980,13 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z118" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA118" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB118" s="21" t="str">
-        <x:v>1038406132baf06556f6abda8f1620ac4774984b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC118" s="21" t="str">
         <x:v>En cours</x:v>
@@ -11077,7 +11077,7 @@
         <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB119" s="21" t="str">
-        <x:v>622dd61d9ef0f43f5a9090416fe6cf21e4224e20</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC119" s="21" t="str">
         <x:v>En cours</x:v>
@@ -11168,7 +11168,7 @@
         <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB120" s="21" t="str">
-        <x:v>622dd61d9ef0f43f5a9090416fe6cf21e4224e20</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC120" s="21" t="str">
         <x:v>En cours</x:v>
@@ -11253,10 +11253,10 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z121" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA121" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB121" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -11344,10 +11344,10 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z122" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA122" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB122" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -11435,10 +11435,10 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z123" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA123" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB123" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -11526,10 +11526,10 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z124" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA124" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB124" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -11623,7 +11623,7 @@
         <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB125" s="21" t="str">
-        <x:v>622dd61d9ef0f43f5a9090416fe6cf21e4224e20</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC125" s="21" t="str">
         <x:v>En cours</x:v>
@@ -11714,7 +11714,7 @@
         <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB126" s="21" t="str">
-        <x:v>fc0d47528b092ffae3e49cc020fbc27e902dc01b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC126" s="21" t="str">
         <x:v>En cours</x:v>
@@ -11799,10 +11799,10 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z127" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA127" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB127" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -11890,13 +11890,13 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z128" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA128" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB128" s="21" t="str">
-        <x:v>1038406132baf06556f6abda8f1620ac4774984b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC128" s="21" t="str">
         <x:v>En cours</x:v>
@@ -11981,10 +11981,10 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z129" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA129" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB129" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -12078,7 +12078,7 @@
         <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB130" s="21" t="str">
-        <x:v>622dd61d9ef0f43f5a9090416fe6cf21e4224e20</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC130" s="21" t="str">
         <x:v>En cours</x:v>
@@ -12163,10 +12163,10 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z131" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA131" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB131" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -12254,10 +12254,10 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z132" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA132" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB132" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -12351,7 +12351,7 @@
         <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB133" s="21" t="str">
-        <x:v>fc0d47528b092ffae3e49cc020fbc27e902dc01b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC133" s="21" t="str">
         <x:v>En cours</x:v>
@@ -12436,10 +12436,10 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z134" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA134" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB134" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -12527,13 +12527,13 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z135" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA135" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB135" s="21" t="str">
-        <x:v>1038406132baf06556f6abda8f1620ac4774984b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC135" s="21" t="str">
         <x:v>En cours</x:v>
@@ -12618,10 +12618,10 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z136" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA136" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB136" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -12715,7 +12715,7 @@
         <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB137" s="21" t="str">
-        <x:v>622dd61d9ef0f43f5a9090416fe6cf21e4224e20</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC137" s="21" t="str">
         <x:v>En cours</x:v>
@@ -12800,10 +12800,10 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z138" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA138" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB138" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -12897,7 +12897,7 @@
         <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB139" s="21" t="str">
-        <x:v>fc0d47528b092ffae3e49cc020fbc27e902dc01b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC139" s="21" t="str">
         <x:v>En cours</x:v>
@@ -12982,13 +12982,13 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z140" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA140" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB140" s="21" t="str">
-        <x:v>1038406132baf06556f6abda8f1620ac4774984b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC140" s="21" t="str">
         <x:v>En cours</x:v>
@@ -13073,13 +13073,13 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z141" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA141" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB141" s="21" t="str">
-        <x:v>1038406132baf06556f6abda8f1620ac4774984b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC141" s="21" t="str">
         <x:v>En cours</x:v>
@@ -13164,10 +13164,10 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z142" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA142" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB142" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -13255,10 +13255,10 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z143" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA143" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB143" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -13346,10 +13346,10 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z144" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA144" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB144" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -13437,13 +13437,13 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z145" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA145" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB145" s="21" t="str">
-        <x:v>1038406132baf06556f6abda8f1620ac4774984b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC145" s="21" t="str">
         <x:v>En cours</x:v>
@@ -13528,10 +13528,10 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z146" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA146" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB146" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -13625,7 +13625,7 @@
         <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB147" s="21" t="str">
-        <x:v>fc0d47528b092ffae3e49cc020fbc27e902dc01b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC147" s="21" t="str">
         <x:v>En cours</x:v>
@@ -13710,10 +13710,10 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z148" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA148" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB148" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -13807,7 +13807,7 @@
         <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB149" s="21" t="str">
-        <x:v>622dd61d9ef0f43f5a9090416fe6cf21e4224e20</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC149" s="21" t="str">
         <x:v>En cours</x:v>
@@ -13892,13 +13892,13 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z150" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA150" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB150" s="21" t="str">
-        <x:v>1038406132baf06556f6abda8f1620ac4774984b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC150" s="21" t="str">
         <x:v>En cours</x:v>
@@ -13983,13 +13983,13 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z151" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA151" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB151" s="21" t="str">
-        <x:v>1038406132baf06556f6abda8f1620ac4774984b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC151" s="21" t="str">
         <x:v>En cours</x:v>
@@ -14074,13 +14074,13 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z152" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA152" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB152" s="21" t="str">
-        <x:v>1038406132baf06556f6abda8f1620ac4774984b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC152" s="21" t="str">
         <x:v>En cours</x:v>
@@ -14165,10 +14165,10 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z153" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA153" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB153" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -14256,13 +14256,13 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z154" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA154" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB154" s="21" t="str">
-        <x:v>1038406132baf06556f6abda8f1620ac4774984b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC154" s="21" t="str">
         <x:v>En cours</x:v>
@@ -14353,7 +14353,7 @@
         <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB155" s="21" t="str">
-        <x:v>622dd61d9ef0f43f5a9090416fe6cf21e4224e20</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC155" s="21" t="str">
         <x:v>En cours</x:v>
@@ -14438,10 +14438,10 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z156" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA156" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB156" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -14535,7 +14535,7 @@
         <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB157" s="21" t="str">
-        <x:v>fc0d47528b092ffae3e49cc020fbc27e902dc01b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC157" s="21" t="str">
         <x:v>En cours</x:v>
@@ -14626,7 +14626,7 @@
         <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB158" s="21" t="str">
-        <x:v>fc0d47528b092ffae3e49cc020fbc27e902dc01b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC158" s="21" t="str">
         <x:v>En cours</x:v>
@@ -14717,7 +14717,7 @@
         <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB159" s="21" t="str">
-        <x:v>fc0d47528b092ffae3e49cc020fbc27e902dc01b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC159" s="21" t="str">
         <x:v>En cours</x:v>
@@ -14808,7 +14808,7 @@
         <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB160" s="21" t="str">
-        <x:v>622dd61d9ef0f43f5a9090416fe6cf21e4224e20</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC160" s="21" t="str">
         <x:v>En cours</x:v>
@@ -14893,10 +14893,10 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z161" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA161" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB161" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -14984,13 +14984,13 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z162" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA162" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB162" s="21" t="str">
-        <x:v>1038406132baf06556f6abda8f1620ac4774984b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC162" s="21" t="str">
         <x:v>En cours</x:v>
@@ -15075,13 +15075,13 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z163" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA163" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB163" s="21" t="str">
-        <x:v>1038406132baf06556f6abda8f1620ac4774984b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC163" s="21" t="str">
         <x:v>En cours</x:v>
@@ -15166,10 +15166,10 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z164" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA164" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB164" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -15257,10 +15257,10 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z165" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA165" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB165" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -15348,13 +15348,13 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z166" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA166" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB166" s="21" t="str">
-        <x:v>1038406132baf06556f6abda8f1620ac4774984b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC166" s="21" t="str">
         <x:v>En cours</x:v>
@@ -15439,13 +15439,13 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z167" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA167" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB167" s="21" t="str">
-        <x:v>1038406132baf06556f6abda8f1620ac4774984b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC167" s="21" t="str">
         <x:v>En cours</x:v>
@@ -15530,10 +15530,10 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z168" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA168" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB168" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -15621,10 +15621,10 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z169" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA169" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB169" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -15718,7 +15718,7 @@
         <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB170" s="21" t="str">
-        <x:v>622dd61d9ef0f43f5a9090416fe6cf21e4224e20</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC170" s="21" t="str">
         <x:v>En cours</x:v>
@@ -15809,7 +15809,7 @@
         <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB171" s="21" t="str">
-        <x:v>fc0d47528b092ffae3e49cc020fbc27e902dc01b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC171" s="21" t="str">
         <x:v>En cours</x:v>
@@ -15894,10 +15894,10 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z172" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA172" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB172" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -15985,13 +15985,13 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z173" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA173" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB173" s="21" t="str">
-        <x:v>1038406132baf06556f6abda8f1620ac4774984b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC173" s="21" t="str">
         <x:v>En cours</x:v>
@@ -16076,10 +16076,10 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z174" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA174" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB174" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -16167,10 +16167,10 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z175" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA175" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB175" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -16258,10 +16258,10 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z176" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA176" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB176" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -16355,7 +16355,7 @@
         <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB177" s="21" t="str">
-        <x:v>622dd61d9ef0f43f5a9090416fe6cf21e4224e20</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC177" s="21" t="str">
         <x:v>En cours</x:v>
@@ -16440,10 +16440,10 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z178" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA178" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB178" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -16537,7 +16537,7 @@
         <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB179" s="21" t="str">
-        <x:v>fc0d47528b092ffae3e49cc020fbc27e902dc01b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC179" s="21" t="str">
         <x:v>En cours</x:v>
@@ -16622,13 +16622,13 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z180" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA180" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB180" s="21" t="str">
-        <x:v>1038406132baf06556f6abda8f1620ac4774984b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC180" s="21" t="str">
         <x:v>En cours</x:v>
@@ -16719,7 +16719,7 @@
         <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB181" s="21" t="str">
-        <x:v>622dd61d9ef0f43f5a9090416fe6cf21e4224e20</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC181" s="21" t="str">
         <x:v>En cours</x:v>
@@ -16810,7 +16810,7 @@
         <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB182" s="21" t="str">
-        <x:v>622dd61d9ef0f43f5a9090416fe6cf21e4224e20</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC182" s="21" t="str">
         <x:v>En cours</x:v>
@@ -16895,10 +16895,10 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z183" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA183" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB183" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -16986,13 +16986,13 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z184" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA184" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB184" s="21" t="str">
-        <x:v>1038406132baf06556f6abda8f1620ac4774984b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC184" s="21" t="str">
         <x:v>En cours</x:v>
@@ -17009,84 +17009,84 @@
         <x:v>175</x:v>
       </x:c>
       <x:c r="D185" s="24" t="str">
-        <x:v>Lot 12 (prévu)</x:v>
+        <x:v>Lot 12 (master)</x:v>
       </x:c>
       <x:c r="E185" s="25" t="str">
         <x:v>Objets</x:v>
       </x:c>
       <x:c r="F185" s="24" t="str">
         <x:f>IF(AND(G185=8,COUNTIF(Q185:V185,"Atlas")=6),"Intégré","À faire")</x:f>
-        <x:v>À faire</x:v>
+        <x:v>Intégré</x:v>
       </x:c>
       <x:c r="G185" s="27" t="n">
         <x:f>COUNTIF(I185:P185,"Présent")</x:f>
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H185" s="24" t="str">
-        <x:v>À assembler</x:v>
+        <x:v>Réutilisé master #509</x:v>
       </x:c>
       <x:c r="I185" s="24" t="str">
-        <x:v>Référence</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="J185" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="K185" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="L185" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="M185" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="N185" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="O185" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="P185" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="Q185" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="R185" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="S185" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="T185" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="U185" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="V185" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="W185" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="X185" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="Y185" s="24" t="str">
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z185" s="24" t="str">
-        <x:v>Périmée (5/6)</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA185" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB185" s="21" t="str">
-        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC185" s="21" t="str">
-        <x:v>À intégrer</x:v>
+        <x:v>En cours</x:v>
       </x:c>
     </x:row>
     <x:row r="186" ht="40" customHeight="1">
@@ -17174,7 +17174,7 @@
         <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB186" s="21" t="str">
-        <x:v>fc0d47528b092ffae3e49cc020fbc27e902dc01b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC186" s="21" t="str">
         <x:v>En cours</x:v>
@@ -17265,7 +17265,7 @@
         <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB187" s="21" t="str">
-        <x:v>fc0d47528b092ffae3e49cc020fbc27e902dc01b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC187" s="21" t="str">
         <x:v>En cours</x:v>
@@ -17356,7 +17356,7 @@
         <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB188" s="21" t="str">
-        <x:v>622dd61d9ef0f43f5a9090416fe6cf21e4224e20</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC188" s="21" t="str">
         <x:v>En cours</x:v>
@@ -17447,7 +17447,7 @@
         <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB189" s="21" t="str">
-        <x:v>622dd61d9ef0f43f5a9090416fe6cf21e4224e20</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC189" s="21" t="str">
         <x:v>En cours</x:v>
@@ -17532,13 +17532,13 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z190" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA190" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB190" s="21" t="str">
-        <x:v>1038406132baf06556f6abda8f1620ac4774984b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC190" s="21" t="str">
         <x:v>En cours</x:v>
@@ -17623,13 +17623,13 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z191" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA191" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB191" s="21" t="str">
-        <x:v>1038406132baf06556f6abda8f1620ac4774984b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC191" s="21" t="str">
         <x:v>En cours</x:v>
@@ -17720,7 +17720,7 @@
         <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB192" s="21" t="str">
-        <x:v>fc0d47528b092ffae3e49cc020fbc27e902dc01b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC192" s="21" t="str">
         <x:v>En cours</x:v>
@@ -17811,7 +17811,7 @@
         <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB193" s="21" t="str">
-        <x:v>622dd61d9ef0f43f5a9090416fe6cf21e4224e20</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC193" s="21" t="str">
         <x:v>En cours</x:v>
@@ -17896,13 +17896,13 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z194" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA194" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB194" s="21" t="str">
-        <x:v>1038406132baf06556f6abda8f1620ac4774984b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC194" s="21" t="str">
         <x:v>En cours</x:v>
@@ -17987,13 +17987,13 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z195" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA195" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB195" s="21" t="str">
-        <x:v>1038406132baf06556f6abda8f1620ac4774984b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC195" s="21" t="str">
         <x:v>En cours</x:v>
@@ -18084,7 +18084,7 @@
         <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB196" s="21" t="str">
-        <x:v>622dd61d9ef0f43f5a9090416fe6cf21e4224e20</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC196" s="21" t="str">
         <x:v>En cours</x:v>
@@ -18169,10 +18169,10 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z197" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA197" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB197" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -18260,10 +18260,10 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z198" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA198" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB198" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -18357,7 +18357,7 @@
         <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB199" s="21" t="str">
-        <x:v>622dd61d9ef0f43f5a9090416fe6cf21e4224e20</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC199" s="21" t="str">
         <x:v>En cours</x:v>
@@ -18448,7 +18448,7 @@
         <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB200" s="21" t="str">
-        <x:v>fc0d47528b092ffae3e49cc020fbc27e902dc01b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC200" s="21" t="str">
         <x:v>En cours</x:v>
@@ -18539,7 +18539,7 @@
         <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB201" s="21" t="str">
-        <x:v>622dd61d9ef0f43f5a9090416fe6cf21e4224e20</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC201" s="21" t="str">
         <x:v>En cours</x:v>
@@ -18624,10 +18624,10 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z202" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA202" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB202" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -18721,7 +18721,7 @@
         <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB203" s="21" t="str">
-        <x:v>fc0d47528b092ffae3e49cc020fbc27e902dc01b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC203" s="21" t="str">
         <x:v>En cours</x:v>
@@ -18812,7 +18812,7 @@
         <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB204" s="21" t="str">
-        <x:v>622dd61d9ef0f43f5a9090416fe6cf21e4224e20</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC204" s="21" t="str">
         <x:v>En cours</x:v>
@@ -18903,7 +18903,7 @@
         <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB205" s="21" t="str">
-        <x:v>622dd61d9ef0f43f5a9090416fe6cf21e4224e20</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC205" s="21" t="str">
         <x:v>En cours</x:v>
@@ -18988,10 +18988,10 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z206" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA206" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB206" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -19079,10 +19079,10 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z207" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA207" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB207" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -19170,13 +19170,13 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z208" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA208" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB208" s="21" t="str">
-        <x:v>1038406132baf06556f6abda8f1620ac4774984b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC208" s="21" t="str">
         <x:v>En cours</x:v>
@@ -19261,10 +19261,10 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z209" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA209" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB209" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -19358,7 +19358,7 @@
         <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB210" s="21" t="str">
-        <x:v>fc0d47528b092ffae3e49cc020fbc27e902dc01b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC210" s="21" t="str">
         <x:v>En cours</x:v>
@@ -19443,10 +19443,10 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z211" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA211" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB211" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -19534,10 +19534,10 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z212" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA212" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB212" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -19625,13 +19625,13 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z213" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA213" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB213" s="21" t="str">
-        <x:v>1038406132baf06556f6abda8f1620ac4774984b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC213" s="21" t="str">
         <x:v>En cours</x:v>
@@ -19716,10 +19716,10 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z214" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA214" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB214" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -19813,7 +19813,7 @@
         <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB215" s="21" t="str">
-        <x:v>622dd61d9ef0f43f5a9090416fe6cf21e4224e20</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC215" s="21" t="str">
         <x:v>En cours</x:v>
@@ -19904,7 +19904,7 @@
         <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB216" s="21" t="str">
-        <x:v>fc0d47528b092ffae3e49cc020fbc27e902dc01b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC216" s="21" t="str">
         <x:v>En cours</x:v>
@@ -19989,10 +19989,10 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z217" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA217" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB217" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -20086,7 +20086,7 @@
         <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB218" s="21" t="str">
-        <x:v>622dd61d9ef0f43f5a9090416fe6cf21e4224e20</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC218" s="21" t="str">
         <x:v>En cours</x:v>
@@ -20171,10 +20171,10 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z219" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA219" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB219" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -20262,10 +20262,10 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z220" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA220" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB220" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -20353,13 +20353,13 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z221" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA221" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB221" s="21" t="str">
-        <x:v>1038406132baf06556f6abda8f1620ac4774984b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC221" s="21" t="str">
         <x:v>En cours</x:v>
@@ -20450,7 +20450,7 @@
         <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB222" s="21" t="str">
-        <x:v>fc0d47528b092ffae3e49cc020fbc27e902dc01b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC222" s="21" t="str">
         <x:v>En cours</x:v>
@@ -20541,7 +20541,7 @@
         <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB223" s="21" t="str">
-        <x:v>622dd61d9ef0f43f5a9090416fe6cf21e4224e20</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC223" s="21" t="str">
         <x:v>En cours</x:v>
@@ -20632,7 +20632,7 @@
         <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB224" s="21" t="str">
-        <x:v>fc0d47528b092ffae3e49cc020fbc27e902dc01b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC224" s="21" t="str">
         <x:v>En cours</x:v>
@@ -20723,7 +20723,7 @@
         <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB225" s="21" t="str">
-        <x:v>fc0d47528b092ffae3e49cc020fbc27e902dc01b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC225" s="21" t="str">
         <x:v>En cours</x:v>
@@ -20808,13 +20808,13 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z226" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA226" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB226" s="21" t="str">
-        <x:v>1038406132baf06556f6abda8f1620ac4774984b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC226" s="21" t="str">
         <x:v>En cours</x:v>
@@ -20899,10 +20899,10 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z227" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA227" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB227" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -20990,10 +20990,10 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z228" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA228" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB228" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -21087,7 +21087,7 @@
         <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB229" s="21" t="str">
-        <x:v>622dd61d9ef0f43f5a9090416fe6cf21e4224e20</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC229" s="21" t="str">
         <x:v>En cours</x:v>
@@ -21172,10 +21172,10 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z230" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA230" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB230" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -21263,10 +21263,10 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z231" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA231" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB231" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -21354,13 +21354,13 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z232" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA232" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB232" s="21" t="str">
-        <x:v>1038406132baf06556f6abda8f1620ac4774984b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC232" s="21" t="str">
         <x:v>En cours</x:v>
@@ -21445,10 +21445,10 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z233" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA233" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB233" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -21536,10 +21536,10 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z234" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA234" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB234" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -21633,7 +21633,7 @@
         <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB235" s="21" t="str">
-        <x:v>622dd61d9ef0f43f5a9090416fe6cf21e4224e20</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC235" s="21" t="str">
         <x:v>En cours</x:v>
@@ -21718,13 +21718,13 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z236" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA236" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB236" s="21" t="str">
-        <x:v>1038406132baf06556f6abda8f1620ac4774984b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC236" s="21" t="str">
         <x:v>En cours</x:v>
@@ -21815,7 +21815,7 @@
         <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB237" s="21" t="str">
-        <x:v>622dd61d9ef0f43f5a9090416fe6cf21e4224e20</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC237" s="21" t="str">
         <x:v>En cours</x:v>
@@ -21900,10 +21900,10 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z238" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA238" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB238" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -21991,10 +21991,10 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z239" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA239" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB239" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -22088,7 +22088,7 @@
         <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB240" s="21" t="str">
-        <x:v>622dd61d9ef0f43f5a9090416fe6cf21e4224e20</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC240" s="21" t="str">
         <x:v>En cours</x:v>
@@ -22173,10 +22173,10 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z241" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA241" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB241" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -22264,10 +22264,10 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z242" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA242" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB242" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -22355,10 +22355,10 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z243" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA243" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB243" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -22452,7 +22452,7 @@
         <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB244" s="21" t="str">
-        <x:v>fc0d47528b092ffae3e49cc020fbc27e902dc01b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC244" s="21" t="str">
         <x:v>En cours</x:v>
@@ -22543,7 +22543,7 @@
         <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB245" s="21" t="str">
-        <x:v>fc0d47528b092ffae3e49cc020fbc27e902dc01b</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC245" s="21" t="str">
         <x:v>En cours</x:v>
@@ -22628,10 +22628,10 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z246" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA246" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB246" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -22651,84 +22651,84 @@
         <x:v>237</x:v>
       </x:c>
       <x:c r="D247" s="24" t="str">
-        <x:v>Lot 12 (prévu)</x:v>
+        <x:v>Lot 12 (master)</x:v>
       </x:c>
       <x:c r="E247" s="25" t="str">
         <x:v>Nature</x:v>
       </x:c>
       <x:c r="F247" s="24" t="str">
         <x:f>IF(AND(G247=8,COUNTIF(Q247:V247,"Atlas")=6),"Intégré","À faire")</x:f>
-        <x:v>À faire</x:v>
+        <x:v>Intégré</x:v>
       </x:c>
       <x:c r="G247" s="27" t="n">
         <x:f>COUNTIF(I247:P247,"Présent")</x:f>
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H247" s="24" t="str">
-        <x:v>À assembler</x:v>
+        <x:v>Réutilisé master #509</x:v>
       </x:c>
       <x:c r="I247" s="24" t="str">
-        <x:v>Référence</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="J247" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="K247" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="L247" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="M247" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="N247" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="O247" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="P247" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="Q247" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="R247" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="S247" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="T247" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="U247" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="V247" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="W247" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="X247" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="Y247" s="24" t="str">
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z247" s="24" t="str">
-        <x:v>Périmée (5/6)</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA247" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB247" s="21" t="str">
-        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC247" s="21" t="str">
-        <x:v>À intégrer</x:v>
+        <x:v>En cours</x:v>
       </x:c>
     </x:row>
     <x:row r="248" ht="40" customHeight="1">
@@ -22810,10 +22810,10 @@
         <x:v>Non consignée</x:v>
       </x:c>
       <x:c r="Z248" s="24" t="str">
-        <x:v>Publié 6/6</x:v>
+        <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA248" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication actuelle consignée. </x:v>
+        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB248" s="21" t="str">
         <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
@@ -22907,7 +22907,7 @@
         <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB249" s="21" t="str">
-        <x:v>622dd61d9ef0f43f5a9090416fe6cf21e4224e20</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC249" s="21" t="str">
         <x:v>En cours</x:v>
@@ -22998,7 +22998,7 @@
         <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB250" s="21" t="str">
-        <x:v>622dd61d9ef0f43f5a9090416fe6cf21e4224e20</x:v>
+        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
       </x:c>
       <x:c r="AC250" s="21" t="str">
         <x:v>En cours</x:v>
@@ -23094,7 +23094,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R675b355f137f4a0b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc86cc9929d6b4791"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs(symbols): qualify lot 12 and update Excel CSV to 200 packs
</commit_message>
<xml_diff>
--- a/doc_web_interne/docs/suivi-symboles/suivi-240-symboles-6-langues.xlsx
+++ b/doc_web_interne/docs/suivi-symboles/suivi-240-symboles-6-langues.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Suivi symboles" sheetId="1" r:id="Reb337a6b48024bfa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Suivi symboles" sheetId="1" r:id="R8d12d01cd7514264"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -811,7 +811,7 @@
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="7" t="str">
-        <x:v>Lot 11 en branche : 29 couvertures conservées, 203 nouveaux PNG. Preuves antérieures inchangées conservées.</x:v>
+        <x:v>Lot 12 en branche : 25 couvertures conservées, 175 nouveaux PNG. Preuves antérieures inchangées conservées.</x:v>
       </x:c>
       <x:c r="B3" s="7"/>
       <x:c r="C3" s="7"/>
@@ -848,21 +848,21 @@
       </x:c>
       <x:c r="B4" s="9" t="n">
         <x:f>COUNTIF(F11:F250,"Intégré")</x:f>
-        <x:v>175</x:v>
+        <x:v>200</x:v>
       </x:c>
       <x:c r="C4" s="3" t="str">
         <x:v>Packs à terminer</x:v>
       </x:c>
       <x:c r="D4" s="9" t="n">
         <x:f>COUNTA(B11:B250)-B4</x:f>
-        <x:v>65</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="E4" s="3" t="str">
         <x:v>Pages avec pack</x:v>
       </x:c>
       <x:c r="F4" s="9" t="n">
         <x:f>COUNTIF(Q11:V250,"Atlas")</x:f>
-        <x:v>1050</x:v>
+        <x:v>1200</x:v>
       </x:c>
       <x:c r="G4" s="3" t="str">
         <x:v>Pages web</x:v>
@@ -899,14 +899,14 @@
       </x:c>
       <x:c r="B5" s="9" t="n">
         <x:f>COUNTIF(W11:W250,"6/6 actuelles")</x:f>
-        <x:v>175</x:v>
+        <x:v>200</x:v>
       </x:c>
       <x:c r="C5" s="3" t="str">
         <x:v>QA 2560 px</x:v>
       </x:c>
       <x:c r="D5" s="9" t="n">
         <x:f>COUNTIF(X11:X250,"6/6 actuelles")</x:f>
-        <x:v>175</x:v>
+        <x:v>200</x:v>
       </x:c>
       <x:c r="E5" s="3" t="str">
         <x:v>Accord Thanh</x:v>
@@ -980,7 +980,7 @@
     </x:row>
     <x:row r="7" ht="20" customHeight="1">
       <x:c r="A7" s="7" t="str">
-        <x:v>175 packs ; 65 à compléter. Cadre commun : 1 440 pages. Publication antérieure conservée dans les reçus.</x:v>
+        <x:v>200 packs ; 40 à compléter. Cadre commun : 1 440 pages. Publication antérieure conservée dans les reçus.</x:v>
       </x:c>
       <x:c r="B7" s="7"/>
       <x:c r="C7" s="7"/>
@@ -1013,7 +1013,7 @@
     </x:row>
     <x:row r="8" ht="20" customHeight="1">
       <x:c r="A8" s="7" t="str">
-        <x:v>Source : rapport canonique du 20/10/2026, empreinte 7721867ea6eecebc. Révision : 34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>Source : rapport canonique du 20/10/2026, empreinte 42ee542429cbc3ed. Révision : b17117db72da867328bfee7e7b5ac7c17acc0aab</x:v>
       </x:c>
       <x:c r="B8" s="7"/>
       <x:c r="C8" s="7"/>
@@ -8637,69 +8637,69 @@
         <x:v>83</x:v>
       </x:c>
       <x:c r="D93" s="24" t="str">
-        <x:v>À planifier</x:v>
+        <x:v>Lot 12</x:v>
       </x:c>
       <x:c r="E93" s="25" t="str">
         <x:v>Animaux</x:v>
       </x:c>
       <x:c r="F93" s="24" t="str">
         <x:f>IF(AND(G93=8,COUNTIF(Q93:V93,"Atlas")=6),"Intégré","À faire")</x:f>
-        <x:v>À faire</x:v>
+        <x:v>Intégré</x:v>
       </x:c>
       <x:c r="G93" s="27" t="n">
         <x:f>COUNTIF(I93:P93,"Présent")</x:f>
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H93" s="24" t="str">
-        <x:v>À assembler</x:v>
+        <x:v>Archivé Drive</x:v>
       </x:c>
       <x:c r="I93" s="24" t="str">
-        <x:v>Référence</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="J93" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="K93" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="L93" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="M93" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="N93" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="O93" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="P93" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="Q93" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="R93" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="S93" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="T93" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="U93" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="V93" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="W93" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="X93" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="Y93" s="24" t="str">
         <x:v>Non consignée</x:v>
@@ -8708,13 +8708,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA93" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB93" s="21" t="str">
-        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
+        <x:v>b17117db72da867328bfee7e7b5ac7c17acc0aab</x:v>
       </x:c>
       <x:c r="AC93" s="21" t="str">
-        <x:v>À intégrer</x:v>
+        <x:v>En cours</x:v>
       </x:c>
     </x:row>
     <x:row r="94" ht="40" customHeight="1">
@@ -10002,69 +10002,69 @@
         <x:v>98</x:v>
       </x:c>
       <x:c r="D108" s="24" t="str">
-        <x:v>À planifier</x:v>
+        <x:v>Lot 12</x:v>
       </x:c>
       <x:c r="E108" s="25" t="str">
         <x:v>Corps</x:v>
       </x:c>
       <x:c r="F108" s="24" t="str">
         <x:f>IF(AND(G108=8,COUNTIF(Q108:V108,"Atlas")=6),"Intégré","À faire")</x:f>
-        <x:v>À faire</x:v>
+        <x:v>Intégré</x:v>
       </x:c>
       <x:c r="G108" s="27" t="n">
         <x:f>COUNTIF(I108:P108,"Présent")</x:f>
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H108" s="24" t="str">
-        <x:v>À assembler</x:v>
+        <x:v>Archivé Drive</x:v>
       </x:c>
       <x:c r="I108" s="24" t="str">
-        <x:v>Référence</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="J108" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="K108" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="L108" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="M108" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="N108" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="O108" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="P108" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="Q108" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="R108" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="S108" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="T108" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="U108" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="V108" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="W108" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="X108" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="Y108" s="24" t="str">
         <x:v>Non consignée</x:v>
@@ -10073,13 +10073,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA108" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB108" s="21" t="str">
-        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
+        <x:v>b17117db72da867328bfee7e7b5ac7c17acc0aab</x:v>
       </x:c>
       <x:c r="AC108" s="21" t="str">
-        <x:v>À intégrer</x:v>
+        <x:v>En cours</x:v>
       </x:c>
     </x:row>
     <x:row r="109" ht="40" customHeight="1">
@@ -10093,69 +10093,69 @@
         <x:v>99</x:v>
       </x:c>
       <x:c r="D109" s="24" t="str">
-        <x:v>À planifier</x:v>
+        <x:v>Lot 12</x:v>
       </x:c>
       <x:c r="E109" s="25" t="str">
         <x:v>Animaux</x:v>
       </x:c>
       <x:c r="F109" s="24" t="str">
         <x:f>IF(AND(G109=8,COUNTIF(Q109:V109,"Atlas")=6),"Intégré","À faire")</x:f>
-        <x:v>À faire</x:v>
+        <x:v>Intégré</x:v>
       </x:c>
       <x:c r="G109" s="27" t="n">
         <x:f>COUNTIF(I109:P109,"Présent")</x:f>
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H109" s="24" t="str">
-        <x:v>À assembler</x:v>
+        <x:v>Archivé Drive</x:v>
       </x:c>
       <x:c r="I109" s="24" t="str">
-        <x:v>Référence</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="J109" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="K109" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="L109" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="M109" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="N109" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="O109" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="P109" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="Q109" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="R109" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="S109" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="T109" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="U109" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="V109" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="W109" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="X109" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="Y109" s="24" t="str">
         <x:v>Non consignée</x:v>
@@ -10164,13 +10164,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA109" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB109" s="21" t="str">
-        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
+        <x:v>b17117db72da867328bfee7e7b5ac7c17acc0aab</x:v>
       </x:c>
       <x:c r="AC109" s="21" t="str">
-        <x:v>À intégrer</x:v>
+        <x:v>En cours</x:v>
       </x:c>
     </x:row>
     <x:row r="110" ht="40" customHeight="1">
@@ -10366,69 +10366,69 @@
         <x:v>102</x:v>
       </x:c>
       <x:c r="D112" s="24" t="str">
-        <x:v>À planifier</x:v>
+        <x:v>Lot 12</x:v>
       </x:c>
       <x:c r="E112" s="25" t="str">
         <x:v>Lieux</x:v>
       </x:c>
       <x:c r="F112" s="24" t="str">
         <x:f>IF(AND(G112=8,COUNTIF(Q112:V112,"Atlas")=6),"Intégré","À faire")</x:f>
-        <x:v>À faire</x:v>
+        <x:v>Intégré</x:v>
       </x:c>
       <x:c r="G112" s="27" t="n">
         <x:f>COUNTIF(I112:P112,"Présent")</x:f>
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H112" s="24" t="str">
-        <x:v>À assembler</x:v>
+        <x:v>Archivé Drive</x:v>
       </x:c>
       <x:c r="I112" s="24" t="str">
-        <x:v>Référence</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="J112" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="K112" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="L112" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="M112" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="N112" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="O112" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="P112" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="Q112" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="R112" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="S112" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="T112" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="U112" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="V112" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="W112" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="X112" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="Y112" s="24" t="str">
         <x:v>Non consignée</x:v>
@@ -10437,13 +10437,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA112" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB112" s="21" t="str">
-        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
+        <x:v>b17117db72da867328bfee7e7b5ac7c17acc0aab</x:v>
       </x:c>
       <x:c r="AC112" s="21" t="str">
-        <x:v>À intégrer</x:v>
+        <x:v>En cours</x:v>
       </x:c>
     </x:row>
     <x:row r="113" ht="40" customHeight="1">
@@ -10730,69 +10730,69 @@
         <x:v>106</x:v>
       </x:c>
       <x:c r="D116" s="24" t="str">
-        <x:v>À planifier</x:v>
+        <x:v>Lot 12</x:v>
       </x:c>
       <x:c r="E116" s="25" t="str">
         <x:v>Objets</x:v>
       </x:c>
       <x:c r="F116" s="24" t="str">
         <x:f>IF(AND(G116=8,COUNTIF(Q116:V116,"Atlas")=6),"Intégré","À faire")</x:f>
-        <x:v>À faire</x:v>
+        <x:v>Intégré</x:v>
       </x:c>
       <x:c r="G116" s="27" t="n">
         <x:f>COUNTIF(I116:P116,"Présent")</x:f>
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H116" s="24" t="str">
-        <x:v>À assembler</x:v>
+        <x:v>Archivé Drive</x:v>
       </x:c>
       <x:c r="I116" s="24" t="str">
-        <x:v>Référence</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="J116" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="K116" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="L116" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="M116" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="N116" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="O116" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="P116" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="Q116" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="R116" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="S116" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="T116" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="U116" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="V116" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="W116" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="X116" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="Y116" s="24" t="str">
         <x:v>Non consignée</x:v>
@@ -10801,13 +10801,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA116" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB116" s="21" t="str">
-        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
+        <x:v>b17117db72da867328bfee7e7b5ac7c17acc0aab</x:v>
       </x:c>
       <x:c r="AC116" s="21" t="str">
-        <x:v>À intégrer</x:v>
+        <x:v>En cours</x:v>
       </x:c>
     </x:row>
     <x:row r="117" ht="40" customHeight="1">
@@ -11731,69 +11731,69 @@
         <x:v>117</x:v>
       </x:c>
       <x:c r="D127" s="24" t="str">
-        <x:v>À planifier</x:v>
+        <x:v>Lot 12</x:v>
       </x:c>
       <x:c r="E127" s="25" t="str">
         <x:v>Animaux</x:v>
       </x:c>
       <x:c r="F127" s="24" t="str">
         <x:f>IF(AND(G127=8,COUNTIF(Q127:V127,"Atlas")=6),"Intégré","À faire")</x:f>
-        <x:v>À faire</x:v>
+        <x:v>Intégré</x:v>
       </x:c>
       <x:c r="G127" s="27" t="n">
         <x:f>COUNTIF(I127:P127,"Présent")</x:f>
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H127" s="24" t="str">
-        <x:v>À assembler</x:v>
+        <x:v>Archivé Drive</x:v>
       </x:c>
       <x:c r="I127" s="24" t="str">
-        <x:v>Référence</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="J127" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="K127" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="L127" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="M127" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="N127" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="O127" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="P127" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="Q127" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="R127" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="S127" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="T127" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="U127" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="V127" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="W127" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="X127" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="Y127" s="24" t="str">
         <x:v>Non consignée</x:v>
@@ -11802,13 +11802,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA127" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB127" s="21" t="str">
-        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
+        <x:v>b17117db72da867328bfee7e7b5ac7c17acc0aab</x:v>
       </x:c>
       <x:c r="AC127" s="21" t="str">
-        <x:v>À intégrer</x:v>
+        <x:v>En cours</x:v>
       </x:c>
     </x:row>
     <x:row r="128" ht="40" customHeight="1">
@@ -12095,69 +12095,69 @@
         <x:v>121</x:v>
       </x:c>
       <x:c r="D131" s="24" t="str">
-        <x:v>À planifier</x:v>
+        <x:v>Lot 12</x:v>
       </x:c>
       <x:c r="E131" s="25" t="str">
         <x:v>Animaux</x:v>
       </x:c>
       <x:c r="F131" s="24" t="str">
         <x:f>IF(AND(G131=8,COUNTIF(Q131:V131,"Atlas")=6),"Intégré","À faire")</x:f>
-        <x:v>À faire</x:v>
+        <x:v>Intégré</x:v>
       </x:c>
       <x:c r="G131" s="27" t="n">
         <x:f>COUNTIF(I131:P131,"Présent")</x:f>
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H131" s="24" t="str">
-        <x:v>À assembler</x:v>
+        <x:v>Archivé Drive</x:v>
       </x:c>
       <x:c r="I131" s="24" t="str">
-        <x:v>Référence</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="J131" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="K131" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="L131" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="M131" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="N131" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="O131" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="P131" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="Q131" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="R131" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="S131" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="T131" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="U131" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="V131" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="W131" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="X131" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="Y131" s="24" t="str">
         <x:v>Non consignée</x:v>
@@ -12166,13 +12166,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA131" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB131" s="21" t="str">
-        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
+        <x:v>b17117db72da867328bfee7e7b5ac7c17acc0aab</x:v>
       </x:c>
       <x:c r="AC131" s="21" t="str">
-        <x:v>À intégrer</x:v>
+        <x:v>En cours</x:v>
       </x:c>
     </x:row>
     <x:row r="132" ht="40" customHeight="1">
@@ -12368,69 +12368,69 @@
         <x:v>124</x:v>
       </x:c>
       <x:c r="D134" s="24" t="str">
-        <x:v>À planifier</x:v>
+        <x:v>Lot 12</x:v>
       </x:c>
       <x:c r="E134" s="25" t="str">
         <x:v>Animaux</x:v>
       </x:c>
       <x:c r="F134" s="24" t="str">
         <x:f>IF(AND(G134=8,COUNTIF(Q134:V134,"Atlas")=6),"Intégré","À faire")</x:f>
-        <x:v>À faire</x:v>
+        <x:v>Intégré</x:v>
       </x:c>
       <x:c r="G134" s="27" t="n">
         <x:f>COUNTIF(I134:P134,"Présent")</x:f>
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H134" s="24" t="str">
-        <x:v>À assembler</x:v>
+        <x:v>Archivé Drive</x:v>
       </x:c>
       <x:c r="I134" s="24" t="str">
-        <x:v>Référence</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="J134" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="K134" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="L134" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="M134" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="N134" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="O134" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="P134" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="Q134" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="R134" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="S134" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="T134" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="U134" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="V134" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="W134" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="X134" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="Y134" s="24" t="str">
         <x:v>Non consignée</x:v>
@@ -12439,13 +12439,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA134" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB134" s="21" t="str">
-        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
+        <x:v>b17117db72da867328bfee7e7b5ac7c17acc0aab</x:v>
       </x:c>
       <x:c r="AC134" s="21" t="str">
-        <x:v>À intégrer</x:v>
+        <x:v>En cours</x:v>
       </x:c>
     </x:row>
     <x:row r="135" ht="40" customHeight="1">
@@ -13187,69 +13187,69 @@
         <x:v>133</x:v>
       </x:c>
       <x:c r="D143" s="24" t="str">
-        <x:v>À planifier</x:v>
+        <x:v>Lot 12</x:v>
       </x:c>
       <x:c r="E143" s="25" t="str">
         <x:v>Animaux</x:v>
       </x:c>
       <x:c r="F143" s="24" t="str">
         <x:f>IF(AND(G143=8,COUNTIF(Q143:V143,"Atlas")=6),"Intégré","À faire")</x:f>
-        <x:v>À faire</x:v>
+        <x:v>Intégré</x:v>
       </x:c>
       <x:c r="G143" s="27" t="n">
         <x:f>COUNTIF(I143:P143,"Présent")</x:f>
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H143" s="24" t="str">
-        <x:v>À assembler</x:v>
+        <x:v>Archivé Drive</x:v>
       </x:c>
       <x:c r="I143" s="24" t="str">
-        <x:v>Référence</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="J143" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="K143" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="L143" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="M143" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="N143" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="O143" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="P143" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="Q143" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="R143" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="S143" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="T143" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="U143" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="V143" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="W143" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="X143" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="Y143" s="24" t="str">
         <x:v>Non consignée</x:v>
@@ -13258,13 +13258,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA143" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB143" s="21" t="str">
-        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
+        <x:v>b17117db72da867328bfee7e7b5ac7c17acc0aab</x:v>
       </x:c>
       <x:c r="AC143" s="21" t="str">
-        <x:v>À intégrer</x:v>
+        <x:v>En cours</x:v>
       </x:c>
     </x:row>
     <x:row r="144" ht="40" customHeight="1">
@@ -14370,69 +14370,69 @@
         <x:v>146</x:v>
       </x:c>
       <x:c r="D156" s="24" t="str">
-        <x:v>À planifier</x:v>
+        <x:v>Lot 12</x:v>
       </x:c>
       <x:c r="E156" s="25" t="str">
         <x:v>Animaux</x:v>
       </x:c>
       <x:c r="F156" s="24" t="str">
         <x:f>IF(AND(G156=8,COUNTIF(Q156:V156,"Atlas")=6),"Intégré","À faire")</x:f>
-        <x:v>À faire</x:v>
+        <x:v>Intégré</x:v>
       </x:c>
       <x:c r="G156" s="27" t="n">
         <x:f>COUNTIF(I156:P156,"Présent")</x:f>
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H156" s="24" t="str">
-        <x:v>À assembler</x:v>
+        <x:v>Archivé Drive</x:v>
       </x:c>
       <x:c r="I156" s="24" t="str">
-        <x:v>Référence</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="J156" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="K156" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="L156" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="M156" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="N156" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="O156" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="P156" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="Q156" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="R156" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="S156" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="T156" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="U156" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="V156" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="W156" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="X156" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="Y156" s="24" t="str">
         <x:v>Non consignée</x:v>
@@ -14441,13 +14441,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA156" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB156" s="21" t="str">
-        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
+        <x:v>b17117db72da867328bfee7e7b5ac7c17acc0aab</x:v>
       </x:c>
       <x:c r="AC156" s="21" t="str">
-        <x:v>À intégrer</x:v>
+        <x:v>En cours</x:v>
       </x:c>
     </x:row>
     <x:row r="157" ht="40" customHeight="1">
@@ -14825,69 +14825,69 @@
         <x:v>151</x:v>
       </x:c>
       <x:c r="D161" s="24" t="str">
-        <x:v>À planifier</x:v>
+        <x:v>Lot 12</x:v>
       </x:c>
       <x:c r="E161" s="25" t="str">
         <x:v>Animaux</x:v>
       </x:c>
       <x:c r="F161" s="24" t="str">
         <x:f>IF(AND(G161=8,COUNTIF(Q161:V161,"Atlas")=6),"Intégré","À faire")</x:f>
-        <x:v>À faire</x:v>
+        <x:v>Intégré</x:v>
       </x:c>
       <x:c r="G161" s="27" t="n">
         <x:f>COUNTIF(I161:P161,"Présent")</x:f>
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H161" s="24" t="str">
-        <x:v>À assembler</x:v>
+        <x:v>Archivé Drive</x:v>
       </x:c>
       <x:c r="I161" s="24" t="str">
-        <x:v>Référence</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="J161" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="K161" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="L161" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="M161" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="N161" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="O161" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="P161" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="Q161" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="R161" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="S161" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="T161" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="U161" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="V161" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="W161" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="X161" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="Y161" s="24" t="str">
         <x:v>Non consignée</x:v>
@@ -14896,13 +14896,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA161" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB161" s="21" t="str">
-        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
+        <x:v>b17117db72da867328bfee7e7b5ac7c17acc0aab</x:v>
       </x:c>
       <x:c r="AC161" s="21" t="str">
-        <x:v>À intégrer</x:v>
+        <x:v>En cours</x:v>
       </x:c>
     </x:row>
     <x:row r="162" ht="40" customHeight="1">
@@ -15462,69 +15462,69 @@
         <x:v>158</x:v>
       </x:c>
       <x:c r="D168" s="24" t="str">
-        <x:v>À planifier</x:v>
+        <x:v>Lot 12</x:v>
       </x:c>
       <x:c r="E168" s="25" t="str">
         <x:v>Lieux</x:v>
       </x:c>
       <x:c r="F168" s="24" t="str">
         <x:f>IF(AND(G168=8,COUNTIF(Q168:V168,"Atlas")=6),"Intégré","À faire")</x:f>
-        <x:v>À faire</x:v>
+        <x:v>Intégré</x:v>
       </x:c>
       <x:c r="G168" s="27" t="n">
         <x:f>COUNTIF(I168:P168,"Présent")</x:f>
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H168" s="24" t="str">
-        <x:v>À assembler</x:v>
+        <x:v>Archivé Drive</x:v>
       </x:c>
       <x:c r="I168" s="24" t="str">
-        <x:v>Référence</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="J168" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="K168" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="L168" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="M168" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="N168" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="O168" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="P168" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="Q168" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="R168" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="S168" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="T168" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="U168" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="V168" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="W168" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="X168" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="Y168" s="24" t="str">
         <x:v>Non consignée</x:v>
@@ -15533,13 +15533,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA168" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB168" s="21" t="str">
-        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
+        <x:v>b17117db72da867328bfee7e7b5ac7c17acc0aab</x:v>
       </x:c>
       <x:c r="AC168" s="21" t="str">
-        <x:v>À intégrer</x:v>
+        <x:v>En cours</x:v>
       </x:c>
     </x:row>
     <x:row r="169" ht="40" customHeight="1">
@@ -15553,69 +15553,69 @@
         <x:v>159</x:v>
       </x:c>
       <x:c r="D169" s="24" t="str">
-        <x:v>À planifier</x:v>
+        <x:v>Lot 12</x:v>
       </x:c>
       <x:c r="E169" s="25" t="str">
         <x:v>Lieux</x:v>
       </x:c>
       <x:c r="F169" s="24" t="str">
         <x:f>IF(AND(G169=8,COUNTIF(Q169:V169,"Atlas")=6),"Intégré","À faire")</x:f>
-        <x:v>À faire</x:v>
+        <x:v>Intégré</x:v>
       </x:c>
       <x:c r="G169" s="27" t="n">
         <x:f>COUNTIF(I169:P169,"Présent")</x:f>
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H169" s="24" t="str">
-        <x:v>À assembler</x:v>
+        <x:v>Archivé Drive</x:v>
       </x:c>
       <x:c r="I169" s="24" t="str">
-        <x:v>Référence</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="J169" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="K169" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="L169" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="M169" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="N169" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="O169" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="P169" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="Q169" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="R169" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="S169" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="T169" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="U169" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="V169" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="W169" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="X169" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="Y169" s="24" t="str">
         <x:v>Non consignée</x:v>
@@ -15624,13 +15624,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA169" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB169" s="21" t="str">
-        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
+        <x:v>b17117db72da867328bfee7e7b5ac7c17acc0aab</x:v>
       </x:c>
       <x:c r="AC169" s="21" t="str">
-        <x:v>À intégrer</x:v>
+        <x:v>En cours</x:v>
       </x:c>
     </x:row>
     <x:row r="170" ht="40" customHeight="1">
@@ -16008,69 +16008,69 @@
         <x:v>164</x:v>
       </x:c>
       <x:c r="D174" s="24" t="str">
-        <x:v>À planifier</x:v>
+        <x:v>Lot 12</x:v>
       </x:c>
       <x:c r="E174" s="25" t="str">
         <x:v>Lieux</x:v>
       </x:c>
       <x:c r="F174" s="24" t="str">
         <x:f>IF(AND(G174=8,COUNTIF(Q174:V174,"Atlas")=6),"Intégré","À faire")</x:f>
-        <x:v>À faire</x:v>
+        <x:v>Intégré</x:v>
       </x:c>
       <x:c r="G174" s="27" t="n">
         <x:f>COUNTIF(I174:P174,"Présent")</x:f>
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H174" s="24" t="str">
-        <x:v>À assembler</x:v>
+        <x:v>Archivé Drive</x:v>
       </x:c>
       <x:c r="I174" s="24" t="str">
-        <x:v>Référence</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="J174" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="K174" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="L174" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="M174" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="N174" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="O174" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="P174" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="Q174" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="R174" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="S174" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="T174" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="U174" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="V174" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="W174" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="X174" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="Y174" s="24" t="str">
         <x:v>Non consignée</x:v>
@@ -16079,13 +16079,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA174" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB174" s="21" t="str">
-        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
+        <x:v>b17117db72da867328bfee7e7b5ac7c17acc0aab</x:v>
       </x:c>
       <x:c r="AC174" s="21" t="str">
-        <x:v>À intégrer</x:v>
+        <x:v>En cours</x:v>
       </x:c>
     </x:row>
     <x:row r="175" ht="40" customHeight="1">
@@ -16099,69 +16099,69 @@
         <x:v>165</x:v>
       </x:c>
       <x:c r="D175" s="24" t="str">
-        <x:v>À planifier</x:v>
+        <x:v>Lot 12</x:v>
       </x:c>
       <x:c r="E175" s="25" t="str">
         <x:v>Nature</x:v>
       </x:c>
       <x:c r="F175" s="24" t="str">
         <x:f>IF(AND(G175=8,COUNTIF(Q175:V175,"Atlas")=6),"Intégré","À faire")</x:f>
-        <x:v>À faire</x:v>
+        <x:v>Intégré</x:v>
       </x:c>
       <x:c r="G175" s="27" t="n">
         <x:f>COUNTIF(I175:P175,"Présent")</x:f>
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H175" s="24" t="str">
-        <x:v>À assembler</x:v>
+        <x:v>Archivé Drive</x:v>
       </x:c>
       <x:c r="I175" s="24" t="str">
-        <x:v>Référence</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="J175" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="K175" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="L175" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="M175" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="N175" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="O175" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="P175" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="Q175" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="R175" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="S175" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="T175" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="U175" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="V175" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="W175" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="X175" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="Y175" s="24" t="str">
         <x:v>Non consignée</x:v>
@@ -16170,13 +16170,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA175" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB175" s="21" t="str">
-        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
+        <x:v>b17117db72da867328bfee7e7b5ac7c17acc0aab</x:v>
       </x:c>
       <x:c r="AC175" s="21" t="str">
-        <x:v>À intégrer</x:v>
+        <x:v>En cours</x:v>
       </x:c>
     </x:row>
     <x:row r="176" ht="40" customHeight="1">
@@ -16190,69 +16190,69 @@
         <x:v>166</x:v>
       </x:c>
       <x:c r="D176" s="24" t="str">
-        <x:v>À planifier</x:v>
+        <x:v>Lot 12</x:v>
       </x:c>
       <x:c r="E176" s="25" t="str">
         <x:v>Animaux</x:v>
       </x:c>
       <x:c r="F176" s="24" t="str">
         <x:f>IF(AND(G176=8,COUNTIF(Q176:V176,"Atlas")=6),"Intégré","À faire")</x:f>
-        <x:v>À faire</x:v>
+        <x:v>Intégré</x:v>
       </x:c>
       <x:c r="G176" s="27" t="n">
         <x:f>COUNTIF(I176:P176,"Présent")</x:f>
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H176" s="24" t="str">
-        <x:v>À assembler</x:v>
+        <x:v>Archivé Drive</x:v>
       </x:c>
       <x:c r="I176" s="24" t="str">
-        <x:v>Référence</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="J176" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="K176" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="L176" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="M176" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="N176" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="O176" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="P176" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="Q176" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="R176" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="S176" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="T176" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="U176" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="V176" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="W176" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="X176" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="Y176" s="24" t="str">
         <x:v>Non consignée</x:v>
@@ -16261,13 +16261,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA176" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB176" s="21" t="str">
-        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
+        <x:v>b17117db72da867328bfee7e7b5ac7c17acc0aab</x:v>
       </x:c>
       <x:c r="AC176" s="21" t="str">
-        <x:v>À intégrer</x:v>
+        <x:v>En cours</x:v>
       </x:c>
     </x:row>
     <x:row r="177" ht="40" customHeight="1">
@@ -18192,69 +18192,69 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="D198" s="24" t="str">
-        <x:v>À planifier</x:v>
+        <x:v>Lot 12</x:v>
       </x:c>
       <x:c r="E198" s="25" t="str">
         <x:v>Animaux</x:v>
       </x:c>
       <x:c r="F198" s="24" t="str">
         <x:f>IF(AND(G198=8,COUNTIF(Q198:V198,"Atlas")=6),"Intégré","À faire")</x:f>
-        <x:v>À faire</x:v>
+        <x:v>Intégré</x:v>
       </x:c>
       <x:c r="G198" s="27" t="n">
         <x:f>COUNTIF(I198:P198,"Présent")</x:f>
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H198" s="24" t="str">
-        <x:v>À assembler</x:v>
+        <x:v>Archivé Drive</x:v>
       </x:c>
       <x:c r="I198" s="24" t="str">
-        <x:v>Référence</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="J198" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="K198" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="L198" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="M198" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="N198" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="O198" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="P198" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="Q198" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="R198" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="S198" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="T198" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="U198" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="V198" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="W198" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="X198" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="Y198" s="24" t="str">
         <x:v>Non consignée</x:v>
@@ -18263,13 +18263,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA198" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB198" s="21" t="str">
-        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
+        <x:v>b17117db72da867328bfee7e7b5ac7c17acc0aab</x:v>
       </x:c>
       <x:c r="AC198" s="21" t="str">
-        <x:v>À intégrer</x:v>
+        <x:v>En cours</x:v>
       </x:c>
     </x:row>
     <x:row r="199" ht="40" customHeight="1">
@@ -19193,69 +19193,69 @@
         <x:v>199</x:v>
       </x:c>
       <x:c r="D209" s="24" t="str">
-        <x:v>À planifier</x:v>
+        <x:v>Lot 12</x:v>
       </x:c>
       <x:c r="E209" s="25" t="str">
         <x:v>Animaux</x:v>
       </x:c>
       <x:c r="F209" s="24" t="str">
         <x:f>IF(AND(G209=8,COUNTIF(Q209:V209,"Atlas")=6),"Intégré","À faire")</x:f>
-        <x:v>À faire</x:v>
+        <x:v>Intégré</x:v>
       </x:c>
       <x:c r="G209" s="27" t="n">
         <x:f>COUNTIF(I209:P209,"Présent")</x:f>
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H209" s="24" t="str">
-        <x:v>À assembler</x:v>
+        <x:v>Archivé Drive</x:v>
       </x:c>
       <x:c r="I209" s="24" t="str">
-        <x:v>Référence</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="J209" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="K209" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="L209" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="M209" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="N209" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="O209" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="P209" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="Q209" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="R209" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="S209" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="T209" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="U209" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="V209" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="W209" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="X209" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="Y209" s="24" t="str">
         <x:v>Non consignée</x:v>
@@ -19264,13 +19264,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA209" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB209" s="21" t="str">
-        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
+        <x:v>b17117db72da867328bfee7e7b5ac7c17acc0aab</x:v>
       </x:c>
       <x:c r="AC209" s="21" t="str">
-        <x:v>À intégrer</x:v>
+        <x:v>En cours</x:v>
       </x:c>
     </x:row>
     <x:row r="210" ht="40" customHeight="1">
@@ -19921,69 +19921,69 @@
         <x:v>207</x:v>
       </x:c>
       <x:c r="D217" s="24" t="str">
-        <x:v>À planifier</x:v>
+        <x:v>Lot 12</x:v>
       </x:c>
       <x:c r="E217" s="25" t="str">
         <x:v>Animaux</x:v>
       </x:c>
       <x:c r="F217" s="24" t="str">
         <x:f>IF(AND(G217=8,COUNTIF(Q217:V217,"Atlas")=6),"Intégré","À faire")</x:f>
-        <x:v>À faire</x:v>
+        <x:v>Intégré</x:v>
       </x:c>
       <x:c r="G217" s="27" t="n">
         <x:f>COUNTIF(I217:P217,"Présent")</x:f>
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H217" s="24" t="str">
-        <x:v>À assembler</x:v>
+        <x:v>Archivé Drive</x:v>
       </x:c>
       <x:c r="I217" s="24" t="str">
-        <x:v>Référence</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="J217" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="K217" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="L217" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="M217" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="N217" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="O217" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="P217" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="Q217" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="R217" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="S217" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="T217" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="U217" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="V217" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="W217" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="X217" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="Y217" s="24" t="str">
         <x:v>Non consignée</x:v>
@@ -19992,13 +19992,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA217" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB217" s="21" t="str">
-        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
+        <x:v>b17117db72da867328bfee7e7b5ac7c17acc0aab</x:v>
       </x:c>
       <x:c r="AC217" s="21" t="str">
-        <x:v>À intégrer</x:v>
+        <x:v>En cours</x:v>
       </x:c>
     </x:row>
     <x:row r="218" ht="40" customHeight="1">
@@ -20103,69 +20103,69 @@
         <x:v>209</x:v>
       </x:c>
       <x:c r="D219" s="24" t="str">
-        <x:v>À planifier</x:v>
+        <x:v>Lot 12</x:v>
       </x:c>
       <x:c r="E219" s="25" t="str">
         <x:v>Animaux</x:v>
       </x:c>
       <x:c r="F219" s="24" t="str">
         <x:f>IF(AND(G219=8,COUNTIF(Q219:V219,"Atlas")=6),"Intégré","À faire")</x:f>
-        <x:v>À faire</x:v>
+        <x:v>Intégré</x:v>
       </x:c>
       <x:c r="G219" s="27" t="n">
         <x:f>COUNTIF(I219:P219,"Présent")</x:f>
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H219" s="24" t="str">
-        <x:v>À assembler</x:v>
+        <x:v>Archivé Drive</x:v>
       </x:c>
       <x:c r="I219" s="24" t="str">
-        <x:v>Référence</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="J219" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="K219" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="L219" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="M219" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="N219" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="O219" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="P219" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="Q219" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="R219" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="S219" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="T219" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="U219" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="V219" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="W219" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="X219" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="Y219" s="24" t="str">
         <x:v>Non consignée</x:v>
@@ -20174,13 +20174,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA219" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB219" s="21" t="str">
-        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
+        <x:v>b17117db72da867328bfee7e7b5ac7c17acc0aab</x:v>
       </x:c>
       <x:c r="AC219" s="21" t="str">
-        <x:v>À intégrer</x:v>
+        <x:v>En cours</x:v>
       </x:c>
     </x:row>
     <x:row r="220" ht="40" customHeight="1">
@@ -20194,69 +20194,69 @@
         <x:v>210</x:v>
       </x:c>
       <x:c r="D220" s="24" t="str">
-        <x:v>À planifier</x:v>
+        <x:v>Lot 12</x:v>
       </x:c>
       <x:c r="E220" s="25" t="str">
         <x:v>Nature</x:v>
       </x:c>
       <x:c r="F220" s="24" t="str">
         <x:f>IF(AND(G220=8,COUNTIF(Q220:V220,"Atlas")=6),"Intégré","À faire")</x:f>
-        <x:v>À faire</x:v>
+        <x:v>Intégré</x:v>
       </x:c>
       <x:c r="G220" s="27" t="n">
         <x:f>COUNTIF(I220:P220,"Présent")</x:f>
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H220" s="24" t="str">
-        <x:v>À assembler</x:v>
+        <x:v>Archivé Drive</x:v>
       </x:c>
       <x:c r="I220" s="24" t="str">
-        <x:v>Référence</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="J220" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="K220" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="L220" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="M220" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="N220" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="O220" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="P220" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="Q220" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="R220" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="S220" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="T220" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="U220" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="V220" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="W220" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="X220" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="Y220" s="24" t="str">
         <x:v>Non consignée</x:v>
@@ -20265,13 +20265,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA220" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB220" s="21" t="str">
-        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
+        <x:v>b17117db72da867328bfee7e7b5ac7c17acc0aab</x:v>
       </x:c>
       <x:c r="AC220" s="21" t="str">
-        <x:v>À intégrer</x:v>
+        <x:v>En cours</x:v>
       </x:c>
     </x:row>
     <x:row r="221" ht="40" customHeight="1">
@@ -21468,69 +21468,69 @@
         <x:v>224</x:v>
       </x:c>
       <x:c r="D234" s="24" t="str">
-        <x:v>À planifier</x:v>
+        <x:v>Lot 12</x:v>
       </x:c>
       <x:c r="E234" s="25" t="str">
         <x:v>Animaux</x:v>
       </x:c>
       <x:c r="F234" s="24" t="str">
         <x:f>IF(AND(G234=8,COUNTIF(Q234:V234,"Atlas")=6),"Intégré","À faire")</x:f>
-        <x:v>À faire</x:v>
+        <x:v>Intégré</x:v>
       </x:c>
       <x:c r="G234" s="27" t="n">
         <x:f>COUNTIF(I234:P234,"Présent")</x:f>
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H234" s="24" t="str">
-        <x:v>À assembler</x:v>
+        <x:v>Archivé Drive</x:v>
       </x:c>
       <x:c r="I234" s="24" t="str">
-        <x:v>Référence</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="J234" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="K234" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="L234" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="M234" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="N234" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="O234" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="P234" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="Q234" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="R234" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="S234" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="T234" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="U234" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="V234" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="W234" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="X234" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="Y234" s="24" t="str">
         <x:v>Non consignée</x:v>
@@ -21539,13 +21539,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA234" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB234" s="21" t="str">
-        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
+        <x:v>b17117db72da867328bfee7e7b5ac7c17acc0aab</x:v>
       </x:c>
       <x:c r="AC234" s="21" t="str">
-        <x:v>À intégrer</x:v>
+        <x:v>En cours</x:v>
       </x:c>
     </x:row>
     <x:row r="235" ht="40" customHeight="1">
@@ -21923,69 +21923,69 @@
         <x:v>229</x:v>
       </x:c>
       <x:c r="D239" s="24" t="str">
-        <x:v>À planifier</x:v>
+        <x:v>Lot 12</x:v>
       </x:c>
       <x:c r="E239" s="25" t="str">
         <x:v>Nature</x:v>
       </x:c>
       <x:c r="F239" s="24" t="str">
         <x:f>IF(AND(G239=8,COUNTIF(Q239:V239,"Atlas")=6),"Intégré","À faire")</x:f>
-        <x:v>À faire</x:v>
+        <x:v>Intégré</x:v>
       </x:c>
       <x:c r="G239" s="27" t="n">
         <x:f>COUNTIF(I239:P239,"Présent")</x:f>
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H239" s="24" t="str">
-        <x:v>À assembler</x:v>
+        <x:v>Archivé Drive</x:v>
       </x:c>
       <x:c r="I239" s="24" t="str">
-        <x:v>Référence</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="J239" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="K239" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="L239" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="M239" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="N239" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="O239" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="P239" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="Q239" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="R239" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="S239" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="T239" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="U239" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="V239" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="W239" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="X239" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="Y239" s="24" t="str">
         <x:v>Non consignée</x:v>
@@ -21994,13 +21994,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA239" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB239" s="21" t="str">
-        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
+        <x:v>b17117db72da867328bfee7e7b5ac7c17acc0aab</x:v>
       </x:c>
       <x:c r="AC239" s="21" t="str">
-        <x:v>À intégrer</x:v>
+        <x:v>En cours</x:v>
       </x:c>
     </x:row>
     <x:row r="240" ht="40" customHeight="1">
@@ -22287,69 +22287,69 @@
         <x:v>233</x:v>
       </x:c>
       <x:c r="D243" s="24" t="str">
-        <x:v>À planifier</x:v>
+        <x:v>Lot 12</x:v>
       </x:c>
       <x:c r="E243" s="25" t="str">
         <x:v>Animaux</x:v>
       </x:c>
       <x:c r="F243" s="24" t="str">
         <x:f>IF(AND(G243=8,COUNTIF(Q243:V243,"Atlas")=6),"Intégré","À faire")</x:f>
-        <x:v>À faire</x:v>
+        <x:v>Intégré</x:v>
       </x:c>
       <x:c r="G243" s="27" t="n">
         <x:f>COUNTIF(I243:P243,"Présent")</x:f>
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H243" s="24" t="str">
-        <x:v>À assembler</x:v>
+        <x:v>Archivé Drive</x:v>
       </x:c>
       <x:c r="I243" s="24" t="str">
-        <x:v>Référence</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="J243" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="K243" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="L243" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="M243" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="N243" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="O243" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="P243" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="Q243" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="R243" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="S243" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="T243" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="U243" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="V243" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="W243" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="X243" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="Y243" s="24" t="str">
         <x:v>Non consignée</x:v>
@@ -22358,13 +22358,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA243" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB243" s="21" t="str">
-        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
+        <x:v>b17117db72da867328bfee7e7b5ac7c17acc0aab</x:v>
       </x:c>
       <x:c r="AC243" s="21" t="str">
-        <x:v>À intégrer</x:v>
+        <x:v>En cours</x:v>
       </x:c>
     </x:row>
     <x:row r="244" ht="40" customHeight="1">
@@ -22560,69 +22560,69 @@
         <x:v>236</x:v>
       </x:c>
       <x:c r="D246" s="24" t="str">
-        <x:v>À planifier</x:v>
+        <x:v>Lot 12</x:v>
       </x:c>
       <x:c r="E246" s="25" t="str">
         <x:v>Animaux</x:v>
       </x:c>
       <x:c r="F246" s="24" t="str">
         <x:f>IF(AND(G246=8,COUNTIF(Q246:V246,"Atlas")=6),"Intégré","À faire")</x:f>
-        <x:v>À faire</x:v>
+        <x:v>Intégré</x:v>
       </x:c>
       <x:c r="G246" s="27" t="n">
         <x:f>COUNTIF(I246:P246,"Présent")</x:f>
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H246" s="24" t="str">
-        <x:v>À assembler</x:v>
+        <x:v>Archivé Drive</x:v>
       </x:c>
       <x:c r="I246" s="24" t="str">
-        <x:v>Référence</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="J246" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="K246" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="L246" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="M246" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="N246" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="O246" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="P246" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="Q246" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="R246" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="S246" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="T246" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="U246" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="V246" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="W246" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="X246" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="Y246" s="24" t="str">
         <x:v>Non consignée</x:v>
@@ -22631,13 +22631,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA246" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB246" s="21" t="str">
-        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
+        <x:v>b17117db72da867328bfee7e7b5ac7c17acc0aab</x:v>
       </x:c>
       <x:c r="AC246" s="21" t="str">
-        <x:v>À intégrer</x:v>
+        <x:v>En cours</x:v>
       </x:c>
     </x:row>
     <x:row r="247" ht="40" customHeight="1">
@@ -23094,7 +23094,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc86cc9929d6b4791"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8a2930917a3348ef"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Qualify lot 13 and refresh Excel CSV at 230 complete packs
</commit_message>
<xml_diff>
--- a/doc_web_interne/docs/suivi-symboles/suivi-240-symboles-6-langues.xlsx
+++ b/doc_web_interne/docs/suivi-symboles/suivi-240-symboles-6-langues.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Suivi symboles" sheetId="1" r:id="R8d12d01cd7514264"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Suivi symboles" sheetId="1" r:id="R92a6341196e445d8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -811,7 +811,7 @@
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="7" t="str">
-        <x:v>Lot 12 en branche : 25 couvertures conservées, 175 nouveaux PNG. Preuves antérieures inchangées conservées.</x:v>
+        <x:v>Lot 13 en branche : 29 couvertures conservées, 211 nouveaux PNG. Preuves antérieures inchangées conservées.</x:v>
       </x:c>
       <x:c r="B3" s="7"/>
       <x:c r="C3" s="7"/>
@@ -848,21 +848,21 @@
       </x:c>
       <x:c r="B4" s="9" t="n">
         <x:f>COUNTIF(F11:F250,"Intégré")</x:f>
-        <x:v>200</x:v>
+        <x:v>230</x:v>
       </x:c>
       <x:c r="C4" s="3" t="str">
         <x:v>Packs à terminer</x:v>
       </x:c>
       <x:c r="D4" s="9" t="n">
         <x:f>COUNTA(B11:B250)-B4</x:f>
-        <x:v>40</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="E4" s="3" t="str">
         <x:v>Pages avec pack</x:v>
       </x:c>
       <x:c r="F4" s="9" t="n">
         <x:f>COUNTIF(Q11:V250,"Atlas")</x:f>
-        <x:v>1200</x:v>
+        <x:v>1380</x:v>
       </x:c>
       <x:c r="G4" s="3" t="str">
         <x:v>Pages web</x:v>
@@ -899,14 +899,14 @@
       </x:c>
       <x:c r="B5" s="9" t="n">
         <x:f>COUNTIF(W11:W250,"6/6 actuelles")</x:f>
-        <x:v>200</x:v>
+        <x:v>230</x:v>
       </x:c>
       <x:c r="C5" s="3" t="str">
         <x:v>QA 2560 px</x:v>
       </x:c>
       <x:c r="D5" s="9" t="n">
         <x:f>COUNTIF(X11:X250,"6/6 actuelles")</x:f>
-        <x:v>200</x:v>
+        <x:v>230</x:v>
       </x:c>
       <x:c r="E5" s="3" t="str">
         <x:v>Accord Thanh</x:v>
@@ -980,7 +980,7 @@
     </x:row>
     <x:row r="7" ht="20" customHeight="1">
       <x:c r="A7" s="7" t="str">
-        <x:v>200 packs ; 40 à compléter. Cadre commun : 1 440 pages. Publication antérieure conservée dans les reçus.</x:v>
+        <x:v>230 packs ; 10 à compléter. Cadre commun : 1 440 pages. Publication antérieure conservée dans les reçus.</x:v>
       </x:c>
       <x:c r="B7" s="7"/>
       <x:c r="C7" s="7"/>
@@ -1013,7 +1013,7 @@
     </x:row>
     <x:row r="8" ht="20" customHeight="1">
       <x:c r="A8" s="7" t="str">
-        <x:v>Source : rapport canonique du 20/10/2026, empreinte 42ee542429cbc3ed. Révision : b17117db72da867328bfee7e7b5ac7c17acc0aab</x:v>
+        <x:v>Source : rapport canonique actuel, empreinte b6be04037927f2da. Révision : e03821783020a61aeaaa58d22886e2118781efaa</x:v>
       </x:c>
       <x:c r="B8" s="7"/>
       <x:c r="C8" s="7"/>
@@ -3359,69 +3359,69 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="D35" s="24" t="str">
-        <x:v>Lot 04 proposé</x:v>
+        <x:v>Lot 13</x:v>
       </x:c>
       <x:c r="E35" s="25" t="str">
         <x:v>Corps</x:v>
       </x:c>
       <x:c r="F35" s="24" t="str">
         <x:f>IF(AND(G35=8,COUNTIF(Q35:V35,"Atlas")=6),"Intégré","À faire")</x:f>
-        <x:v>À faire</x:v>
+        <x:v>Intégré</x:v>
       </x:c>
       <x:c r="G35" s="27" t="n">
         <x:f>COUNTIF(I35:P35,"Présent")</x:f>
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H35" s="24" t="str">
-        <x:v>À assembler</x:v>
+        <x:v>Archivé Drive</x:v>
       </x:c>
       <x:c r="I35" s="24" t="str">
-        <x:v>Référence</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="J35" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="K35" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="L35" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="M35" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="N35" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="O35" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="P35" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="Q35" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="R35" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="S35" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="T35" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="U35" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="V35" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="W35" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="X35" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="Y35" s="24" t="str">
         <x:v>Non consignée</x:v>
@@ -3430,13 +3430,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA35" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB35" s="21" t="str">
-        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
+        <x:v>e03821783020a61aeaaa58d22886e2118781efaa</x:v>
       </x:c>
       <x:c r="AC35" s="21" t="str">
-        <x:v>À intégrer</x:v>
+        <x:v>En cours</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="40" customHeight="1">
@@ -10275,69 +10275,69 @@
         <x:v>101</x:v>
       </x:c>
       <x:c r="D111" s="24" t="str">
-        <x:v>À planifier</x:v>
+        <x:v>Lot 13</x:v>
       </x:c>
       <x:c r="E111" s="25" t="str">
         <x:v>Personnes</x:v>
       </x:c>
       <x:c r="F111" s="24" t="str">
         <x:f>IF(AND(G111=8,COUNTIF(Q111:V111,"Atlas")=6),"Intégré","À faire")</x:f>
-        <x:v>À faire</x:v>
+        <x:v>Intégré</x:v>
       </x:c>
       <x:c r="G111" s="27" t="n">
         <x:f>COUNTIF(I111:P111,"Présent")</x:f>
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H111" s="24" t="str">
-        <x:v>À assembler</x:v>
+        <x:v>Archivé Drive</x:v>
       </x:c>
       <x:c r="I111" s="24" t="str">
-        <x:v>Référence</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="J111" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="K111" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="L111" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="M111" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="N111" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="O111" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="P111" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="Q111" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="R111" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="S111" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="T111" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="U111" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="V111" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="W111" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="X111" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="Y111" s="24" t="str">
         <x:v>Non consignée</x:v>
@@ -10346,13 +10346,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA111" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB111" s="21" t="str">
-        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
+        <x:v>e03821783020a61aeaaa58d22886e2118781efaa</x:v>
       </x:c>
       <x:c r="AC111" s="21" t="str">
-        <x:v>À intégrer</x:v>
+        <x:v>En cours</x:v>
       </x:c>
     </x:row>
     <x:row r="112" ht="40" customHeight="1">
@@ -10548,69 +10548,69 @@
         <x:v>104</x:v>
       </x:c>
       <x:c r="D114" s="24" t="str">
-        <x:v>À planifier</x:v>
+        <x:v>Lot 13</x:v>
       </x:c>
       <x:c r="E114" s="25" t="str">
         <x:v>Animaux</x:v>
       </x:c>
       <x:c r="F114" s="24" t="str">
         <x:f>IF(AND(G114=8,COUNTIF(Q114:V114,"Atlas")=6),"Intégré","À faire")</x:f>
-        <x:v>À faire</x:v>
+        <x:v>Intégré</x:v>
       </x:c>
       <x:c r="G114" s="27" t="n">
         <x:f>COUNTIF(I114:P114,"Présent")</x:f>
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H114" s="24" t="str">
-        <x:v>À assembler</x:v>
+        <x:v>Archivé Drive</x:v>
       </x:c>
       <x:c r="I114" s="24" t="str">
-        <x:v>Référence</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="J114" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="K114" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="L114" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="M114" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="N114" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="O114" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="P114" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="Q114" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="R114" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="S114" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="T114" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="U114" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="V114" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="W114" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="X114" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="Y114" s="24" t="str">
         <x:v>Non consignée</x:v>
@@ -10619,13 +10619,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA114" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB114" s="21" t="str">
-        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
+        <x:v>e03821783020a61aeaaa58d22886e2118781efaa</x:v>
       </x:c>
       <x:c r="AC114" s="21" t="str">
-        <x:v>À intégrer</x:v>
+        <x:v>En cours</x:v>
       </x:c>
     </x:row>
     <x:row r="115" ht="40" customHeight="1">
@@ -10821,69 +10821,69 @@
         <x:v>107</x:v>
       </x:c>
       <x:c r="D117" s="24" t="str">
-        <x:v>À planifier</x:v>
+        <x:v>Lot 13</x:v>
       </x:c>
       <x:c r="E117" s="25" t="str">
         <x:v>Animaux</x:v>
       </x:c>
       <x:c r="F117" s="24" t="str">
         <x:f>IF(AND(G117=8,COUNTIF(Q117:V117,"Atlas")=6),"Intégré","À faire")</x:f>
-        <x:v>À faire</x:v>
+        <x:v>Intégré</x:v>
       </x:c>
       <x:c r="G117" s="27" t="n">
         <x:f>COUNTIF(I117:P117,"Présent")</x:f>
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H117" s="24" t="str">
-        <x:v>À assembler</x:v>
+        <x:v>Archivé Drive</x:v>
       </x:c>
       <x:c r="I117" s="24" t="str">
-        <x:v>Référence</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="J117" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="K117" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="L117" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="M117" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="N117" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="O117" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="P117" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="Q117" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="R117" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="S117" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="T117" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="U117" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="V117" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="W117" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="X117" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="Y117" s="24" t="str">
         <x:v>Non consignée</x:v>
@@ -10892,13 +10892,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA117" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB117" s="21" t="str">
-        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
+        <x:v>e03821783020a61aeaaa58d22886e2118781efaa</x:v>
       </x:c>
       <x:c r="AC117" s="21" t="str">
-        <x:v>À intégrer</x:v>
+        <x:v>En cours</x:v>
       </x:c>
     </x:row>
     <x:row r="118" ht="40" customHeight="1">
@@ -11276,69 +11276,69 @@
         <x:v>112</x:v>
       </x:c>
       <x:c r="D122" s="24" t="str">
-        <x:v>À planifier</x:v>
+        <x:v>Lot 13</x:v>
       </x:c>
       <x:c r="E122" s="25" t="str">
         <x:v>Lieux</x:v>
       </x:c>
       <x:c r="F122" s="24" t="str">
         <x:f>IF(AND(G122=8,COUNTIF(Q122:V122,"Atlas")=6),"Intégré","À faire")</x:f>
-        <x:v>À faire</x:v>
+        <x:v>Intégré</x:v>
       </x:c>
       <x:c r="G122" s="27" t="n">
         <x:f>COUNTIF(I122:P122,"Présent")</x:f>
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H122" s="24" t="str">
-        <x:v>À assembler</x:v>
+        <x:v>Archivé Drive</x:v>
       </x:c>
       <x:c r="I122" s="24" t="str">
-        <x:v>Référence</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="J122" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="K122" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="L122" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="M122" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="N122" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="O122" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="P122" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="Q122" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="R122" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="S122" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="T122" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="U122" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="V122" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="W122" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="X122" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="Y122" s="24" t="str">
         <x:v>Non consignée</x:v>
@@ -11347,13 +11347,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA122" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB122" s="21" t="str">
-        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
+        <x:v>e03821783020a61aeaaa58d22886e2118781efaa</x:v>
       </x:c>
       <x:c r="AC122" s="21" t="str">
-        <x:v>À intégrer</x:v>
+        <x:v>En cours</x:v>
       </x:c>
     </x:row>
     <x:row r="123" ht="40" customHeight="1">
@@ -11458,69 +11458,69 @@
         <x:v>114</x:v>
       </x:c>
       <x:c r="D124" s="24" t="str">
-        <x:v>À planifier</x:v>
+        <x:v>Lot 13</x:v>
       </x:c>
       <x:c r="E124" s="25" t="str">
         <x:v>Animaux</x:v>
       </x:c>
       <x:c r="F124" s="24" t="str">
         <x:f>IF(AND(G124=8,COUNTIF(Q124:V124,"Atlas")=6),"Intégré","À faire")</x:f>
-        <x:v>À faire</x:v>
+        <x:v>Intégré</x:v>
       </x:c>
       <x:c r="G124" s="27" t="n">
         <x:f>COUNTIF(I124:P124,"Présent")</x:f>
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H124" s="24" t="str">
-        <x:v>À assembler</x:v>
+        <x:v>Archivé Drive</x:v>
       </x:c>
       <x:c r="I124" s="24" t="str">
-        <x:v>Référence</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="J124" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="K124" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="L124" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="M124" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="N124" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="O124" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="P124" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="Q124" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="R124" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="S124" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="T124" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="U124" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="V124" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="W124" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="X124" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="Y124" s="24" t="str">
         <x:v>Non consignée</x:v>
@@ -11529,13 +11529,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA124" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB124" s="21" t="str">
-        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
+        <x:v>e03821783020a61aeaaa58d22886e2118781efaa</x:v>
       </x:c>
       <x:c r="AC124" s="21" t="str">
-        <x:v>À intégrer</x:v>
+        <x:v>En cours</x:v>
       </x:c>
     </x:row>
     <x:row r="125" ht="40" customHeight="1">
@@ -12186,69 +12186,69 @@
         <x:v>122</x:v>
       </x:c>
       <x:c r="D132" s="24" t="str">
-        <x:v>À planifier</x:v>
+        <x:v>Lot 13</x:v>
       </x:c>
       <x:c r="E132" s="25" t="str">
         <x:v>Personnes</x:v>
       </x:c>
       <x:c r="F132" s="24" t="str">
         <x:f>IF(AND(G132=8,COUNTIF(Q132:V132,"Atlas")=6),"Intégré","À faire")</x:f>
-        <x:v>À faire</x:v>
+        <x:v>Intégré</x:v>
       </x:c>
       <x:c r="G132" s="27" t="n">
         <x:f>COUNTIF(I132:P132,"Présent")</x:f>
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H132" s="24" t="str">
-        <x:v>À assembler</x:v>
+        <x:v>Archivé Drive</x:v>
       </x:c>
       <x:c r="I132" s="24" t="str">
-        <x:v>Référence</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="J132" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="K132" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="L132" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="M132" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="N132" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="O132" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="P132" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="Q132" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="R132" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="S132" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="T132" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="U132" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="V132" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="W132" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="X132" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="Y132" s="24" t="str">
         <x:v>Non consignée</x:v>
@@ -12257,13 +12257,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA132" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB132" s="21" t="str">
-        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
+        <x:v>e03821783020a61aeaaa58d22886e2118781efaa</x:v>
       </x:c>
       <x:c r="AC132" s="21" t="str">
-        <x:v>À intégrer</x:v>
+        <x:v>En cours</x:v>
       </x:c>
     </x:row>
     <x:row r="133" ht="40" customHeight="1">
@@ -12550,69 +12550,69 @@
         <x:v>126</x:v>
       </x:c>
       <x:c r="D136" s="24" t="str">
-        <x:v>À planifier</x:v>
+        <x:v>Lot 13</x:v>
       </x:c>
       <x:c r="E136" s="25" t="str">
         <x:v>Actions</x:v>
       </x:c>
       <x:c r="F136" s="24" t="str">
         <x:f>IF(AND(G136=8,COUNTIF(Q136:V136,"Atlas")=6),"Intégré","À faire")</x:f>
-        <x:v>À faire</x:v>
+        <x:v>Intégré</x:v>
       </x:c>
       <x:c r="G136" s="27" t="n">
         <x:f>COUNTIF(I136:P136,"Présent")</x:f>
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H136" s="24" t="str">
-        <x:v>À assembler</x:v>
+        <x:v>Archivé Drive</x:v>
       </x:c>
       <x:c r="I136" s="24" t="str">
-        <x:v>Référence</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="J136" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="K136" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="L136" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="M136" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="N136" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="O136" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="P136" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="Q136" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="R136" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="S136" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="T136" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="U136" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="V136" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="W136" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="X136" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="Y136" s="24" t="str">
         <x:v>Non consignée</x:v>
@@ -12621,13 +12621,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA136" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB136" s="21" t="str">
-        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
+        <x:v>e03821783020a61aeaaa58d22886e2118781efaa</x:v>
       </x:c>
       <x:c r="AC136" s="21" t="str">
-        <x:v>À intégrer</x:v>
+        <x:v>En cours</x:v>
       </x:c>
     </x:row>
     <x:row r="137" ht="40" customHeight="1">
@@ -13096,69 +13096,69 @@
         <x:v>132</x:v>
       </x:c>
       <x:c r="D142" s="24" t="str">
-        <x:v>À planifier</x:v>
+        <x:v>Lot 13</x:v>
       </x:c>
       <x:c r="E142" s="25" t="str">
         <x:v>Lieux</x:v>
       </x:c>
       <x:c r="F142" s="24" t="str">
         <x:f>IF(AND(G142=8,COUNTIF(Q142:V142,"Atlas")=6),"Intégré","À faire")</x:f>
-        <x:v>À faire</x:v>
+        <x:v>Intégré</x:v>
       </x:c>
       <x:c r="G142" s="27" t="n">
         <x:f>COUNTIF(I142:P142,"Présent")</x:f>
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H142" s="24" t="str">
-        <x:v>À assembler</x:v>
+        <x:v>Archivé Drive</x:v>
       </x:c>
       <x:c r="I142" s="24" t="str">
-        <x:v>Référence</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="J142" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="K142" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="L142" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="M142" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="N142" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="O142" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="P142" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="Q142" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="R142" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="S142" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="T142" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="U142" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="V142" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="W142" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="X142" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="Y142" s="24" t="str">
         <x:v>Non consignée</x:v>
@@ -13167,13 +13167,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA142" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB142" s="21" t="str">
-        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
+        <x:v>e03821783020a61aeaaa58d22886e2118781efaa</x:v>
       </x:c>
       <x:c r="AC142" s="21" t="str">
-        <x:v>À intégrer</x:v>
+        <x:v>En cours</x:v>
       </x:c>
     </x:row>
     <x:row r="143" ht="40" customHeight="1">
@@ -13278,69 +13278,69 @@
         <x:v>134</x:v>
       </x:c>
       <x:c r="D144" s="24" t="str">
-        <x:v>À planifier</x:v>
+        <x:v>Lot 13</x:v>
       </x:c>
       <x:c r="E144" s="25" t="str">
         <x:v>Actions</x:v>
       </x:c>
       <x:c r="F144" s="24" t="str">
         <x:f>IF(AND(G144=8,COUNTIF(Q144:V144,"Atlas")=6),"Intégré","À faire")</x:f>
-        <x:v>À faire</x:v>
+        <x:v>Intégré</x:v>
       </x:c>
       <x:c r="G144" s="27" t="n">
         <x:f>COUNTIF(I144:P144,"Présent")</x:f>
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H144" s="24" t="str">
-        <x:v>À assembler</x:v>
+        <x:v>Archivé Drive</x:v>
       </x:c>
       <x:c r="I144" s="24" t="str">
-        <x:v>Référence</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="J144" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="K144" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="L144" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="M144" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="N144" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="O144" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="P144" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="Q144" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="R144" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="S144" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="T144" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="U144" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="V144" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="W144" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="X144" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="Y144" s="24" t="str">
         <x:v>Non consignée</x:v>
@@ -13349,13 +13349,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA144" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB144" s="21" t="str">
-        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
+        <x:v>e03821783020a61aeaaa58d22886e2118781efaa</x:v>
       </x:c>
       <x:c r="AC144" s="21" t="str">
-        <x:v>À intégrer</x:v>
+        <x:v>En cours</x:v>
       </x:c>
     </x:row>
     <x:row r="145" ht="40" customHeight="1">
@@ -13460,69 +13460,69 @@
         <x:v>136</x:v>
       </x:c>
       <x:c r="D146" s="24" t="str">
-        <x:v>À planifier</x:v>
+        <x:v>Lot 13</x:v>
       </x:c>
       <x:c r="E146" s="25" t="str">
         <x:v>Actions</x:v>
       </x:c>
       <x:c r="F146" s="24" t="str">
         <x:f>IF(AND(G146=8,COUNTIF(Q146:V146,"Atlas")=6),"Intégré","À faire")</x:f>
-        <x:v>À faire</x:v>
+        <x:v>Intégré</x:v>
       </x:c>
       <x:c r="G146" s="27" t="n">
         <x:f>COUNTIF(I146:P146,"Présent")</x:f>
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H146" s="24" t="str">
-        <x:v>À assembler</x:v>
+        <x:v>Archivé Drive</x:v>
       </x:c>
       <x:c r="I146" s="24" t="str">
-        <x:v>Référence</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="J146" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="K146" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="L146" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="M146" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="N146" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="O146" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="P146" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="Q146" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="R146" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="S146" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="T146" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="U146" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="V146" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="W146" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="X146" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="Y146" s="24" t="str">
         <x:v>Non consignée</x:v>
@@ -13531,13 +13531,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA146" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB146" s="21" t="str">
-        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
+        <x:v>e03821783020a61aeaaa58d22886e2118781efaa</x:v>
       </x:c>
       <x:c r="AC146" s="21" t="str">
-        <x:v>À intégrer</x:v>
+        <x:v>En cours</x:v>
       </x:c>
     </x:row>
     <x:row r="147" ht="40" customHeight="1">
@@ -13642,69 +13642,69 @@
         <x:v>138</x:v>
       </x:c>
       <x:c r="D148" s="24" t="str">
-        <x:v>À planifier</x:v>
+        <x:v>Lot 13</x:v>
       </x:c>
       <x:c r="E148" s="25" t="str">
         <x:v>Actions</x:v>
       </x:c>
       <x:c r="F148" s="24" t="str">
         <x:f>IF(AND(G148=8,COUNTIF(Q148:V148,"Atlas")=6),"Intégré","À faire")</x:f>
-        <x:v>À faire</x:v>
+        <x:v>Intégré</x:v>
       </x:c>
       <x:c r="G148" s="27" t="n">
         <x:f>COUNTIF(I148:P148,"Présent")</x:f>
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H148" s="24" t="str">
-        <x:v>À assembler</x:v>
+        <x:v>Archivé Drive</x:v>
       </x:c>
       <x:c r="I148" s="24" t="str">
-        <x:v>Référence</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="J148" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="K148" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="L148" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="M148" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="N148" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="O148" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="P148" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="Q148" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="R148" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="S148" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="T148" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="U148" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="V148" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="W148" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="X148" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="Y148" s="24" t="str">
         <x:v>Non consignée</x:v>
@@ -13713,13 +13713,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA148" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB148" s="21" t="str">
-        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
+        <x:v>e03821783020a61aeaaa58d22886e2118781efaa</x:v>
       </x:c>
       <x:c r="AC148" s="21" t="str">
-        <x:v>À intégrer</x:v>
+        <x:v>En cours</x:v>
       </x:c>
     </x:row>
     <x:row r="149" ht="40" customHeight="1">
@@ -14097,69 +14097,69 @@
         <x:v>143</x:v>
       </x:c>
       <x:c r="D153" s="24" t="str">
-        <x:v>À planifier</x:v>
+        <x:v>Lot 13</x:v>
       </x:c>
       <x:c r="E153" s="25" t="str">
         <x:v>Personnes</x:v>
       </x:c>
       <x:c r="F153" s="24" t="str">
         <x:f>IF(AND(G153=8,COUNTIF(Q153:V153,"Atlas")=6),"Intégré","À faire")</x:f>
-        <x:v>À faire</x:v>
+        <x:v>Intégré</x:v>
       </x:c>
       <x:c r="G153" s="27" t="n">
         <x:f>COUNTIF(I153:P153,"Présent")</x:f>
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H153" s="24" t="str">
-        <x:v>À assembler</x:v>
+        <x:v>Archivé Drive</x:v>
       </x:c>
       <x:c r="I153" s="24" t="str">
-        <x:v>Référence</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="J153" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="K153" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="L153" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="M153" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="N153" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="O153" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="P153" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="Q153" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="R153" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="S153" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="T153" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="U153" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="V153" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="W153" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="X153" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="Y153" s="24" t="str">
         <x:v>Non consignée</x:v>
@@ -14168,13 +14168,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA153" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB153" s="21" t="str">
-        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
+        <x:v>e03821783020a61aeaaa58d22886e2118781efaa</x:v>
       </x:c>
       <x:c r="AC153" s="21" t="str">
-        <x:v>À intégrer</x:v>
+        <x:v>En cours</x:v>
       </x:c>
     </x:row>
     <x:row r="154" ht="40" customHeight="1">
@@ -15098,69 +15098,69 @@
         <x:v>154</x:v>
       </x:c>
       <x:c r="D164" s="24" t="str">
-        <x:v>À planifier</x:v>
+        <x:v>Lot 13</x:v>
       </x:c>
       <x:c r="E164" s="25" t="str">
         <x:v>Animaux</x:v>
       </x:c>
       <x:c r="F164" s="24" t="str">
         <x:f>IF(AND(G164=8,COUNTIF(Q164:V164,"Atlas")=6),"Intégré","À faire")</x:f>
-        <x:v>À faire</x:v>
+        <x:v>Intégré</x:v>
       </x:c>
       <x:c r="G164" s="27" t="n">
         <x:f>COUNTIF(I164:P164,"Présent")</x:f>
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H164" s="24" t="str">
-        <x:v>À assembler</x:v>
+        <x:v>Archivé Drive</x:v>
       </x:c>
       <x:c r="I164" s="24" t="str">
-        <x:v>Référence</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="J164" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="K164" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="L164" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="M164" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="N164" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="O164" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="P164" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="Q164" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="R164" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="S164" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="T164" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="U164" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="V164" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="W164" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="X164" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="Y164" s="24" t="str">
         <x:v>Non consignée</x:v>
@@ -15169,13 +15169,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA164" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB164" s="21" t="str">
-        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
+        <x:v>e03821783020a61aeaaa58d22886e2118781efaa</x:v>
       </x:c>
       <x:c r="AC164" s="21" t="str">
-        <x:v>À intégrer</x:v>
+        <x:v>En cours</x:v>
       </x:c>
     </x:row>
     <x:row r="165" ht="40" customHeight="1">
@@ -15189,69 +15189,69 @@
         <x:v>155</x:v>
       </x:c>
       <x:c r="D165" s="24" t="str">
-        <x:v>À planifier</x:v>
+        <x:v>Lot 13</x:v>
       </x:c>
       <x:c r="E165" s="25" t="str">
         <x:v>Actions</x:v>
       </x:c>
       <x:c r="F165" s="24" t="str">
         <x:f>IF(AND(G165=8,COUNTIF(Q165:V165,"Atlas")=6),"Intégré","À faire")</x:f>
-        <x:v>À faire</x:v>
+        <x:v>Intégré</x:v>
       </x:c>
       <x:c r="G165" s="27" t="n">
         <x:f>COUNTIF(I165:P165,"Présent")</x:f>
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H165" s="24" t="str">
-        <x:v>À assembler</x:v>
+        <x:v>Archivé Drive</x:v>
       </x:c>
       <x:c r="I165" s="24" t="str">
-        <x:v>Référence</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="J165" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="K165" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="L165" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="M165" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="N165" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="O165" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="P165" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="Q165" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="R165" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="S165" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="T165" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="U165" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="V165" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="W165" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="X165" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="Y165" s="24" t="str">
         <x:v>Non consignée</x:v>
@@ -15260,13 +15260,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA165" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB165" s="21" t="str">
-        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
+        <x:v>e03821783020a61aeaaa58d22886e2118781efaa</x:v>
       </x:c>
       <x:c r="AC165" s="21" t="str">
-        <x:v>À intégrer</x:v>
+        <x:v>En cours</x:v>
       </x:c>
     </x:row>
     <x:row r="166" ht="40" customHeight="1">
@@ -15826,69 +15826,69 @@
         <x:v>162</x:v>
       </x:c>
       <x:c r="D172" s="24" t="str">
-        <x:v>À planifier</x:v>
+        <x:v>Lot 13</x:v>
       </x:c>
       <x:c r="E172" s="25" t="str">
         <x:v>Actions</x:v>
       </x:c>
       <x:c r="F172" s="24" t="str">
         <x:f>IF(AND(G172=8,COUNTIF(Q172:V172,"Atlas")=6),"Intégré","À faire")</x:f>
-        <x:v>À faire</x:v>
+        <x:v>Intégré</x:v>
       </x:c>
       <x:c r="G172" s="27" t="n">
         <x:f>COUNTIF(I172:P172,"Présent")</x:f>
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H172" s="24" t="str">
-        <x:v>À assembler</x:v>
+        <x:v>Archivé Drive</x:v>
       </x:c>
       <x:c r="I172" s="24" t="str">
-        <x:v>Référence</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="J172" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="K172" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="L172" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="M172" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="N172" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="O172" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="P172" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="Q172" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="R172" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="S172" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="T172" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="U172" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="V172" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="W172" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="X172" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="Y172" s="24" t="str">
         <x:v>Non consignée</x:v>
@@ -15897,13 +15897,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA172" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB172" s="21" t="str">
-        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
+        <x:v>e03821783020a61aeaaa58d22886e2118781efaa</x:v>
       </x:c>
       <x:c r="AC172" s="21" t="str">
-        <x:v>À intégrer</x:v>
+        <x:v>En cours</x:v>
       </x:c>
     </x:row>
     <x:row r="173" ht="40" customHeight="1">
@@ -16372,69 +16372,69 @@
         <x:v>168</x:v>
       </x:c>
       <x:c r="D178" s="24" t="str">
-        <x:v>À planifier</x:v>
+        <x:v>Lot 13</x:v>
       </x:c>
       <x:c r="E178" s="25" t="str">
         <x:v>Animaux</x:v>
       </x:c>
       <x:c r="F178" s="24" t="str">
         <x:f>IF(AND(G178=8,COUNTIF(Q178:V178,"Atlas")=6),"Intégré","À faire")</x:f>
-        <x:v>À faire</x:v>
+        <x:v>Intégré</x:v>
       </x:c>
       <x:c r="G178" s="27" t="n">
         <x:f>COUNTIF(I178:P178,"Présent")</x:f>
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H178" s="24" t="str">
-        <x:v>À assembler</x:v>
+        <x:v>Archivé Drive</x:v>
       </x:c>
       <x:c r="I178" s="24" t="str">
-        <x:v>Référence</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="J178" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="K178" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="L178" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="M178" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="N178" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="O178" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="P178" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="Q178" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="R178" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="S178" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="T178" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="U178" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="V178" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="W178" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="X178" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="Y178" s="24" t="str">
         <x:v>Non consignée</x:v>
@@ -16443,13 +16443,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA178" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB178" s="21" t="str">
-        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
+        <x:v>e03821783020a61aeaaa58d22886e2118781efaa</x:v>
       </x:c>
       <x:c r="AC178" s="21" t="str">
-        <x:v>À intégrer</x:v>
+        <x:v>En cours</x:v>
       </x:c>
     </x:row>
     <x:row r="179" ht="40" customHeight="1">
@@ -16827,69 +16827,69 @@
         <x:v>173</x:v>
       </x:c>
       <x:c r="D183" s="24" t="str">
-        <x:v>À planifier</x:v>
+        <x:v>Lot 13</x:v>
       </x:c>
       <x:c r="E183" s="25" t="str">
         <x:v>Actions</x:v>
       </x:c>
       <x:c r="F183" s="24" t="str">
         <x:f>IF(AND(G183=8,COUNTIF(Q183:V183,"Atlas")=6),"Intégré","À faire")</x:f>
-        <x:v>À faire</x:v>
+        <x:v>Intégré</x:v>
       </x:c>
       <x:c r="G183" s="27" t="n">
         <x:f>COUNTIF(I183:P183,"Présent")</x:f>
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H183" s="24" t="str">
-        <x:v>À assembler</x:v>
+        <x:v>Archivé Drive</x:v>
       </x:c>
       <x:c r="I183" s="24" t="str">
-        <x:v>Référence</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="J183" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="K183" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="L183" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="M183" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="N183" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="O183" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="P183" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="Q183" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="R183" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="S183" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="T183" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="U183" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="V183" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="W183" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="X183" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="Y183" s="24" t="str">
         <x:v>Non consignée</x:v>
@@ -16898,13 +16898,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA183" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB183" s="21" t="str">
-        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
+        <x:v>e03821783020a61aeaaa58d22886e2118781efaa</x:v>
       </x:c>
       <x:c r="AC183" s="21" t="str">
-        <x:v>À intégrer</x:v>
+        <x:v>En cours</x:v>
       </x:c>
     </x:row>
     <x:row r="184" ht="40" customHeight="1">
@@ -18556,69 +18556,69 @@
         <x:v>192</x:v>
       </x:c>
       <x:c r="D202" s="24" t="str">
-        <x:v>À planifier</x:v>
+        <x:v>Lot 13</x:v>
       </x:c>
       <x:c r="E202" s="25" t="str">
         <x:v>Personnes</x:v>
       </x:c>
       <x:c r="F202" s="24" t="str">
         <x:f>IF(AND(G202=8,COUNTIF(Q202:V202,"Atlas")=6),"Intégré","À faire")</x:f>
-        <x:v>À faire</x:v>
+        <x:v>Intégré</x:v>
       </x:c>
       <x:c r="G202" s="27" t="n">
         <x:f>COUNTIF(I202:P202,"Présent")</x:f>
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H202" s="24" t="str">
-        <x:v>À assembler</x:v>
+        <x:v>Archivé Drive</x:v>
       </x:c>
       <x:c r="I202" s="24" t="str">
-        <x:v>Référence</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="J202" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="K202" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="L202" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="M202" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="N202" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="O202" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="P202" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="Q202" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="R202" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="S202" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="T202" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="U202" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="V202" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="W202" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="X202" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="Y202" s="24" t="str">
         <x:v>Non consignée</x:v>
@@ -18627,13 +18627,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA202" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB202" s="21" t="str">
-        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
+        <x:v>e03821783020a61aeaaa58d22886e2118781efaa</x:v>
       </x:c>
       <x:c r="AC202" s="21" t="str">
-        <x:v>À intégrer</x:v>
+        <x:v>En cours</x:v>
       </x:c>
     </x:row>
     <x:row r="203" ht="40" customHeight="1">
@@ -18920,69 +18920,69 @@
         <x:v>196</x:v>
       </x:c>
       <x:c r="D206" s="24" t="str">
-        <x:v>À planifier</x:v>
+        <x:v>Lot 13</x:v>
       </x:c>
       <x:c r="E206" s="25" t="str">
         <x:v>Lieux</x:v>
       </x:c>
       <x:c r="F206" s="24" t="str">
         <x:f>IF(AND(G206=8,COUNTIF(Q206:V206,"Atlas")=6),"Intégré","À faire")</x:f>
-        <x:v>À faire</x:v>
+        <x:v>Intégré</x:v>
       </x:c>
       <x:c r="G206" s="27" t="n">
         <x:f>COUNTIF(I206:P206,"Présent")</x:f>
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H206" s="24" t="str">
-        <x:v>À assembler</x:v>
+        <x:v>Archivé Drive</x:v>
       </x:c>
       <x:c r="I206" s="24" t="str">
-        <x:v>Référence</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="J206" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="K206" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="L206" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="M206" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="N206" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="O206" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="P206" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="Q206" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="R206" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="S206" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="T206" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="U206" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="V206" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="W206" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="X206" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="Y206" s="24" t="str">
         <x:v>Non consignée</x:v>
@@ -18991,13 +18991,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA206" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB206" s="21" t="str">
-        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
+        <x:v>e03821783020a61aeaaa58d22886e2118781efaa</x:v>
       </x:c>
       <x:c r="AC206" s="21" t="str">
-        <x:v>À intégrer</x:v>
+        <x:v>En cours</x:v>
       </x:c>
     </x:row>
     <x:row r="207" ht="40" customHeight="1">
@@ -19011,69 +19011,69 @@
         <x:v>197</x:v>
       </x:c>
       <x:c r="D207" s="24" t="str">
-        <x:v>À planifier</x:v>
+        <x:v>Lot 13</x:v>
       </x:c>
       <x:c r="E207" s="25" t="str">
         <x:v>Lieux</x:v>
       </x:c>
       <x:c r="F207" s="24" t="str">
         <x:f>IF(AND(G207=8,COUNTIF(Q207:V207,"Atlas")=6),"Intégré","À faire")</x:f>
-        <x:v>À faire</x:v>
+        <x:v>Intégré</x:v>
       </x:c>
       <x:c r="G207" s="27" t="n">
         <x:f>COUNTIF(I207:P207,"Présent")</x:f>
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H207" s="24" t="str">
-        <x:v>À assembler</x:v>
+        <x:v>Archivé Drive</x:v>
       </x:c>
       <x:c r="I207" s="24" t="str">
-        <x:v>Référence</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="J207" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="K207" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="L207" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="M207" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="N207" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="O207" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="P207" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="Q207" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="R207" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="S207" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="T207" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="U207" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="V207" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="W207" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="X207" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="Y207" s="24" t="str">
         <x:v>Non consignée</x:v>
@@ -19082,13 +19082,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA207" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB207" s="21" t="str">
-        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
+        <x:v>e03821783020a61aeaaa58d22886e2118781efaa</x:v>
       </x:c>
       <x:c r="AC207" s="21" t="str">
-        <x:v>À intégrer</x:v>
+        <x:v>En cours</x:v>
       </x:c>
     </x:row>
     <x:row r="208" ht="40" customHeight="1">
@@ -19648,69 +19648,69 @@
         <x:v>204</x:v>
       </x:c>
       <x:c r="D214" s="24" t="str">
-        <x:v>À planifier</x:v>
+        <x:v>Lot 13</x:v>
       </x:c>
       <x:c r="E214" s="25" t="str">
         <x:v>Animaux</x:v>
       </x:c>
       <x:c r="F214" s="24" t="str">
         <x:f>IF(AND(G214=8,COUNTIF(Q214:V214,"Atlas")=6),"Intégré","À faire")</x:f>
-        <x:v>À faire</x:v>
+        <x:v>Intégré</x:v>
       </x:c>
       <x:c r="G214" s="27" t="n">
         <x:f>COUNTIF(I214:P214,"Présent")</x:f>
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H214" s="24" t="str">
-        <x:v>À assembler</x:v>
+        <x:v>Archivé Drive</x:v>
       </x:c>
       <x:c r="I214" s="24" t="str">
-        <x:v>Référence</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="J214" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="K214" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="L214" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="M214" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="N214" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="O214" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="P214" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="Q214" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="R214" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="S214" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="T214" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="U214" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="V214" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="W214" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="X214" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="Y214" s="24" t="str">
         <x:v>Non consignée</x:v>
@@ -19719,13 +19719,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA214" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB214" s="21" t="str">
-        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
+        <x:v>e03821783020a61aeaaa58d22886e2118781efaa</x:v>
       </x:c>
       <x:c r="AC214" s="21" t="str">
-        <x:v>À intégrer</x:v>
+        <x:v>En cours</x:v>
       </x:c>
     </x:row>
     <x:row r="215" ht="40" customHeight="1">
@@ -20831,69 +20831,69 @@
         <x:v>217</x:v>
       </x:c>
       <x:c r="D227" s="24" t="str">
-        <x:v>À planifier</x:v>
+        <x:v>Lot 13</x:v>
       </x:c>
       <x:c r="E227" s="25" t="str">
         <x:v>Animaux</x:v>
       </x:c>
       <x:c r="F227" s="24" t="str">
         <x:f>IF(AND(G227=8,COUNTIF(Q227:V227,"Atlas")=6),"Intégré","À faire")</x:f>
-        <x:v>À faire</x:v>
+        <x:v>Intégré</x:v>
       </x:c>
       <x:c r="G227" s="27" t="n">
         <x:f>COUNTIF(I227:P227,"Présent")</x:f>
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H227" s="24" t="str">
-        <x:v>À assembler</x:v>
+        <x:v>Archivé Drive</x:v>
       </x:c>
       <x:c r="I227" s="24" t="str">
-        <x:v>Référence</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="J227" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="K227" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="L227" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="M227" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="N227" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="O227" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="P227" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="Q227" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="R227" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="S227" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="T227" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="U227" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="V227" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="W227" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="X227" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="Y227" s="24" t="str">
         <x:v>Non consignée</x:v>
@@ -20902,13 +20902,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA227" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB227" s="21" t="str">
-        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
+        <x:v>e03821783020a61aeaaa58d22886e2118781efaa</x:v>
       </x:c>
       <x:c r="AC227" s="21" t="str">
-        <x:v>À intégrer</x:v>
+        <x:v>En cours</x:v>
       </x:c>
     </x:row>
     <x:row r="228" ht="40" customHeight="1">
@@ -20922,69 +20922,69 @@
         <x:v>218</x:v>
       </x:c>
       <x:c r="D228" s="24" t="str">
-        <x:v>À planifier</x:v>
+        <x:v>Lot 13</x:v>
       </x:c>
       <x:c r="E228" s="25" t="str">
         <x:v>Actions</x:v>
       </x:c>
       <x:c r="F228" s="24" t="str">
         <x:f>IF(AND(G228=8,COUNTIF(Q228:V228,"Atlas")=6),"Intégré","À faire")</x:f>
-        <x:v>À faire</x:v>
+        <x:v>Intégré</x:v>
       </x:c>
       <x:c r="G228" s="27" t="n">
         <x:f>COUNTIF(I228:P228,"Présent")</x:f>
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H228" s="24" t="str">
-        <x:v>À assembler</x:v>
+        <x:v>Archivé Drive</x:v>
       </x:c>
       <x:c r="I228" s="24" t="str">
-        <x:v>Référence</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="J228" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="K228" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="L228" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="M228" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="N228" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="O228" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="P228" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="Q228" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="R228" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="S228" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="T228" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="U228" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="V228" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="W228" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="X228" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="Y228" s="24" t="str">
         <x:v>Non consignée</x:v>
@@ -20993,13 +20993,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA228" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB228" s="21" t="str">
-        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
+        <x:v>e03821783020a61aeaaa58d22886e2118781efaa</x:v>
       </x:c>
       <x:c r="AC228" s="21" t="str">
-        <x:v>À intégrer</x:v>
+        <x:v>En cours</x:v>
       </x:c>
     </x:row>
     <x:row r="229" ht="40" customHeight="1">
@@ -21104,69 +21104,69 @@
         <x:v>220</x:v>
       </x:c>
       <x:c r="D230" s="24" t="str">
-        <x:v>À planifier</x:v>
+        <x:v>Lot 13</x:v>
       </x:c>
       <x:c r="E230" s="25" t="str">
         <x:v>Actions</x:v>
       </x:c>
       <x:c r="F230" s="24" t="str">
         <x:f>IF(AND(G230=8,COUNTIF(Q230:V230,"Atlas")=6),"Intégré","À faire")</x:f>
-        <x:v>À faire</x:v>
+        <x:v>Intégré</x:v>
       </x:c>
       <x:c r="G230" s="27" t="n">
         <x:f>COUNTIF(I230:P230,"Présent")</x:f>
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H230" s="24" t="str">
-        <x:v>À assembler</x:v>
+        <x:v>Archivé Drive</x:v>
       </x:c>
       <x:c r="I230" s="24" t="str">
-        <x:v>Référence</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="J230" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="K230" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="L230" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="M230" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="N230" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="O230" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="P230" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="Q230" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="R230" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="S230" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="T230" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="U230" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="V230" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="W230" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="X230" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="Y230" s="24" t="str">
         <x:v>Non consignée</x:v>
@@ -21175,13 +21175,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA230" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB230" s="21" t="str">
-        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
+        <x:v>e03821783020a61aeaaa58d22886e2118781efaa</x:v>
       </x:c>
       <x:c r="AC230" s="21" t="str">
-        <x:v>À intégrer</x:v>
+        <x:v>En cours</x:v>
       </x:c>
     </x:row>
     <x:row r="231" ht="40" customHeight="1">
@@ -21195,69 +21195,69 @@
         <x:v>221</x:v>
       </x:c>
       <x:c r="D231" s="24" t="str">
-        <x:v>À planifier</x:v>
+        <x:v>Lot 13</x:v>
       </x:c>
       <x:c r="E231" s="25" t="str">
         <x:v>Animaux</x:v>
       </x:c>
       <x:c r="F231" s="24" t="str">
         <x:f>IF(AND(G231=8,COUNTIF(Q231:V231,"Atlas")=6),"Intégré","À faire")</x:f>
-        <x:v>À faire</x:v>
+        <x:v>Intégré</x:v>
       </x:c>
       <x:c r="G231" s="27" t="n">
         <x:f>COUNTIF(I231:P231,"Présent")</x:f>
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H231" s="24" t="str">
-        <x:v>À assembler</x:v>
+        <x:v>Archivé Drive</x:v>
       </x:c>
       <x:c r="I231" s="24" t="str">
-        <x:v>Référence</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="J231" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="K231" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="L231" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="M231" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="N231" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="O231" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="P231" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="Q231" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="R231" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="S231" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="T231" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="U231" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="V231" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="W231" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="X231" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="Y231" s="24" t="str">
         <x:v>Non consignée</x:v>
@@ -21266,13 +21266,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA231" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB231" s="21" t="str">
-        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
+        <x:v>e03821783020a61aeaaa58d22886e2118781efaa</x:v>
       </x:c>
       <x:c r="AC231" s="21" t="str">
-        <x:v>À intégrer</x:v>
+        <x:v>En cours</x:v>
       </x:c>
     </x:row>
     <x:row r="232" ht="40" customHeight="1">
@@ -21832,69 +21832,69 @@
         <x:v>228</x:v>
       </x:c>
       <x:c r="D238" s="24" t="str">
-        <x:v>À planifier</x:v>
+        <x:v>Lot 13</x:v>
       </x:c>
       <x:c r="E238" s="25" t="str">
         <x:v>Lieux</x:v>
       </x:c>
       <x:c r="F238" s="24" t="str">
         <x:f>IF(AND(G238=8,COUNTIF(Q238:V238,"Atlas")=6),"Intégré","À faire")</x:f>
-        <x:v>À faire</x:v>
+        <x:v>Intégré</x:v>
       </x:c>
       <x:c r="G238" s="27" t="n">
         <x:f>COUNTIF(I238:P238,"Présent")</x:f>
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H238" s="24" t="str">
-        <x:v>À assembler</x:v>
+        <x:v>Archivé Drive</x:v>
       </x:c>
       <x:c r="I238" s="24" t="str">
-        <x:v>Référence</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="J238" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="K238" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="L238" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="M238" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="N238" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="O238" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="P238" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="Q238" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="R238" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="S238" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="T238" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="U238" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="V238" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="W238" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="X238" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="Y238" s="24" t="str">
         <x:v>Non consignée</x:v>
@@ -21903,13 +21903,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA238" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB238" s="21" t="str">
-        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
+        <x:v>e03821783020a61aeaaa58d22886e2118781efaa</x:v>
       </x:c>
       <x:c r="AC238" s="21" t="str">
-        <x:v>À intégrer</x:v>
+        <x:v>En cours</x:v>
       </x:c>
     </x:row>
     <x:row r="239" ht="40" customHeight="1">
@@ -22105,69 +22105,69 @@
         <x:v>231</x:v>
       </x:c>
       <x:c r="D241" s="24" t="str">
-        <x:v>À planifier</x:v>
+        <x:v>Lot 13</x:v>
       </x:c>
       <x:c r="E241" s="25" t="str">
         <x:v>Nature</x:v>
       </x:c>
       <x:c r="F241" s="24" t="str">
         <x:f>IF(AND(G241=8,COUNTIF(Q241:V241,"Atlas")=6),"Intégré","À faire")</x:f>
-        <x:v>À faire</x:v>
+        <x:v>Intégré</x:v>
       </x:c>
       <x:c r="G241" s="27" t="n">
         <x:f>COUNTIF(I241:P241,"Présent")</x:f>
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H241" s="24" t="str">
-        <x:v>À assembler</x:v>
+        <x:v>Archivé Drive</x:v>
       </x:c>
       <x:c r="I241" s="24" t="str">
-        <x:v>Référence</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="J241" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="K241" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="L241" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="M241" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="N241" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="O241" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="P241" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="Q241" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="R241" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="S241" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="T241" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="U241" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="V241" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="W241" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="X241" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="Y241" s="24" t="str">
         <x:v>Non consignée</x:v>
@@ -22176,13 +22176,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA241" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB241" s="21" t="str">
-        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
+        <x:v>e03821783020a61aeaaa58d22886e2118781efaa</x:v>
       </x:c>
       <x:c r="AC241" s="21" t="str">
-        <x:v>À intégrer</x:v>
+        <x:v>En cours</x:v>
       </x:c>
     </x:row>
     <x:row r="242" ht="40" customHeight="1">
@@ -22196,69 +22196,69 @@
         <x:v>232</x:v>
       </x:c>
       <x:c r="D242" s="24" t="str">
-        <x:v>À planifier</x:v>
+        <x:v>Lot 13</x:v>
       </x:c>
       <x:c r="E242" s="25" t="str">
         <x:v>Actions</x:v>
       </x:c>
       <x:c r="F242" s="24" t="str">
         <x:f>IF(AND(G242=8,COUNTIF(Q242:V242,"Atlas")=6),"Intégré","À faire")</x:f>
-        <x:v>À faire</x:v>
+        <x:v>Intégré</x:v>
       </x:c>
       <x:c r="G242" s="27" t="n">
         <x:f>COUNTIF(I242:P242,"Présent")</x:f>
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H242" s="24" t="str">
-        <x:v>À assembler</x:v>
+        <x:v>Archivé Drive</x:v>
       </x:c>
       <x:c r="I242" s="24" t="str">
-        <x:v>Référence</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="J242" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="K242" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="L242" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="M242" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="N242" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="O242" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="P242" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="Q242" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="R242" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="S242" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="T242" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="U242" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="V242" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="W242" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="X242" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="Y242" s="24" t="str">
         <x:v>Non consignée</x:v>
@@ -22267,13 +22267,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA242" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB242" s="21" t="str">
-        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
+        <x:v>e03821783020a61aeaaa58d22886e2118781efaa</x:v>
       </x:c>
       <x:c r="AC242" s="21" t="str">
-        <x:v>À intégrer</x:v>
+        <x:v>En cours</x:v>
       </x:c>
     </x:row>
     <x:row r="243" ht="40" customHeight="1">
@@ -22742,69 +22742,69 @@
         <x:v>238</x:v>
       </x:c>
       <x:c r="D248" s="24" t="str">
-        <x:v>À planifier</x:v>
+        <x:v>Lot 13</x:v>
       </x:c>
       <x:c r="E248" s="25" t="str">
         <x:v>Corps</x:v>
       </x:c>
       <x:c r="F248" s="24" t="str">
         <x:f>IF(AND(G248=8,COUNTIF(Q248:V248,"Atlas")=6),"Intégré","À faire")</x:f>
-        <x:v>À faire</x:v>
+        <x:v>Intégré</x:v>
       </x:c>
       <x:c r="G248" s="27" t="n">
         <x:f>COUNTIF(I248:P248,"Présent")</x:f>
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H248" s="24" t="str">
-        <x:v>À assembler</x:v>
+        <x:v>Archivé Drive</x:v>
       </x:c>
       <x:c r="I248" s="24" t="str">
-        <x:v>Référence</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="J248" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="K248" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="L248" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="M248" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="N248" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="O248" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="P248" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="Q248" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="R248" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="S248" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="T248" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="U248" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="V248" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="W248" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="X248" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="Y248" s="24" t="str">
         <x:v>Non consignée</x:v>
@@ -22813,13 +22813,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA248" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB248" s="21" t="str">
-        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
+        <x:v>e03821783020a61aeaaa58d22886e2118781efaa</x:v>
       </x:c>
       <x:c r="AC248" s="21" t="str">
-        <x:v>À intégrer</x:v>
+        <x:v>En cours</x:v>
       </x:c>
     </x:row>
     <x:row r="249" ht="40" customHeight="1">
@@ -23094,7 +23094,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8a2930917a3348ef"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra1d43efc63e541eb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Record all 240 complete packs and final source backup scope
</commit_message>
<xml_diff>
--- a/doc_web_interne/docs/suivi-symboles/suivi-240-symboles-6-langues.xlsx
+++ b/doc_web_interne/docs/suivi-symboles/suivi-240-symboles-6-langues.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Suivi symboles" sheetId="1" r:id="R92a6341196e445d8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Suivi symboles" sheetId="1" r:id="Rf0f362f846cc441e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -811,7 +811,7 @@
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="7" t="str">
-        <x:v>Lot 13 en branche : 29 couvertures conservées, 211 nouveaux PNG. Preuves antérieures inchangées conservées.</x:v>
+        <x:v>Lot 14 en branche : 10 couvertures conservées, 70 nouveaux PNG. Preuves antérieures inchangées conservées.</x:v>
       </x:c>
       <x:c r="B3" s="7"/>
       <x:c r="C3" s="7"/>
@@ -848,21 +848,21 @@
       </x:c>
       <x:c r="B4" s="9" t="n">
         <x:f>COUNTIF(F11:F250,"Intégré")</x:f>
-        <x:v>230</x:v>
+        <x:v>240</x:v>
       </x:c>
       <x:c r="C4" s="3" t="str">
         <x:v>Packs à terminer</x:v>
       </x:c>
       <x:c r="D4" s="9" t="n">
         <x:f>COUNTA(B11:B250)-B4</x:f>
-        <x:v>10</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="E4" s="3" t="str">
         <x:v>Pages avec pack</x:v>
       </x:c>
       <x:c r="F4" s="9" t="n">
         <x:f>COUNTIF(Q11:V250,"Atlas")</x:f>
-        <x:v>1380</x:v>
+        <x:v>1440</x:v>
       </x:c>
       <x:c r="G4" s="3" t="str">
         <x:v>Pages web</x:v>
@@ -899,14 +899,14 @@
       </x:c>
       <x:c r="B5" s="9" t="n">
         <x:f>COUNTIF(W11:W250,"6/6 actuelles")</x:f>
-        <x:v>230</x:v>
+        <x:v>240</x:v>
       </x:c>
       <x:c r="C5" s="3" t="str">
         <x:v>QA 2560 px</x:v>
       </x:c>
       <x:c r="D5" s="9" t="n">
         <x:f>COUNTIF(X11:X250,"6/6 actuelles")</x:f>
-        <x:v>230</x:v>
+        <x:v>240</x:v>
       </x:c>
       <x:c r="E5" s="3" t="str">
         <x:v>Accord Thanh</x:v>
@@ -980,7 +980,7 @@
     </x:row>
     <x:row r="7" ht="20" customHeight="1">
       <x:c r="A7" s="7" t="str">
-        <x:v>230 packs ; 10 à compléter. Cadre commun : 1 440 pages. Publication antérieure conservée dans les reçus.</x:v>
+        <x:v>240 packs ; 0 à compléter. Cadre commun : 1 440 pages. Publication antérieure conservée dans les reçus.</x:v>
       </x:c>
       <x:c r="B7" s="7"/>
       <x:c r="C7" s="7"/>
@@ -1013,7 +1013,7 @@
     </x:row>
     <x:row r="8" ht="20" customHeight="1">
       <x:c r="A8" s="7" t="str">
-        <x:v>Source : rapport canonique actuel, empreinte b6be04037927f2da. Révision : e03821783020a61aeaaa58d22886e2118781efaa</x:v>
+        <x:v>Source : rapport canonique actuel, empreinte 09ab652d0f30effe. Révision : 3eadba5f121c1017c032929534d269c330aa5abb</x:v>
       </x:c>
       <x:c r="B8" s="7"/>
       <x:c r="C8" s="7"/>
@@ -9365,69 +9365,69 @@
         <x:v>91</x:v>
       </x:c>
       <x:c r="D101" s="24" t="str">
-        <x:v>À planifier</x:v>
+        <x:v>Lot 14</x:v>
       </x:c>
       <x:c r="E101" s="25" t="str">
         <x:v>Objets</x:v>
       </x:c>
       <x:c r="F101" s="24" t="str">
         <x:f>IF(AND(G101=8,COUNTIF(Q101:V101,"Atlas")=6),"Intégré","À faire")</x:f>
-        <x:v>À faire</x:v>
+        <x:v>Intégré</x:v>
       </x:c>
       <x:c r="G101" s="27" t="n">
         <x:f>COUNTIF(I101:P101,"Présent")</x:f>
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H101" s="24" t="str">
-        <x:v>À assembler</x:v>
+        <x:v>Archivé Drive</x:v>
       </x:c>
       <x:c r="I101" s="24" t="str">
-        <x:v>Référence</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="J101" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="K101" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="L101" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="M101" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="N101" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="O101" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="P101" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="Q101" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="R101" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="S101" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="T101" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="U101" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="V101" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="W101" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="X101" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="Y101" s="24" t="str">
         <x:v>Non consignée</x:v>
@@ -9436,13 +9436,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA101" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB101" s="21" t="str">
-        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
+        <x:v>3eadba5f121c1017c032929534d269c330aa5abb</x:v>
       </x:c>
       <x:c r="AC101" s="21" t="str">
-        <x:v>À intégrer</x:v>
+        <x:v>En cours</x:v>
       </x:c>
     </x:row>
     <x:row r="102" ht="40" customHeight="1">
@@ -10457,69 +10457,69 @@
         <x:v>103</x:v>
       </x:c>
       <x:c r="D113" s="24" t="str">
-        <x:v>À planifier</x:v>
+        <x:v>Lot 14</x:v>
       </x:c>
       <x:c r="E113" s="25" t="str">
         <x:v>Objets</x:v>
       </x:c>
       <x:c r="F113" s="24" t="str">
         <x:f>IF(AND(G113=8,COUNTIF(Q113:V113,"Atlas")=6),"Intégré","À faire")</x:f>
-        <x:v>À faire</x:v>
+        <x:v>Intégré</x:v>
       </x:c>
       <x:c r="G113" s="27" t="n">
         <x:f>COUNTIF(I113:P113,"Présent")</x:f>
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H113" s="24" t="str">
-        <x:v>À assembler</x:v>
+        <x:v>Archivé Drive</x:v>
       </x:c>
       <x:c r="I113" s="24" t="str">
-        <x:v>Référence</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="J113" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="K113" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="L113" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="M113" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="N113" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="O113" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="P113" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="Q113" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="R113" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="S113" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="T113" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="U113" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="V113" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="W113" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="X113" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="Y113" s="24" t="str">
         <x:v>Non consignée</x:v>
@@ -10528,13 +10528,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA113" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB113" s="21" t="str">
-        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
+        <x:v>3eadba5f121c1017c032929534d269c330aa5abb</x:v>
       </x:c>
       <x:c r="AC113" s="21" t="str">
-        <x:v>À intégrer</x:v>
+        <x:v>En cours</x:v>
       </x:c>
     </x:row>
     <x:row r="114" ht="40" customHeight="1">
@@ -11185,69 +11185,69 @@
         <x:v>111</x:v>
       </x:c>
       <x:c r="D121" s="24" t="str">
-        <x:v>À planifier</x:v>
+        <x:v>Lot 14</x:v>
       </x:c>
       <x:c r="E121" s="25" t="str">
         <x:v>Ciel</x:v>
       </x:c>
       <x:c r="F121" s="24" t="str">
         <x:f>IF(AND(G121=8,COUNTIF(Q121:V121,"Atlas")=6),"Intégré","À faire")</x:f>
-        <x:v>À faire</x:v>
+        <x:v>Intégré</x:v>
       </x:c>
       <x:c r="G121" s="27" t="n">
         <x:f>COUNTIF(I121:P121,"Présent")</x:f>
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H121" s="24" t="str">
-        <x:v>À assembler</x:v>
+        <x:v>Archivé Drive</x:v>
       </x:c>
       <x:c r="I121" s="24" t="str">
-        <x:v>Référence</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="J121" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="K121" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="L121" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="M121" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="N121" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="O121" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="P121" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="Q121" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="R121" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="S121" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="T121" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="U121" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="V121" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="W121" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="X121" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="Y121" s="24" t="str">
         <x:v>Non consignée</x:v>
@@ -11256,13 +11256,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA121" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB121" s="21" t="str">
-        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
+        <x:v>3eadba5f121c1017c032929534d269c330aa5abb</x:v>
       </x:c>
       <x:c r="AC121" s="21" t="str">
-        <x:v>À intégrer</x:v>
+        <x:v>En cours</x:v>
       </x:c>
     </x:row>
     <x:row r="122" ht="40" customHeight="1">
@@ -11367,69 +11367,69 @@
         <x:v>113</x:v>
       </x:c>
       <x:c r="D123" s="24" t="str">
-        <x:v>À planifier</x:v>
+        <x:v>Lot 14</x:v>
       </x:c>
       <x:c r="E123" s="25" t="str">
         <x:v>Personnes</x:v>
       </x:c>
       <x:c r="F123" s="24" t="str">
         <x:f>IF(AND(G123=8,COUNTIF(Q123:V123,"Atlas")=6),"Intégré","À faire")</x:f>
-        <x:v>À faire</x:v>
+        <x:v>Intégré</x:v>
       </x:c>
       <x:c r="G123" s="27" t="n">
         <x:f>COUNTIF(I123:P123,"Présent")</x:f>
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H123" s="24" t="str">
-        <x:v>À assembler</x:v>
+        <x:v>Archivé Drive</x:v>
       </x:c>
       <x:c r="I123" s="24" t="str">
-        <x:v>Référence</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="J123" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="K123" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="L123" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="M123" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="N123" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="O123" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="P123" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="Q123" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="R123" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="S123" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="T123" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="U123" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="V123" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="W123" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="X123" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="Y123" s="24" t="str">
         <x:v>Non consignée</x:v>
@@ -11438,13 +11438,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA123" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB123" s="21" t="str">
-        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
+        <x:v>3eadba5f121c1017c032929534d269c330aa5abb</x:v>
       </x:c>
       <x:c r="AC123" s="21" t="str">
-        <x:v>À intégrer</x:v>
+        <x:v>En cours</x:v>
       </x:c>
     </x:row>
     <x:row r="124" ht="40" customHeight="1">
@@ -11913,69 +11913,69 @@
         <x:v>119</x:v>
       </x:c>
       <x:c r="D129" s="24" t="str">
-        <x:v>À planifier</x:v>
+        <x:v>Lot 14</x:v>
       </x:c>
       <x:c r="E129" s="25" t="str">
         <x:v>Objets</x:v>
       </x:c>
       <x:c r="F129" s="24" t="str">
         <x:f>IF(AND(G129=8,COUNTIF(Q129:V129,"Atlas")=6),"Intégré","À faire")</x:f>
-        <x:v>À faire</x:v>
+        <x:v>Intégré</x:v>
       </x:c>
       <x:c r="G129" s="27" t="n">
         <x:f>COUNTIF(I129:P129,"Présent")</x:f>
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H129" s="24" t="str">
-        <x:v>À assembler</x:v>
+        <x:v>Archivé Drive</x:v>
       </x:c>
       <x:c r="I129" s="24" t="str">
-        <x:v>Référence</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="J129" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="K129" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="L129" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="M129" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="N129" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="O129" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="P129" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="Q129" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="R129" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="S129" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="T129" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="U129" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="V129" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="W129" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="X129" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="Y129" s="24" t="str">
         <x:v>Non consignée</x:v>
@@ -11984,13 +11984,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA129" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB129" s="21" t="str">
-        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
+        <x:v>3eadba5f121c1017c032929534d269c330aa5abb</x:v>
       </x:c>
       <x:c r="AC129" s="21" t="str">
-        <x:v>À intégrer</x:v>
+        <x:v>En cours</x:v>
       </x:c>
     </x:row>
     <x:row r="130" ht="40" customHeight="1">
@@ -12732,69 +12732,69 @@
         <x:v>128</x:v>
       </x:c>
       <x:c r="D138" s="24" t="str">
-        <x:v>À planifier</x:v>
+        <x:v>Lot 14</x:v>
       </x:c>
       <x:c r="E138" s="25" t="str">
         <x:v>Ciel</x:v>
       </x:c>
       <x:c r="F138" s="24" t="str">
         <x:f>IF(AND(G138=8,COUNTIF(Q138:V138,"Atlas")=6),"Intégré","À faire")</x:f>
-        <x:v>À faire</x:v>
+        <x:v>Intégré</x:v>
       </x:c>
       <x:c r="G138" s="27" t="n">
         <x:f>COUNTIF(I138:P138,"Présent")</x:f>
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H138" s="24" t="str">
-        <x:v>À assembler</x:v>
+        <x:v>Archivé Drive</x:v>
       </x:c>
       <x:c r="I138" s="24" t="str">
-        <x:v>Référence</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="J138" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="K138" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="L138" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="M138" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="N138" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="O138" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="P138" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="Q138" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="R138" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="S138" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="T138" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="U138" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="V138" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="W138" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="X138" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="Y138" s="24" t="str">
         <x:v>Non consignée</x:v>
@@ -12803,13 +12803,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA138" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB138" s="21" t="str">
-        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
+        <x:v>3eadba5f121c1017c032929534d269c330aa5abb</x:v>
       </x:c>
       <x:c r="AC138" s="21" t="str">
-        <x:v>À intégrer</x:v>
+        <x:v>En cours</x:v>
       </x:c>
     </x:row>
     <x:row r="139" ht="40" customHeight="1">
@@ -18101,69 +18101,69 @@
         <x:v>187</x:v>
       </x:c>
       <x:c r="D197" s="24" t="str">
-        <x:v>À planifier</x:v>
+        <x:v>Lot 14</x:v>
       </x:c>
       <x:c r="E197" s="25" t="str">
         <x:v>Objets</x:v>
       </x:c>
       <x:c r="F197" s="24" t="str">
         <x:f>IF(AND(G197=8,COUNTIF(Q197:V197,"Atlas")=6),"Intégré","À faire")</x:f>
-        <x:v>À faire</x:v>
+        <x:v>Intégré</x:v>
       </x:c>
       <x:c r="G197" s="27" t="n">
         <x:f>COUNTIF(I197:P197,"Présent")</x:f>
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H197" s="24" t="str">
-        <x:v>À assembler</x:v>
+        <x:v>Archivé Drive</x:v>
       </x:c>
       <x:c r="I197" s="24" t="str">
-        <x:v>Référence</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="J197" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="K197" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="L197" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="M197" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="N197" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="O197" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="P197" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="Q197" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="R197" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="S197" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="T197" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="U197" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="V197" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="W197" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="X197" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="Y197" s="24" t="str">
         <x:v>Non consignée</x:v>
@@ -18172,13 +18172,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA197" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB197" s="21" t="str">
-        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
+        <x:v>3eadba5f121c1017c032929534d269c330aa5abb</x:v>
       </x:c>
       <x:c r="AC197" s="21" t="str">
-        <x:v>À intégrer</x:v>
+        <x:v>En cours</x:v>
       </x:c>
     </x:row>
     <x:row r="198" ht="40" customHeight="1">
@@ -19375,69 +19375,69 @@
         <x:v>201</x:v>
       </x:c>
       <x:c r="D211" s="24" t="str">
-        <x:v>À planifier</x:v>
+        <x:v>Lot 14</x:v>
       </x:c>
       <x:c r="E211" s="25" t="str">
         <x:v>Objets</x:v>
       </x:c>
       <x:c r="F211" s="24" t="str">
         <x:f>IF(AND(G211=8,COUNTIF(Q211:V211,"Atlas")=6),"Intégré","À faire")</x:f>
-        <x:v>À faire</x:v>
+        <x:v>Intégré</x:v>
       </x:c>
       <x:c r="G211" s="27" t="n">
         <x:f>COUNTIF(I211:P211,"Présent")</x:f>
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H211" s="24" t="str">
-        <x:v>À assembler</x:v>
+        <x:v>Archivé Drive</x:v>
       </x:c>
       <x:c r="I211" s="24" t="str">
-        <x:v>Référence</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="J211" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="K211" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="L211" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="M211" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="N211" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="O211" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="P211" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="Q211" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="R211" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="S211" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="T211" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="U211" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="V211" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="W211" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="X211" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="Y211" s="24" t="str">
         <x:v>Non consignée</x:v>
@@ -19446,13 +19446,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA211" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB211" s="21" t="str">
-        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
+        <x:v>3eadba5f121c1017c032929534d269c330aa5abb</x:v>
       </x:c>
       <x:c r="AC211" s="21" t="str">
-        <x:v>À intégrer</x:v>
+        <x:v>En cours</x:v>
       </x:c>
     </x:row>
     <x:row r="212" ht="40" customHeight="1">
@@ -19466,69 +19466,69 @@
         <x:v>202</x:v>
       </x:c>
       <x:c r="D212" s="24" t="str">
-        <x:v>À planifier</x:v>
+        <x:v>Lot 14</x:v>
       </x:c>
       <x:c r="E212" s="25" t="str">
         <x:v>Objets</x:v>
       </x:c>
       <x:c r="F212" s="24" t="str">
         <x:f>IF(AND(G212=8,COUNTIF(Q212:V212,"Atlas")=6),"Intégré","À faire")</x:f>
-        <x:v>À faire</x:v>
+        <x:v>Intégré</x:v>
       </x:c>
       <x:c r="G212" s="27" t="n">
         <x:f>COUNTIF(I212:P212,"Présent")</x:f>
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H212" s="24" t="str">
-        <x:v>À assembler</x:v>
+        <x:v>Archivé Drive</x:v>
       </x:c>
       <x:c r="I212" s="24" t="str">
-        <x:v>Référence</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="J212" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="K212" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="L212" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="M212" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="N212" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="O212" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="P212" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="Q212" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="R212" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="S212" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="T212" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="U212" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="V212" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="W212" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="X212" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="Y212" s="24" t="str">
         <x:v>Non consignée</x:v>
@@ -19537,13 +19537,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA212" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB212" s="21" t="str">
-        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
+        <x:v>3eadba5f121c1017c032929534d269c330aa5abb</x:v>
       </x:c>
       <x:c r="AC212" s="21" t="str">
-        <x:v>À intégrer</x:v>
+        <x:v>En cours</x:v>
       </x:c>
     </x:row>
     <x:row r="213" ht="40" customHeight="1">
@@ -21377,69 +21377,69 @@
         <x:v>223</x:v>
       </x:c>
       <x:c r="D233" s="24" t="str">
-        <x:v>À planifier</x:v>
+        <x:v>Lot 14</x:v>
       </x:c>
       <x:c r="E233" s="25" t="str">
         <x:v>Personnes</x:v>
       </x:c>
       <x:c r="F233" s="24" t="str">
         <x:f>IF(AND(G233=8,COUNTIF(Q233:V233,"Atlas")=6),"Intégré","À faire")</x:f>
-        <x:v>À faire</x:v>
+        <x:v>Intégré</x:v>
       </x:c>
       <x:c r="G233" s="27" t="n">
         <x:f>COUNTIF(I233:P233,"Présent")</x:f>
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H233" s="24" t="str">
-        <x:v>À assembler</x:v>
+        <x:v>Archivé Drive</x:v>
       </x:c>
       <x:c r="I233" s="24" t="str">
-        <x:v>Référence</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="J233" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="K233" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="L233" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="M233" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="N233" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="O233" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="P233" s="24" t="str">
-        <x:v>Manquant</x:v>
+        <x:v>Présent</x:v>
       </x:c>
       <x:c r="Q233" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="R233" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="S233" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="T233" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="U233" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="V233" s="24" t="str">
-        <x:v>Commun</x:v>
+        <x:v>Atlas</x:v>
       </x:c>
       <x:c r="W233" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="X233" s="24" t="str">
-        <x:v>Non consignée</x:v>
+        <x:v>6/6 actuelles</x:v>
       </x:c>
       <x:c r="Y233" s="24" t="str">
         <x:v>Non consignée</x:v>
@@ -21448,13 +21448,13 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA233" s="23" t="str">
-        <x:v>QA à compléter ou renouveler. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
       </x:c>
       <x:c r="AB233" s="21" t="str">
-        <x:v>76d7e577dfb7eb5251b0898e994e3a5210bfd56c</x:v>
+        <x:v>3eadba5f121c1017c032929534d269c330aa5abb</x:v>
       </x:c>
       <x:c r="AC233" s="21" t="str">
-        <x:v>À intégrer</x:v>
+        <x:v>En cours</x:v>
       </x:c>
     </x:row>
     <x:row r="234" ht="40" customHeight="1">
@@ -23094,7 +23094,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra1d43efc63e541eb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7a56d21d265e4fa6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Compact complete historical rollout registry without dropping evidence
</commit_message>
<xml_diff>
--- a/doc_web_interne/docs/suivi-symboles/suivi-240-symboles-6-langues.xlsx
+++ b/doc_web_interne/docs/suivi-symboles/suivi-240-symboles-6-langues.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Suivi symboles" sheetId="1" r:id="Rf0f362f846cc441e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Suivi symboles" sheetId="1" r:id="Rf4cc105cee8b402e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1013,7 +1013,7 @@
     </x:row>
     <x:row r="8" ht="20" customHeight="1">
       <x:c r="A8" s="7" t="str">
-        <x:v>Source : rapport canonique actuel, empreinte 09ab652d0f30effe. Révision : 3eadba5f121c1017c032929534d269c330aa5abb</x:v>
+        <x:v>Source : rapport canonique actuel, empreinte 88509a9cc8e5e634. Révision : 3eadba5f121c1017c032929534d269c330aa5abb</x:v>
       </x:c>
       <x:c r="B8" s="7"/>
       <x:c r="C8" s="7"/>
@@ -23094,7 +23094,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7a56d21d265e4fa6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2543f6d651e84bc1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs(symbols): record full 240-pack site qualification and source backup
</commit_message>
<xml_diff>
--- a/doc_web_interne/docs/suivi-symboles/suivi-240-symboles-6-langues.xlsx
+++ b/doc_web_interne/docs/suivi-symboles/suivi-240-symboles-6-langues.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Suivi symboles" sheetId="1" r:id="Rf4cc105cee8b402e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Suivi symboles" sheetId="1" r:id="R1952b03bb8c94b9f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -811,7 +811,7 @@
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="7" t="str">
-        <x:v>Lot 14 en branche : 10 couvertures conservées, 70 nouveaux PNG. Preuves antérieures inchangées conservées.</x:v>
+        <x:v>240 packs intégrés dans les six langues. Validation actuelle ; publication assurée par Thanh.</x:v>
       </x:c>
       <x:c r="B3" s="7"/>
       <x:c r="C3" s="7"/>
@@ -980,7 +980,7 @@
     </x:row>
     <x:row r="7" ht="20" customHeight="1">
       <x:c r="A7" s="7" t="str">
-        <x:v>240 packs ; 0 à compléter. Cadre commun : 1 440 pages. Publication antérieure conservée dans les reçus.</x:v>
+        <x:v>240 packs, 1 440 pages. Sources originales des six packs retrouvées et sauvegardées sur Drive.</x:v>
       </x:c>
       <x:c r="B7" s="7"/>
       <x:c r="C7" s="7"/>
@@ -1013,7 +1013,7 @@
     </x:row>
     <x:row r="8" ht="20" customHeight="1">
       <x:c r="A8" s="7" t="str">
-        <x:v>Source : rapport canonique actuel, empreinte 88509a9cc8e5e634. Révision : 3eadba5f121c1017c032929534d269c330aa5abb</x:v>
+        <x:v>Source : rapport canonique 5f96fe5298e47cda. Révision : 674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="B8" s="7"/>
       <x:c r="C8" s="7"/>
@@ -1246,10 +1246,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA11" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB11" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC11" s="21" t="str">
         <x:v>En cours</x:v>
@@ -1337,10 +1337,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA12" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB12" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC12" s="21" t="str">
         <x:v>En cours</x:v>
@@ -1428,10 +1428,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA13" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB13" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC13" s="21" t="str">
         <x:v>En cours</x:v>
@@ -1519,10 +1519,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA14" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB14" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC14" s="21" t="str">
         <x:v>En cours</x:v>
@@ -1610,10 +1610,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA15" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB15" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC15" s="21" t="str">
         <x:v>En cours</x:v>
@@ -1701,10 +1701,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA16" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB16" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC16" s="21" t="str">
         <x:v>En cours</x:v>
@@ -1792,10 +1792,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA17" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB17" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC17" s="21" t="str">
         <x:v>En cours</x:v>
@@ -1883,10 +1883,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA18" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB18" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC18" s="21" t="str">
         <x:v>En cours</x:v>
@@ -1974,10 +1974,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA19" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB19" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC19" s="21" t="str">
         <x:v>En cours</x:v>
@@ -2065,10 +2065,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA20" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB20" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC20" s="21" t="str">
         <x:v>En cours</x:v>
@@ -2156,10 +2156,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA21" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB21" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC21" s="21" t="str">
         <x:v>En cours</x:v>
@@ -2247,10 +2247,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA22" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB22" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC22" s="21" t="str">
         <x:v>En cours</x:v>
@@ -2338,10 +2338,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA23" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB23" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC23" s="21" t="str">
         <x:v>En cours</x:v>
@@ -2429,10 +2429,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA24" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB24" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC24" s="21" t="str">
         <x:v>En cours</x:v>
@@ -2520,10 +2520,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA25" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB25" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC25" s="21" t="str">
         <x:v>En cours</x:v>
@@ -2611,10 +2611,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA26" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB26" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC26" s="21" t="str">
         <x:v>En cours</x:v>
@@ -2702,10 +2702,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA27" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB27" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC27" s="21" t="str">
         <x:v>En cours</x:v>
@@ -2793,10 +2793,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA28" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB28" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC28" s="21" t="str">
         <x:v>En cours</x:v>
@@ -2884,10 +2884,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA29" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB29" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC29" s="21" t="str">
         <x:v>En cours</x:v>
@@ -2975,10 +2975,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA30" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB30" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC30" s="21" t="str">
         <x:v>En cours</x:v>
@@ -3066,10 +3066,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA31" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB31" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC31" s="21" t="str">
         <x:v>En cours</x:v>
@@ -3157,10 +3157,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA32" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB32" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC32" s="21" t="str">
         <x:v>En cours</x:v>
@@ -3248,10 +3248,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA33" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB33" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC33" s="21" t="str">
         <x:v>En cours</x:v>
@@ -3339,10 +3339,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA34" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB34" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC34" s="21" t="str">
         <x:v>En cours</x:v>
@@ -3430,10 +3430,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA35" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB35" s="21" t="str">
-        <x:v>e03821783020a61aeaaa58d22886e2118781efaa</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC35" s="21" t="str">
         <x:v>En cours</x:v>
@@ -3521,10 +3521,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA36" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB36" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC36" s="21" t="str">
         <x:v>En cours</x:v>
@@ -3555,7 +3555,7 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="H37" s="24" t="str">
-        <x:v>Réutilisé master #509</x:v>
+        <x:v>Archive Drive</x:v>
       </x:c>
       <x:c r="I37" s="24" t="str">
         <x:v>Présent</x:v>
@@ -3612,10 +3612,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA37" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB37" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC37" s="21" t="str">
         <x:v>En cours</x:v>
@@ -3703,10 +3703,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA38" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB38" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC38" s="21" t="str">
         <x:v>En cours</x:v>
@@ -3794,10 +3794,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA39" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB39" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC39" s="21" t="str">
         <x:v>En cours</x:v>
@@ -3885,10 +3885,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA40" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB40" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC40" s="21" t="str">
         <x:v>En cours</x:v>
@@ -3976,10 +3976,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA41" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB41" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC41" s="21" t="str">
         <x:v>En cours</x:v>
@@ -4067,10 +4067,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA42" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB42" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC42" s="21" t="str">
         <x:v>En cours</x:v>
@@ -4158,10 +4158,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA43" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB43" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC43" s="21" t="str">
         <x:v>En cours</x:v>
@@ -4249,10 +4249,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA44" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB44" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC44" s="21" t="str">
         <x:v>En cours</x:v>
@@ -4340,10 +4340,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA45" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB45" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC45" s="21" t="str">
         <x:v>En cours</x:v>
@@ -4431,10 +4431,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA46" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB46" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC46" s="21" t="str">
         <x:v>En cours</x:v>
@@ -4522,10 +4522,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA47" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB47" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC47" s="21" t="str">
         <x:v>En cours</x:v>
@@ -4613,10 +4613,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA48" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB48" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC48" s="21" t="str">
         <x:v>En cours</x:v>
@@ -4704,10 +4704,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA49" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB49" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC49" s="21" t="str">
         <x:v>En cours</x:v>
@@ -4795,10 +4795,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA50" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB50" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC50" s="21" t="str">
         <x:v>En cours</x:v>
@@ -4886,10 +4886,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA51" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB51" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC51" s="21" t="str">
         <x:v>En cours</x:v>
@@ -4977,10 +4977,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA52" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB52" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC52" s="21" t="str">
         <x:v>En cours</x:v>
@@ -5068,10 +5068,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA53" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB53" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC53" s="21" t="str">
         <x:v>En cours</x:v>
@@ -5159,10 +5159,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA54" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB54" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC54" s="21" t="str">
         <x:v>En cours</x:v>
@@ -5250,10 +5250,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA55" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB55" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC55" s="21" t="str">
         <x:v>En cours</x:v>
@@ -5341,10 +5341,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA56" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB56" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC56" s="21" t="str">
         <x:v>En cours</x:v>
@@ -5432,10 +5432,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA57" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB57" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC57" s="21" t="str">
         <x:v>En cours</x:v>
@@ -5523,10 +5523,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA58" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB58" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC58" s="21" t="str">
         <x:v>En cours</x:v>
@@ -5614,10 +5614,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA59" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB59" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC59" s="21" t="str">
         <x:v>En cours</x:v>
@@ -5705,10 +5705,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA60" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB60" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC60" s="21" t="str">
         <x:v>En cours</x:v>
@@ -5796,10 +5796,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA61" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB61" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC61" s="21" t="str">
         <x:v>En cours</x:v>
@@ -5887,10 +5887,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA62" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB62" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC62" s="21" t="str">
         <x:v>En cours</x:v>
@@ -5978,10 +5978,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA63" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB63" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC63" s="21" t="str">
         <x:v>En cours</x:v>
@@ -6069,10 +6069,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA64" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB64" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC64" s="21" t="str">
         <x:v>En cours</x:v>
@@ -6160,10 +6160,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA65" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB65" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC65" s="21" t="str">
         <x:v>En cours</x:v>
@@ -6251,10 +6251,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA66" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB66" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC66" s="21" t="str">
         <x:v>En cours</x:v>
@@ -6342,10 +6342,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA67" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB67" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC67" s="21" t="str">
         <x:v>En cours</x:v>
@@ -6433,10 +6433,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA68" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB68" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC68" s="21" t="str">
         <x:v>En cours</x:v>
@@ -6524,10 +6524,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA69" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB69" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC69" s="21" t="str">
         <x:v>En cours</x:v>
@@ -6615,10 +6615,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA70" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB70" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC70" s="21" t="str">
         <x:v>En cours</x:v>
@@ -6706,10 +6706,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA71" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB71" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC71" s="21" t="str">
         <x:v>En cours</x:v>
@@ -6797,10 +6797,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA72" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB72" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC72" s="21" t="str">
         <x:v>En cours</x:v>
@@ -6888,10 +6888,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA73" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB73" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC73" s="21" t="str">
         <x:v>En cours</x:v>
@@ -6979,10 +6979,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA74" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB74" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC74" s="21" t="str">
         <x:v>En cours</x:v>
@@ -7070,10 +7070,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA75" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB75" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC75" s="21" t="str">
         <x:v>En cours</x:v>
@@ -7161,10 +7161,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA76" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB76" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC76" s="21" t="str">
         <x:v>En cours</x:v>
@@ -7252,10 +7252,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA77" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB77" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC77" s="21" t="str">
         <x:v>En cours</x:v>
@@ -7343,10 +7343,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA78" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB78" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC78" s="21" t="str">
         <x:v>En cours</x:v>
@@ -7434,10 +7434,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA79" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB79" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC79" s="21" t="str">
         <x:v>En cours</x:v>
@@ -7525,10 +7525,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA80" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB80" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC80" s="21" t="str">
         <x:v>En cours</x:v>
@@ -7616,10 +7616,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA81" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB81" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC81" s="21" t="str">
         <x:v>En cours</x:v>
@@ -7707,10 +7707,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA82" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB82" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC82" s="21" t="str">
         <x:v>En cours</x:v>
@@ -7798,10 +7798,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA83" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB83" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC83" s="21" t="str">
         <x:v>En cours</x:v>
@@ -7889,10 +7889,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA84" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB84" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC84" s="21" t="str">
         <x:v>En cours</x:v>
@@ -7980,10 +7980,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA85" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB85" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC85" s="21" t="str">
         <x:v>En cours</x:v>
@@ -8071,10 +8071,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA86" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB86" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC86" s="21" t="str">
         <x:v>En cours</x:v>
@@ -8162,10 +8162,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA87" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB87" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC87" s="21" t="str">
         <x:v>En cours</x:v>
@@ -8253,10 +8253,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA88" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB88" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC88" s="21" t="str">
         <x:v>En cours</x:v>
@@ -8344,10 +8344,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA89" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB89" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC89" s="21" t="str">
         <x:v>En cours</x:v>
@@ -8378,7 +8378,7 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="H90" s="24" t="str">
-        <x:v>Réutilisé master #509</x:v>
+        <x:v>Archive Drive</x:v>
       </x:c>
       <x:c r="I90" s="24" t="str">
         <x:v>Présent</x:v>
@@ -8435,10 +8435,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA90" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB90" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC90" s="21" t="str">
         <x:v>En cours</x:v>
@@ -8526,10 +8526,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA91" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB91" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC91" s="21" t="str">
         <x:v>En cours</x:v>
@@ -8617,10 +8617,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA92" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB92" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC92" s="21" t="str">
         <x:v>En cours</x:v>
@@ -8708,10 +8708,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA93" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB93" s="21" t="str">
-        <x:v>b17117db72da867328bfee7e7b5ac7c17acc0aab</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC93" s="21" t="str">
         <x:v>En cours</x:v>
@@ -8799,10 +8799,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA94" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB94" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC94" s="21" t="str">
         <x:v>En cours</x:v>
@@ -8890,10 +8890,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA95" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB95" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC95" s="21" t="str">
         <x:v>En cours</x:v>
@@ -8981,10 +8981,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA96" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB96" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC96" s="21" t="str">
         <x:v>En cours</x:v>
@@ -9072,10 +9072,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA97" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB97" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC97" s="21" t="str">
         <x:v>En cours</x:v>
@@ -9163,10 +9163,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA98" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB98" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC98" s="21" t="str">
         <x:v>En cours</x:v>
@@ -9254,10 +9254,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA99" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB99" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC99" s="21" t="str">
         <x:v>En cours</x:v>
@@ -9345,10 +9345,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA100" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB100" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC100" s="21" t="str">
         <x:v>En cours</x:v>
@@ -9436,10 +9436,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA101" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB101" s="21" t="str">
-        <x:v>3eadba5f121c1017c032929534d269c330aa5abb</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC101" s="21" t="str">
         <x:v>En cours</x:v>
@@ -9527,10 +9527,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA102" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB102" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC102" s="21" t="str">
         <x:v>En cours</x:v>
@@ -9561,7 +9561,7 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="H103" s="24" t="str">
-        <x:v>Réutilisé master #509</x:v>
+        <x:v>Archive Drive</x:v>
       </x:c>
       <x:c r="I103" s="24" t="str">
         <x:v>Présent</x:v>
@@ -9618,10 +9618,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA103" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB103" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC103" s="21" t="str">
         <x:v>En cours</x:v>
@@ -9709,10 +9709,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA104" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB104" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC104" s="21" t="str">
         <x:v>En cours</x:v>
@@ -9800,10 +9800,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA105" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB105" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC105" s="21" t="str">
         <x:v>En cours</x:v>
@@ -9891,10 +9891,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA106" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB106" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC106" s="21" t="str">
         <x:v>En cours</x:v>
@@ -9982,10 +9982,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA107" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB107" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC107" s="21" t="str">
         <x:v>En cours</x:v>
@@ -10073,10 +10073,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA108" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB108" s="21" t="str">
-        <x:v>b17117db72da867328bfee7e7b5ac7c17acc0aab</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC108" s="21" t="str">
         <x:v>En cours</x:v>
@@ -10164,10 +10164,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA109" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB109" s="21" t="str">
-        <x:v>b17117db72da867328bfee7e7b5ac7c17acc0aab</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC109" s="21" t="str">
         <x:v>En cours</x:v>
@@ -10198,7 +10198,7 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="H110" s="24" t="str">
-        <x:v>Réutilisé master #509</x:v>
+        <x:v>Archive Drive</x:v>
       </x:c>
       <x:c r="I110" s="24" t="str">
         <x:v>Présent</x:v>
@@ -10255,10 +10255,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA110" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB110" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC110" s="21" t="str">
         <x:v>En cours</x:v>
@@ -10346,10 +10346,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA111" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB111" s="21" t="str">
-        <x:v>e03821783020a61aeaaa58d22886e2118781efaa</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC111" s="21" t="str">
         <x:v>En cours</x:v>
@@ -10437,10 +10437,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA112" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB112" s="21" t="str">
-        <x:v>b17117db72da867328bfee7e7b5ac7c17acc0aab</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC112" s="21" t="str">
         <x:v>En cours</x:v>
@@ -10528,10 +10528,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA113" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB113" s="21" t="str">
-        <x:v>3eadba5f121c1017c032929534d269c330aa5abb</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC113" s="21" t="str">
         <x:v>En cours</x:v>
@@ -10619,10 +10619,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA114" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB114" s="21" t="str">
-        <x:v>e03821783020a61aeaaa58d22886e2118781efaa</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC114" s="21" t="str">
         <x:v>En cours</x:v>
@@ -10710,10 +10710,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA115" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB115" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC115" s="21" t="str">
         <x:v>En cours</x:v>
@@ -10801,10 +10801,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA116" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB116" s="21" t="str">
-        <x:v>b17117db72da867328bfee7e7b5ac7c17acc0aab</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC116" s="21" t="str">
         <x:v>En cours</x:v>
@@ -10892,10 +10892,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA117" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB117" s="21" t="str">
-        <x:v>e03821783020a61aeaaa58d22886e2118781efaa</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC117" s="21" t="str">
         <x:v>En cours</x:v>
@@ -10983,10 +10983,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA118" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB118" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC118" s="21" t="str">
         <x:v>En cours</x:v>
@@ -11074,10 +11074,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA119" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB119" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC119" s="21" t="str">
         <x:v>En cours</x:v>
@@ -11165,10 +11165,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA120" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB120" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC120" s="21" t="str">
         <x:v>En cours</x:v>
@@ -11256,10 +11256,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA121" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB121" s="21" t="str">
-        <x:v>3eadba5f121c1017c032929534d269c330aa5abb</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC121" s="21" t="str">
         <x:v>En cours</x:v>
@@ -11347,10 +11347,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA122" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB122" s="21" t="str">
-        <x:v>e03821783020a61aeaaa58d22886e2118781efaa</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC122" s="21" t="str">
         <x:v>En cours</x:v>
@@ -11438,10 +11438,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA123" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB123" s="21" t="str">
-        <x:v>3eadba5f121c1017c032929534d269c330aa5abb</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC123" s="21" t="str">
         <x:v>En cours</x:v>
@@ -11529,10 +11529,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA124" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB124" s="21" t="str">
-        <x:v>e03821783020a61aeaaa58d22886e2118781efaa</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC124" s="21" t="str">
         <x:v>En cours</x:v>
@@ -11620,10 +11620,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA125" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB125" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC125" s="21" t="str">
         <x:v>En cours</x:v>
@@ -11711,10 +11711,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA126" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB126" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC126" s="21" t="str">
         <x:v>En cours</x:v>
@@ -11802,10 +11802,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA127" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB127" s="21" t="str">
-        <x:v>b17117db72da867328bfee7e7b5ac7c17acc0aab</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC127" s="21" t="str">
         <x:v>En cours</x:v>
@@ -11893,10 +11893,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA128" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB128" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC128" s="21" t="str">
         <x:v>En cours</x:v>
@@ -11984,10 +11984,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA129" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB129" s="21" t="str">
-        <x:v>3eadba5f121c1017c032929534d269c330aa5abb</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC129" s="21" t="str">
         <x:v>En cours</x:v>
@@ -12075,10 +12075,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA130" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB130" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC130" s="21" t="str">
         <x:v>En cours</x:v>
@@ -12166,10 +12166,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA131" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB131" s="21" t="str">
-        <x:v>b17117db72da867328bfee7e7b5ac7c17acc0aab</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC131" s="21" t="str">
         <x:v>En cours</x:v>
@@ -12257,10 +12257,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA132" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB132" s="21" t="str">
-        <x:v>e03821783020a61aeaaa58d22886e2118781efaa</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC132" s="21" t="str">
         <x:v>En cours</x:v>
@@ -12348,10 +12348,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA133" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB133" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC133" s="21" t="str">
         <x:v>En cours</x:v>
@@ -12439,10 +12439,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA134" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB134" s="21" t="str">
-        <x:v>b17117db72da867328bfee7e7b5ac7c17acc0aab</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC134" s="21" t="str">
         <x:v>En cours</x:v>
@@ -12530,10 +12530,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA135" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB135" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC135" s="21" t="str">
         <x:v>En cours</x:v>
@@ -12621,10 +12621,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA136" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB136" s="21" t="str">
-        <x:v>e03821783020a61aeaaa58d22886e2118781efaa</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC136" s="21" t="str">
         <x:v>En cours</x:v>
@@ -12712,10 +12712,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA137" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB137" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC137" s="21" t="str">
         <x:v>En cours</x:v>
@@ -12803,10 +12803,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA138" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB138" s="21" t="str">
-        <x:v>3eadba5f121c1017c032929534d269c330aa5abb</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC138" s="21" t="str">
         <x:v>En cours</x:v>
@@ -12894,10 +12894,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA139" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB139" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC139" s="21" t="str">
         <x:v>En cours</x:v>
@@ -12985,10 +12985,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA140" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB140" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC140" s="21" t="str">
         <x:v>En cours</x:v>
@@ -13076,10 +13076,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA141" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB141" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC141" s="21" t="str">
         <x:v>En cours</x:v>
@@ -13167,10 +13167,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA142" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB142" s="21" t="str">
-        <x:v>e03821783020a61aeaaa58d22886e2118781efaa</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC142" s="21" t="str">
         <x:v>En cours</x:v>
@@ -13258,10 +13258,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA143" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB143" s="21" t="str">
-        <x:v>b17117db72da867328bfee7e7b5ac7c17acc0aab</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC143" s="21" t="str">
         <x:v>En cours</x:v>
@@ -13349,10 +13349,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA144" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB144" s="21" t="str">
-        <x:v>e03821783020a61aeaaa58d22886e2118781efaa</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC144" s="21" t="str">
         <x:v>En cours</x:v>
@@ -13440,10 +13440,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA145" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB145" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC145" s="21" t="str">
         <x:v>En cours</x:v>
@@ -13531,10 +13531,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA146" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB146" s="21" t="str">
-        <x:v>e03821783020a61aeaaa58d22886e2118781efaa</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC146" s="21" t="str">
         <x:v>En cours</x:v>
@@ -13622,10 +13622,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA147" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB147" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC147" s="21" t="str">
         <x:v>En cours</x:v>
@@ -13713,10 +13713,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA148" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB148" s="21" t="str">
-        <x:v>e03821783020a61aeaaa58d22886e2118781efaa</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC148" s="21" t="str">
         <x:v>En cours</x:v>
@@ -13804,10 +13804,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA149" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB149" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC149" s="21" t="str">
         <x:v>En cours</x:v>
@@ -13895,10 +13895,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA150" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB150" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC150" s="21" t="str">
         <x:v>En cours</x:v>
@@ -13986,10 +13986,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA151" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB151" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC151" s="21" t="str">
         <x:v>En cours</x:v>
@@ -14077,10 +14077,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA152" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB152" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC152" s="21" t="str">
         <x:v>En cours</x:v>
@@ -14168,10 +14168,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA153" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB153" s="21" t="str">
-        <x:v>e03821783020a61aeaaa58d22886e2118781efaa</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC153" s="21" t="str">
         <x:v>En cours</x:v>
@@ -14259,10 +14259,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA154" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB154" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC154" s="21" t="str">
         <x:v>En cours</x:v>
@@ -14350,10 +14350,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA155" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB155" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC155" s="21" t="str">
         <x:v>En cours</x:v>
@@ -14441,10 +14441,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA156" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB156" s="21" t="str">
-        <x:v>b17117db72da867328bfee7e7b5ac7c17acc0aab</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC156" s="21" t="str">
         <x:v>En cours</x:v>
@@ -14532,10 +14532,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA157" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB157" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC157" s="21" t="str">
         <x:v>En cours</x:v>
@@ -14623,10 +14623,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA158" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB158" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC158" s="21" t="str">
         <x:v>En cours</x:v>
@@ -14714,10 +14714,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA159" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB159" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC159" s="21" t="str">
         <x:v>En cours</x:v>
@@ -14805,10 +14805,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA160" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB160" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC160" s="21" t="str">
         <x:v>En cours</x:v>
@@ -14896,10 +14896,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA161" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB161" s="21" t="str">
-        <x:v>b17117db72da867328bfee7e7b5ac7c17acc0aab</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC161" s="21" t="str">
         <x:v>En cours</x:v>
@@ -14987,10 +14987,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA162" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB162" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC162" s="21" t="str">
         <x:v>En cours</x:v>
@@ -15078,10 +15078,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA163" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB163" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC163" s="21" t="str">
         <x:v>En cours</x:v>
@@ -15169,10 +15169,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA164" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB164" s="21" t="str">
-        <x:v>e03821783020a61aeaaa58d22886e2118781efaa</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC164" s="21" t="str">
         <x:v>En cours</x:v>
@@ -15260,10 +15260,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA165" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB165" s="21" t="str">
-        <x:v>e03821783020a61aeaaa58d22886e2118781efaa</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC165" s="21" t="str">
         <x:v>En cours</x:v>
@@ -15351,10 +15351,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA166" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB166" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC166" s="21" t="str">
         <x:v>En cours</x:v>
@@ -15442,10 +15442,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA167" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB167" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC167" s="21" t="str">
         <x:v>En cours</x:v>
@@ -15533,10 +15533,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA168" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB168" s="21" t="str">
-        <x:v>b17117db72da867328bfee7e7b5ac7c17acc0aab</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC168" s="21" t="str">
         <x:v>En cours</x:v>
@@ -15624,10 +15624,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA169" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB169" s="21" t="str">
-        <x:v>b17117db72da867328bfee7e7b5ac7c17acc0aab</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC169" s="21" t="str">
         <x:v>En cours</x:v>
@@ -15715,10 +15715,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA170" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB170" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC170" s="21" t="str">
         <x:v>En cours</x:v>
@@ -15806,10 +15806,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA171" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB171" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC171" s="21" t="str">
         <x:v>En cours</x:v>
@@ -15897,10 +15897,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA172" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB172" s="21" t="str">
-        <x:v>e03821783020a61aeaaa58d22886e2118781efaa</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC172" s="21" t="str">
         <x:v>En cours</x:v>
@@ -15988,10 +15988,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA173" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB173" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC173" s="21" t="str">
         <x:v>En cours</x:v>
@@ -16079,10 +16079,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA174" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB174" s="21" t="str">
-        <x:v>b17117db72da867328bfee7e7b5ac7c17acc0aab</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC174" s="21" t="str">
         <x:v>En cours</x:v>
@@ -16170,10 +16170,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA175" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB175" s="21" t="str">
-        <x:v>b17117db72da867328bfee7e7b5ac7c17acc0aab</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC175" s="21" t="str">
         <x:v>En cours</x:v>
@@ -16261,10 +16261,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA176" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB176" s="21" t="str">
-        <x:v>b17117db72da867328bfee7e7b5ac7c17acc0aab</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC176" s="21" t="str">
         <x:v>En cours</x:v>
@@ -16352,10 +16352,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA177" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB177" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC177" s="21" t="str">
         <x:v>En cours</x:v>
@@ -16443,10 +16443,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA178" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB178" s="21" t="str">
-        <x:v>e03821783020a61aeaaa58d22886e2118781efaa</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC178" s="21" t="str">
         <x:v>En cours</x:v>
@@ -16534,10 +16534,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA179" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB179" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC179" s="21" t="str">
         <x:v>En cours</x:v>
@@ -16625,10 +16625,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA180" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB180" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC180" s="21" t="str">
         <x:v>En cours</x:v>
@@ -16716,10 +16716,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA181" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB181" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC181" s="21" t="str">
         <x:v>En cours</x:v>
@@ -16807,10 +16807,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA182" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB182" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC182" s="21" t="str">
         <x:v>En cours</x:v>
@@ -16898,10 +16898,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA183" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB183" s="21" t="str">
-        <x:v>e03821783020a61aeaaa58d22886e2118781efaa</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC183" s="21" t="str">
         <x:v>En cours</x:v>
@@ -16989,10 +16989,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA184" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB184" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC184" s="21" t="str">
         <x:v>En cours</x:v>
@@ -17023,7 +17023,7 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="H185" s="24" t="str">
-        <x:v>Réutilisé master #509</x:v>
+        <x:v>Archive Drive</x:v>
       </x:c>
       <x:c r="I185" s="24" t="str">
         <x:v>Présent</x:v>
@@ -17080,10 +17080,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA185" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB185" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC185" s="21" t="str">
         <x:v>En cours</x:v>
@@ -17171,10 +17171,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA186" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB186" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC186" s="21" t="str">
         <x:v>En cours</x:v>
@@ -17262,10 +17262,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA187" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB187" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC187" s="21" t="str">
         <x:v>En cours</x:v>
@@ -17353,10 +17353,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA188" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB188" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC188" s="21" t="str">
         <x:v>En cours</x:v>
@@ -17444,10 +17444,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA189" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB189" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC189" s="21" t="str">
         <x:v>En cours</x:v>
@@ -17535,10 +17535,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA190" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB190" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC190" s="21" t="str">
         <x:v>En cours</x:v>
@@ -17626,10 +17626,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA191" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB191" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC191" s="21" t="str">
         <x:v>En cours</x:v>
@@ -17717,10 +17717,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA192" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB192" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC192" s="21" t="str">
         <x:v>En cours</x:v>
@@ -17808,10 +17808,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA193" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB193" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC193" s="21" t="str">
         <x:v>En cours</x:v>
@@ -17899,10 +17899,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA194" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB194" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC194" s="21" t="str">
         <x:v>En cours</x:v>
@@ -17990,10 +17990,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA195" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB195" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC195" s="21" t="str">
         <x:v>En cours</x:v>
@@ -18081,10 +18081,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA196" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB196" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC196" s="21" t="str">
         <x:v>En cours</x:v>
@@ -18172,10 +18172,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA197" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB197" s="21" t="str">
-        <x:v>3eadba5f121c1017c032929534d269c330aa5abb</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC197" s="21" t="str">
         <x:v>En cours</x:v>
@@ -18263,10 +18263,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA198" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB198" s="21" t="str">
-        <x:v>b17117db72da867328bfee7e7b5ac7c17acc0aab</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC198" s="21" t="str">
         <x:v>En cours</x:v>
@@ -18354,10 +18354,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA199" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB199" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC199" s="21" t="str">
         <x:v>En cours</x:v>
@@ -18445,10 +18445,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA200" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB200" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC200" s="21" t="str">
         <x:v>En cours</x:v>
@@ -18536,10 +18536,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA201" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB201" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC201" s="21" t="str">
         <x:v>En cours</x:v>
@@ -18627,10 +18627,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA202" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB202" s="21" t="str">
-        <x:v>e03821783020a61aeaaa58d22886e2118781efaa</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC202" s="21" t="str">
         <x:v>En cours</x:v>
@@ -18718,10 +18718,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA203" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB203" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC203" s="21" t="str">
         <x:v>En cours</x:v>
@@ -18809,10 +18809,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA204" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB204" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC204" s="21" t="str">
         <x:v>En cours</x:v>
@@ -18900,10 +18900,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA205" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB205" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC205" s="21" t="str">
         <x:v>En cours</x:v>
@@ -18991,10 +18991,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA206" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB206" s="21" t="str">
-        <x:v>e03821783020a61aeaaa58d22886e2118781efaa</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC206" s="21" t="str">
         <x:v>En cours</x:v>
@@ -19082,10 +19082,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA207" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB207" s="21" t="str">
-        <x:v>e03821783020a61aeaaa58d22886e2118781efaa</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC207" s="21" t="str">
         <x:v>En cours</x:v>
@@ -19173,10 +19173,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA208" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB208" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC208" s="21" t="str">
         <x:v>En cours</x:v>
@@ -19264,10 +19264,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA209" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB209" s="21" t="str">
-        <x:v>b17117db72da867328bfee7e7b5ac7c17acc0aab</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC209" s="21" t="str">
         <x:v>En cours</x:v>
@@ -19355,10 +19355,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA210" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB210" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC210" s="21" t="str">
         <x:v>En cours</x:v>
@@ -19446,10 +19446,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA211" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB211" s="21" t="str">
-        <x:v>3eadba5f121c1017c032929534d269c330aa5abb</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC211" s="21" t="str">
         <x:v>En cours</x:v>
@@ -19537,10 +19537,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA212" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB212" s="21" t="str">
-        <x:v>3eadba5f121c1017c032929534d269c330aa5abb</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC212" s="21" t="str">
         <x:v>En cours</x:v>
@@ -19628,10 +19628,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA213" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB213" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC213" s="21" t="str">
         <x:v>En cours</x:v>
@@ -19719,10 +19719,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA214" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB214" s="21" t="str">
-        <x:v>e03821783020a61aeaaa58d22886e2118781efaa</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC214" s="21" t="str">
         <x:v>En cours</x:v>
@@ -19810,10 +19810,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA215" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB215" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC215" s="21" t="str">
         <x:v>En cours</x:v>
@@ -19901,10 +19901,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA216" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB216" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC216" s="21" t="str">
         <x:v>En cours</x:v>
@@ -19992,10 +19992,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA217" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB217" s="21" t="str">
-        <x:v>b17117db72da867328bfee7e7b5ac7c17acc0aab</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC217" s="21" t="str">
         <x:v>En cours</x:v>
@@ -20083,10 +20083,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA218" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB218" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC218" s="21" t="str">
         <x:v>En cours</x:v>
@@ -20174,10 +20174,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA219" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB219" s="21" t="str">
-        <x:v>b17117db72da867328bfee7e7b5ac7c17acc0aab</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC219" s="21" t="str">
         <x:v>En cours</x:v>
@@ -20265,10 +20265,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA220" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB220" s="21" t="str">
-        <x:v>b17117db72da867328bfee7e7b5ac7c17acc0aab</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC220" s="21" t="str">
         <x:v>En cours</x:v>
@@ -20356,10 +20356,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA221" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB221" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC221" s="21" t="str">
         <x:v>En cours</x:v>
@@ -20447,10 +20447,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA222" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB222" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC222" s="21" t="str">
         <x:v>En cours</x:v>
@@ -20538,10 +20538,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA223" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB223" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC223" s="21" t="str">
         <x:v>En cours</x:v>
@@ -20629,10 +20629,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA224" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB224" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC224" s="21" t="str">
         <x:v>En cours</x:v>
@@ -20720,10 +20720,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA225" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB225" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC225" s="21" t="str">
         <x:v>En cours</x:v>
@@ -20811,10 +20811,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA226" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB226" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC226" s="21" t="str">
         <x:v>En cours</x:v>
@@ -20902,10 +20902,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA227" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB227" s="21" t="str">
-        <x:v>e03821783020a61aeaaa58d22886e2118781efaa</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC227" s="21" t="str">
         <x:v>En cours</x:v>
@@ -20993,10 +20993,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA228" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB228" s="21" t="str">
-        <x:v>e03821783020a61aeaaa58d22886e2118781efaa</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC228" s="21" t="str">
         <x:v>En cours</x:v>
@@ -21084,10 +21084,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA229" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB229" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC229" s="21" t="str">
         <x:v>En cours</x:v>
@@ -21175,10 +21175,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA230" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB230" s="21" t="str">
-        <x:v>e03821783020a61aeaaa58d22886e2118781efaa</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC230" s="21" t="str">
         <x:v>En cours</x:v>
@@ -21266,10 +21266,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA231" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB231" s="21" t="str">
-        <x:v>e03821783020a61aeaaa58d22886e2118781efaa</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC231" s="21" t="str">
         <x:v>En cours</x:v>
@@ -21357,10 +21357,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA232" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB232" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC232" s="21" t="str">
         <x:v>En cours</x:v>
@@ -21448,10 +21448,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA233" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB233" s="21" t="str">
-        <x:v>3eadba5f121c1017c032929534d269c330aa5abb</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC233" s="21" t="str">
         <x:v>En cours</x:v>
@@ -21539,10 +21539,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA234" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB234" s="21" t="str">
-        <x:v>b17117db72da867328bfee7e7b5ac7c17acc0aab</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC234" s="21" t="str">
         <x:v>En cours</x:v>
@@ -21630,10 +21630,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA235" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB235" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC235" s="21" t="str">
         <x:v>En cours</x:v>
@@ -21721,10 +21721,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA236" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB236" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC236" s="21" t="str">
         <x:v>En cours</x:v>
@@ -21812,10 +21812,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA237" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB237" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC237" s="21" t="str">
         <x:v>En cours</x:v>
@@ -21903,10 +21903,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA238" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB238" s="21" t="str">
-        <x:v>e03821783020a61aeaaa58d22886e2118781efaa</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC238" s="21" t="str">
         <x:v>En cours</x:v>
@@ -21994,10 +21994,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA239" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB239" s="21" t="str">
-        <x:v>b17117db72da867328bfee7e7b5ac7c17acc0aab</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC239" s="21" t="str">
         <x:v>En cours</x:v>
@@ -22085,10 +22085,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA240" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB240" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC240" s="21" t="str">
         <x:v>En cours</x:v>
@@ -22176,10 +22176,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA241" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB241" s="21" t="str">
-        <x:v>e03821783020a61aeaaa58d22886e2118781efaa</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC241" s="21" t="str">
         <x:v>En cours</x:v>
@@ -22267,10 +22267,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA242" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB242" s="21" t="str">
-        <x:v>e03821783020a61aeaaa58d22886e2118781efaa</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC242" s="21" t="str">
         <x:v>En cours</x:v>
@@ -22358,10 +22358,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA243" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB243" s="21" t="str">
-        <x:v>b17117db72da867328bfee7e7b5ac7c17acc0aab</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC243" s="21" t="str">
         <x:v>En cours</x:v>
@@ -22449,10 +22449,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA244" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB244" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC244" s="21" t="str">
         <x:v>En cours</x:v>
@@ -22540,10 +22540,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA245" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB245" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC245" s="21" t="str">
         <x:v>En cours</x:v>
@@ -22631,10 +22631,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA246" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB246" s="21" t="str">
-        <x:v>b17117db72da867328bfee7e7b5ac7c17acc0aab</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC246" s="21" t="str">
         <x:v>En cours</x:v>
@@ -22665,7 +22665,7 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="H247" s="24" t="str">
-        <x:v>Réutilisé master #509</x:v>
+        <x:v>Archive Drive</x:v>
       </x:c>
       <x:c r="I247" s="24" t="str">
         <x:v>Présent</x:v>
@@ -22722,10 +22722,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA247" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB247" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC247" s="21" t="str">
         <x:v>En cours</x:v>
@@ -22813,10 +22813,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA248" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB248" s="21" t="str">
-        <x:v>e03821783020a61aeaaa58d22886e2118781efaa</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC248" s="21" t="str">
         <x:v>En cours</x:v>
@@ -22904,10 +22904,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA249" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB249" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC249" s="21" t="str">
         <x:v>En cours</x:v>
@@ -22995,10 +22995,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA250" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB250" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC250" s="21" t="str">
         <x:v>En cours</x:v>
@@ -23094,7 +23094,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2543f6d651e84bc1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7f35598b33e1450e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs(symbols): record full 240-pack site qualification and source backup (#549)
</commit_message>
<xml_diff>
--- a/doc_web_interne/docs/suivi-symboles/suivi-240-symboles-6-langues.xlsx
+++ b/doc_web_interne/docs/suivi-symboles/suivi-240-symboles-6-langues.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Suivi symboles" sheetId="1" r:id="Rf4cc105cee8b402e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Suivi symboles" sheetId="1" r:id="R1952b03bb8c94b9f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -811,7 +811,7 @@
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="7" t="str">
-        <x:v>Lot 14 en branche : 10 couvertures conservées, 70 nouveaux PNG. Preuves antérieures inchangées conservées.</x:v>
+        <x:v>240 packs intégrés dans les six langues. Validation actuelle ; publication assurée par Thanh.</x:v>
       </x:c>
       <x:c r="B3" s="7"/>
       <x:c r="C3" s="7"/>
@@ -980,7 +980,7 @@
     </x:row>
     <x:row r="7" ht="20" customHeight="1">
       <x:c r="A7" s="7" t="str">
-        <x:v>240 packs ; 0 à compléter. Cadre commun : 1 440 pages. Publication antérieure conservée dans les reçus.</x:v>
+        <x:v>240 packs, 1 440 pages. Sources originales des six packs retrouvées et sauvegardées sur Drive.</x:v>
       </x:c>
       <x:c r="B7" s="7"/>
       <x:c r="C7" s="7"/>
@@ -1013,7 +1013,7 @@
     </x:row>
     <x:row r="8" ht="20" customHeight="1">
       <x:c r="A8" s="7" t="str">
-        <x:v>Source : rapport canonique actuel, empreinte 88509a9cc8e5e634. Révision : 3eadba5f121c1017c032929534d269c330aa5abb</x:v>
+        <x:v>Source : rapport canonique 5f96fe5298e47cda. Révision : 674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="B8" s="7"/>
       <x:c r="C8" s="7"/>
@@ -1246,10 +1246,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA11" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB11" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC11" s="21" t="str">
         <x:v>En cours</x:v>
@@ -1337,10 +1337,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA12" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB12" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC12" s="21" t="str">
         <x:v>En cours</x:v>
@@ -1428,10 +1428,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA13" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB13" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC13" s="21" t="str">
         <x:v>En cours</x:v>
@@ -1519,10 +1519,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA14" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB14" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC14" s="21" t="str">
         <x:v>En cours</x:v>
@@ -1610,10 +1610,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA15" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB15" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC15" s="21" t="str">
         <x:v>En cours</x:v>
@@ -1701,10 +1701,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA16" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB16" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC16" s="21" t="str">
         <x:v>En cours</x:v>
@@ -1792,10 +1792,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA17" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB17" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC17" s="21" t="str">
         <x:v>En cours</x:v>
@@ -1883,10 +1883,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA18" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB18" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC18" s="21" t="str">
         <x:v>En cours</x:v>
@@ -1974,10 +1974,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA19" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB19" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC19" s="21" t="str">
         <x:v>En cours</x:v>
@@ -2065,10 +2065,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA20" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB20" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC20" s="21" t="str">
         <x:v>En cours</x:v>
@@ -2156,10 +2156,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA21" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB21" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC21" s="21" t="str">
         <x:v>En cours</x:v>
@@ -2247,10 +2247,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA22" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB22" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC22" s="21" t="str">
         <x:v>En cours</x:v>
@@ -2338,10 +2338,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA23" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB23" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC23" s="21" t="str">
         <x:v>En cours</x:v>
@@ -2429,10 +2429,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA24" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB24" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC24" s="21" t="str">
         <x:v>En cours</x:v>
@@ -2520,10 +2520,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA25" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB25" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC25" s="21" t="str">
         <x:v>En cours</x:v>
@@ -2611,10 +2611,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA26" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB26" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC26" s="21" t="str">
         <x:v>En cours</x:v>
@@ -2702,10 +2702,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA27" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB27" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC27" s="21" t="str">
         <x:v>En cours</x:v>
@@ -2793,10 +2793,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA28" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB28" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC28" s="21" t="str">
         <x:v>En cours</x:v>
@@ -2884,10 +2884,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA29" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB29" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC29" s="21" t="str">
         <x:v>En cours</x:v>
@@ -2975,10 +2975,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA30" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB30" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC30" s="21" t="str">
         <x:v>En cours</x:v>
@@ -3066,10 +3066,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA31" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB31" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC31" s="21" t="str">
         <x:v>En cours</x:v>
@@ -3157,10 +3157,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA32" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB32" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC32" s="21" t="str">
         <x:v>En cours</x:v>
@@ -3248,10 +3248,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA33" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB33" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC33" s="21" t="str">
         <x:v>En cours</x:v>
@@ -3339,10 +3339,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA34" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB34" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC34" s="21" t="str">
         <x:v>En cours</x:v>
@@ -3430,10 +3430,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA35" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB35" s="21" t="str">
-        <x:v>e03821783020a61aeaaa58d22886e2118781efaa</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC35" s="21" t="str">
         <x:v>En cours</x:v>
@@ -3521,10 +3521,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA36" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB36" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC36" s="21" t="str">
         <x:v>En cours</x:v>
@@ -3555,7 +3555,7 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="H37" s="24" t="str">
-        <x:v>Réutilisé master #509</x:v>
+        <x:v>Archive Drive</x:v>
       </x:c>
       <x:c r="I37" s="24" t="str">
         <x:v>Présent</x:v>
@@ -3612,10 +3612,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA37" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB37" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC37" s="21" t="str">
         <x:v>En cours</x:v>
@@ -3703,10 +3703,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA38" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB38" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC38" s="21" t="str">
         <x:v>En cours</x:v>
@@ -3794,10 +3794,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA39" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB39" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC39" s="21" t="str">
         <x:v>En cours</x:v>
@@ -3885,10 +3885,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA40" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB40" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC40" s="21" t="str">
         <x:v>En cours</x:v>
@@ -3976,10 +3976,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA41" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB41" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC41" s="21" t="str">
         <x:v>En cours</x:v>
@@ -4067,10 +4067,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA42" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB42" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC42" s="21" t="str">
         <x:v>En cours</x:v>
@@ -4158,10 +4158,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA43" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB43" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC43" s="21" t="str">
         <x:v>En cours</x:v>
@@ -4249,10 +4249,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA44" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB44" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC44" s="21" t="str">
         <x:v>En cours</x:v>
@@ -4340,10 +4340,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA45" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB45" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC45" s="21" t="str">
         <x:v>En cours</x:v>
@@ -4431,10 +4431,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA46" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB46" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC46" s="21" t="str">
         <x:v>En cours</x:v>
@@ -4522,10 +4522,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA47" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB47" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC47" s="21" t="str">
         <x:v>En cours</x:v>
@@ -4613,10 +4613,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA48" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB48" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC48" s="21" t="str">
         <x:v>En cours</x:v>
@@ -4704,10 +4704,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA49" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB49" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC49" s="21" t="str">
         <x:v>En cours</x:v>
@@ -4795,10 +4795,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA50" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB50" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC50" s="21" t="str">
         <x:v>En cours</x:v>
@@ -4886,10 +4886,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA51" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB51" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC51" s="21" t="str">
         <x:v>En cours</x:v>
@@ -4977,10 +4977,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA52" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB52" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC52" s="21" t="str">
         <x:v>En cours</x:v>
@@ -5068,10 +5068,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA53" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB53" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC53" s="21" t="str">
         <x:v>En cours</x:v>
@@ -5159,10 +5159,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA54" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB54" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC54" s="21" t="str">
         <x:v>En cours</x:v>
@@ -5250,10 +5250,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA55" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB55" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC55" s="21" t="str">
         <x:v>En cours</x:v>
@@ -5341,10 +5341,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA56" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB56" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC56" s="21" t="str">
         <x:v>En cours</x:v>
@@ -5432,10 +5432,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA57" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB57" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC57" s="21" t="str">
         <x:v>En cours</x:v>
@@ -5523,10 +5523,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA58" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB58" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC58" s="21" t="str">
         <x:v>En cours</x:v>
@@ -5614,10 +5614,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA59" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB59" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC59" s="21" t="str">
         <x:v>En cours</x:v>
@@ -5705,10 +5705,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA60" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB60" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC60" s="21" t="str">
         <x:v>En cours</x:v>
@@ -5796,10 +5796,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA61" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB61" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC61" s="21" t="str">
         <x:v>En cours</x:v>
@@ -5887,10 +5887,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA62" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB62" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC62" s="21" t="str">
         <x:v>En cours</x:v>
@@ -5978,10 +5978,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA63" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB63" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC63" s="21" t="str">
         <x:v>En cours</x:v>
@@ -6069,10 +6069,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA64" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB64" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC64" s="21" t="str">
         <x:v>En cours</x:v>
@@ -6160,10 +6160,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA65" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB65" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC65" s="21" t="str">
         <x:v>En cours</x:v>
@@ -6251,10 +6251,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA66" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB66" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC66" s="21" t="str">
         <x:v>En cours</x:v>
@@ -6342,10 +6342,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA67" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB67" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC67" s="21" t="str">
         <x:v>En cours</x:v>
@@ -6433,10 +6433,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA68" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB68" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC68" s="21" t="str">
         <x:v>En cours</x:v>
@@ -6524,10 +6524,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA69" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB69" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC69" s="21" t="str">
         <x:v>En cours</x:v>
@@ -6615,10 +6615,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA70" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB70" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC70" s="21" t="str">
         <x:v>En cours</x:v>
@@ -6706,10 +6706,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA71" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB71" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC71" s="21" t="str">
         <x:v>En cours</x:v>
@@ -6797,10 +6797,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA72" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB72" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC72" s="21" t="str">
         <x:v>En cours</x:v>
@@ -6888,10 +6888,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA73" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB73" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC73" s="21" t="str">
         <x:v>En cours</x:v>
@@ -6979,10 +6979,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA74" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB74" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC74" s="21" t="str">
         <x:v>En cours</x:v>
@@ -7070,10 +7070,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA75" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB75" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC75" s="21" t="str">
         <x:v>En cours</x:v>
@@ -7161,10 +7161,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA76" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB76" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC76" s="21" t="str">
         <x:v>En cours</x:v>
@@ -7252,10 +7252,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA77" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB77" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC77" s="21" t="str">
         <x:v>En cours</x:v>
@@ -7343,10 +7343,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA78" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB78" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC78" s="21" t="str">
         <x:v>En cours</x:v>
@@ -7434,10 +7434,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA79" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB79" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC79" s="21" t="str">
         <x:v>En cours</x:v>
@@ -7525,10 +7525,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA80" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB80" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC80" s="21" t="str">
         <x:v>En cours</x:v>
@@ -7616,10 +7616,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA81" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB81" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC81" s="21" t="str">
         <x:v>En cours</x:v>
@@ -7707,10 +7707,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA82" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB82" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC82" s="21" t="str">
         <x:v>En cours</x:v>
@@ -7798,10 +7798,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA83" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB83" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC83" s="21" t="str">
         <x:v>En cours</x:v>
@@ -7889,10 +7889,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA84" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB84" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC84" s="21" t="str">
         <x:v>En cours</x:v>
@@ -7980,10 +7980,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA85" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB85" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC85" s="21" t="str">
         <x:v>En cours</x:v>
@@ -8071,10 +8071,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA86" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB86" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC86" s="21" t="str">
         <x:v>En cours</x:v>
@@ -8162,10 +8162,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA87" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB87" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC87" s="21" t="str">
         <x:v>En cours</x:v>
@@ -8253,10 +8253,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA88" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB88" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC88" s="21" t="str">
         <x:v>En cours</x:v>
@@ -8344,10 +8344,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA89" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB89" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC89" s="21" t="str">
         <x:v>En cours</x:v>
@@ -8378,7 +8378,7 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="H90" s="24" t="str">
-        <x:v>Réutilisé master #509</x:v>
+        <x:v>Archive Drive</x:v>
       </x:c>
       <x:c r="I90" s="24" t="str">
         <x:v>Présent</x:v>
@@ -8435,10 +8435,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA90" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB90" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC90" s="21" t="str">
         <x:v>En cours</x:v>
@@ -8526,10 +8526,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA91" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB91" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC91" s="21" t="str">
         <x:v>En cours</x:v>
@@ -8617,10 +8617,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA92" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB92" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC92" s="21" t="str">
         <x:v>En cours</x:v>
@@ -8708,10 +8708,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA93" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB93" s="21" t="str">
-        <x:v>b17117db72da867328bfee7e7b5ac7c17acc0aab</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC93" s="21" t="str">
         <x:v>En cours</x:v>
@@ -8799,10 +8799,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA94" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB94" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC94" s="21" t="str">
         <x:v>En cours</x:v>
@@ -8890,10 +8890,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA95" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB95" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC95" s="21" t="str">
         <x:v>En cours</x:v>
@@ -8981,10 +8981,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA96" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB96" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC96" s="21" t="str">
         <x:v>En cours</x:v>
@@ -9072,10 +9072,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA97" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB97" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC97" s="21" t="str">
         <x:v>En cours</x:v>
@@ -9163,10 +9163,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA98" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB98" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC98" s="21" t="str">
         <x:v>En cours</x:v>
@@ -9254,10 +9254,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA99" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB99" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC99" s="21" t="str">
         <x:v>En cours</x:v>
@@ -9345,10 +9345,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA100" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB100" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC100" s="21" t="str">
         <x:v>En cours</x:v>
@@ -9436,10 +9436,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA101" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB101" s="21" t="str">
-        <x:v>3eadba5f121c1017c032929534d269c330aa5abb</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC101" s="21" t="str">
         <x:v>En cours</x:v>
@@ -9527,10 +9527,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA102" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB102" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC102" s="21" t="str">
         <x:v>En cours</x:v>
@@ -9561,7 +9561,7 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="H103" s="24" t="str">
-        <x:v>Réutilisé master #509</x:v>
+        <x:v>Archive Drive</x:v>
       </x:c>
       <x:c r="I103" s="24" t="str">
         <x:v>Présent</x:v>
@@ -9618,10 +9618,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA103" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB103" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC103" s="21" t="str">
         <x:v>En cours</x:v>
@@ -9709,10 +9709,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA104" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB104" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC104" s="21" t="str">
         <x:v>En cours</x:v>
@@ -9800,10 +9800,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA105" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB105" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC105" s="21" t="str">
         <x:v>En cours</x:v>
@@ -9891,10 +9891,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA106" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB106" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC106" s="21" t="str">
         <x:v>En cours</x:v>
@@ -9982,10 +9982,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA107" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB107" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC107" s="21" t="str">
         <x:v>En cours</x:v>
@@ -10073,10 +10073,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA108" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB108" s="21" t="str">
-        <x:v>b17117db72da867328bfee7e7b5ac7c17acc0aab</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC108" s="21" t="str">
         <x:v>En cours</x:v>
@@ -10164,10 +10164,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA109" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB109" s="21" t="str">
-        <x:v>b17117db72da867328bfee7e7b5ac7c17acc0aab</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC109" s="21" t="str">
         <x:v>En cours</x:v>
@@ -10198,7 +10198,7 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="H110" s="24" t="str">
-        <x:v>Réutilisé master #509</x:v>
+        <x:v>Archive Drive</x:v>
       </x:c>
       <x:c r="I110" s="24" t="str">
         <x:v>Présent</x:v>
@@ -10255,10 +10255,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA110" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB110" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC110" s="21" t="str">
         <x:v>En cours</x:v>
@@ -10346,10 +10346,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA111" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB111" s="21" t="str">
-        <x:v>e03821783020a61aeaaa58d22886e2118781efaa</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC111" s="21" t="str">
         <x:v>En cours</x:v>
@@ -10437,10 +10437,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA112" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB112" s="21" t="str">
-        <x:v>b17117db72da867328bfee7e7b5ac7c17acc0aab</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC112" s="21" t="str">
         <x:v>En cours</x:v>
@@ -10528,10 +10528,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA113" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB113" s="21" t="str">
-        <x:v>3eadba5f121c1017c032929534d269c330aa5abb</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC113" s="21" t="str">
         <x:v>En cours</x:v>
@@ -10619,10 +10619,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA114" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB114" s="21" t="str">
-        <x:v>e03821783020a61aeaaa58d22886e2118781efaa</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC114" s="21" t="str">
         <x:v>En cours</x:v>
@@ -10710,10 +10710,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA115" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB115" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC115" s="21" t="str">
         <x:v>En cours</x:v>
@@ -10801,10 +10801,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA116" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB116" s="21" t="str">
-        <x:v>b17117db72da867328bfee7e7b5ac7c17acc0aab</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC116" s="21" t="str">
         <x:v>En cours</x:v>
@@ -10892,10 +10892,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA117" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB117" s="21" t="str">
-        <x:v>e03821783020a61aeaaa58d22886e2118781efaa</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC117" s="21" t="str">
         <x:v>En cours</x:v>
@@ -10983,10 +10983,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA118" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB118" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC118" s="21" t="str">
         <x:v>En cours</x:v>
@@ -11074,10 +11074,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA119" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB119" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC119" s="21" t="str">
         <x:v>En cours</x:v>
@@ -11165,10 +11165,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA120" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB120" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC120" s="21" t="str">
         <x:v>En cours</x:v>
@@ -11256,10 +11256,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA121" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB121" s="21" t="str">
-        <x:v>3eadba5f121c1017c032929534d269c330aa5abb</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC121" s="21" t="str">
         <x:v>En cours</x:v>
@@ -11347,10 +11347,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA122" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB122" s="21" t="str">
-        <x:v>e03821783020a61aeaaa58d22886e2118781efaa</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC122" s="21" t="str">
         <x:v>En cours</x:v>
@@ -11438,10 +11438,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA123" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB123" s="21" t="str">
-        <x:v>3eadba5f121c1017c032929534d269c330aa5abb</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC123" s="21" t="str">
         <x:v>En cours</x:v>
@@ -11529,10 +11529,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA124" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB124" s="21" t="str">
-        <x:v>e03821783020a61aeaaa58d22886e2118781efaa</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC124" s="21" t="str">
         <x:v>En cours</x:v>
@@ -11620,10 +11620,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA125" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB125" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC125" s="21" t="str">
         <x:v>En cours</x:v>
@@ -11711,10 +11711,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA126" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB126" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC126" s="21" t="str">
         <x:v>En cours</x:v>
@@ -11802,10 +11802,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA127" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB127" s="21" t="str">
-        <x:v>b17117db72da867328bfee7e7b5ac7c17acc0aab</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC127" s="21" t="str">
         <x:v>En cours</x:v>
@@ -11893,10 +11893,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA128" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB128" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC128" s="21" t="str">
         <x:v>En cours</x:v>
@@ -11984,10 +11984,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA129" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB129" s="21" t="str">
-        <x:v>3eadba5f121c1017c032929534d269c330aa5abb</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC129" s="21" t="str">
         <x:v>En cours</x:v>
@@ -12075,10 +12075,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA130" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB130" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC130" s="21" t="str">
         <x:v>En cours</x:v>
@@ -12166,10 +12166,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA131" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB131" s="21" t="str">
-        <x:v>b17117db72da867328bfee7e7b5ac7c17acc0aab</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC131" s="21" t="str">
         <x:v>En cours</x:v>
@@ -12257,10 +12257,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA132" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB132" s="21" t="str">
-        <x:v>e03821783020a61aeaaa58d22886e2118781efaa</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC132" s="21" t="str">
         <x:v>En cours</x:v>
@@ -12348,10 +12348,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA133" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB133" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC133" s="21" t="str">
         <x:v>En cours</x:v>
@@ -12439,10 +12439,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA134" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB134" s="21" t="str">
-        <x:v>b17117db72da867328bfee7e7b5ac7c17acc0aab</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC134" s="21" t="str">
         <x:v>En cours</x:v>
@@ -12530,10 +12530,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA135" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB135" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC135" s="21" t="str">
         <x:v>En cours</x:v>
@@ -12621,10 +12621,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA136" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB136" s="21" t="str">
-        <x:v>e03821783020a61aeaaa58d22886e2118781efaa</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC136" s="21" t="str">
         <x:v>En cours</x:v>
@@ -12712,10 +12712,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA137" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB137" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC137" s="21" t="str">
         <x:v>En cours</x:v>
@@ -12803,10 +12803,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA138" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB138" s="21" t="str">
-        <x:v>3eadba5f121c1017c032929534d269c330aa5abb</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC138" s="21" t="str">
         <x:v>En cours</x:v>
@@ -12894,10 +12894,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA139" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB139" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC139" s="21" t="str">
         <x:v>En cours</x:v>
@@ -12985,10 +12985,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA140" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB140" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC140" s="21" t="str">
         <x:v>En cours</x:v>
@@ -13076,10 +13076,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA141" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB141" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC141" s="21" t="str">
         <x:v>En cours</x:v>
@@ -13167,10 +13167,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA142" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB142" s="21" t="str">
-        <x:v>e03821783020a61aeaaa58d22886e2118781efaa</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC142" s="21" t="str">
         <x:v>En cours</x:v>
@@ -13258,10 +13258,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA143" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB143" s="21" t="str">
-        <x:v>b17117db72da867328bfee7e7b5ac7c17acc0aab</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC143" s="21" t="str">
         <x:v>En cours</x:v>
@@ -13349,10 +13349,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA144" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB144" s="21" t="str">
-        <x:v>e03821783020a61aeaaa58d22886e2118781efaa</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC144" s="21" t="str">
         <x:v>En cours</x:v>
@@ -13440,10 +13440,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA145" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB145" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC145" s="21" t="str">
         <x:v>En cours</x:v>
@@ -13531,10 +13531,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA146" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB146" s="21" t="str">
-        <x:v>e03821783020a61aeaaa58d22886e2118781efaa</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC146" s="21" t="str">
         <x:v>En cours</x:v>
@@ -13622,10 +13622,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA147" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB147" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC147" s="21" t="str">
         <x:v>En cours</x:v>
@@ -13713,10 +13713,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA148" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB148" s="21" t="str">
-        <x:v>e03821783020a61aeaaa58d22886e2118781efaa</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC148" s="21" t="str">
         <x:v>En cours</x:v>
@@ -13804,10 +13804,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA149" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB149" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC149" s="21" t="str">
         <x:v>En cours</x:v>
@@ -13895,10 +13895,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA150" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB150" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC150" s="21" t="str">
         <x:v>En cours</x:v>
@@ -13986,10 +13986,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA151" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB151" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC151" s="21" t="str">
         <x:v>En cours</x:v>
@@ -14077,10 +14077,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA152" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB152" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC152" s="21" t="str">
         <x:v>En cours</x:v>
@@ -14168,10 +14168,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA153" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB153" s="21" t="str">
-        <x:v>e03821783020a61aeaaa58d22886e2118781efaa</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC153" s="21" t="str">
         <x:v>En cours</x:v>
@@ -14259,10 +14259,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA154" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB154" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC154" s="21" t="str">
         <x:v>En cours</x:v>
@@ -14350,10 +14350,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA155" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB155" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC155" s="21" t="str">
         <x:v>En cours</x:v>
@@ -14441,10 +14441,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA156" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB156" s="21" t="str">
-        <x:v>b17117db72da867328bfee7e7b5ac7c17acc0aab</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC156" s="21" t="str">
         <x:v>En cours</x:v>
@@ -14532,10 +14532,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA157" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB157" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC157" s="21" t="str">
         <x:v>En cours</x:v>
@@ -14623,10 +14623,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA158" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB158" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC158" s="21" t="str">
         <x:v>En cours</x:v>
@@ -14714,10 +14714,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA159" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB159" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC159" s="21" t="str">
         <x:v>En cours</x:v>
@@ -14805,10 +14805,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA160" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB160" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC160" s="21" t="str">
         <x:v>En cours</x:v>
@@ -14896,10 +14896,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA161" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB161" s="21" t="str">
-        <x:v>b17117db72da867328bfee7e7b5ac7c17acc0aab</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC161" s="21" t="str">
         <x:v>En cours</x:v>
@@ -14987,10 +14987,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA162" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB162" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC162" s="21" t="str">
         <x:v>En cours</x:v>
@@ -15078,10 +15078,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA163" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB163" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC163" s="21" t="str">
         <x:v>En cours</x:v>
@@ -15169,10 +15169,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA164" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB164" s="21" t="str">
-        <x:v>e03821783020a61aeaaa58d22886e2118781efaa</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC164" s="21" t="str">
         <x:v>En cours</x:v>
@@ -15260,10 +15260,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA165" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB165" s="21" t="str">
-        <x:v>e03821783020a61aeaaa58d22886e2118781efaa</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC165" s="21" t="str">
         <x:v>En cours</x:v>
@@ -15351,10 +15351,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA166" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB166" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC166" s="21" t="str">
         <x:v>En cours</x:v>
@@ -15442,10 +15442,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA167" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB167" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC167" s="21" t="str">
         <x:v>En cours</x:v>
@@ -15533,10 +15533,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA168" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB168" s="21" t="str">
-        <x:v>b17117db72da867328bfee7e7b5ac7c17acc0aab</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC168" s="21" t="str">
         <x:v>En cours</x:v>
@@ -15624,10 +15624,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA169" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB169" s="21" t="str">
-        <x:v>b17117db72da867328bfee7e7b5ac7c17acc0aab</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC169" s="21" t="str">
         <x:v>En cours</x:v>
@@ -15715,10 +15715,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA170" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB170" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC170" s="21" t="str">
         <x:v>En cours</x:v>
@@ -15806,10 +15806,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA171" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB171" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC171" s="21" t="str">
         <x:v>En cours</x:v>
@@ -15897,10 +15897,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA172" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB172" s="21" t="str">
-        <x:v>e03821783020a61aeaaa58d22886e2118781efaa</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC172" s="21" t="str">
         <x:v>En cours</x:v>
@@ -15988,10 +15988,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA173" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB173" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC173" s="21" t="str">
         <x:v>En cours</x:v>
@@ -16079,10 +16079,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA174" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB174" s="21" t="str">
-        <x:v>b17117db72da867328bfee7e7b5ac7c17acc0aab</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC174" s="21" t="str">
         <x:v>En cours</x:v>
@@ -16170,10 +16170,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA175" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB175" s="21" t="str">
-        <x:v>b17117db72da867328bfee7e7b5ac7c17acc0aab</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC175" s="21" t="str">
         <x:v>En cours</x:v>
@@ -16261,10 +16261,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA176" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB176" s="21" t="str">
-        <x:v>b17117db72da867328bfee7e7b5ac7c17acc0aab</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC176" s="21" t="str">
         <x:v>En cours</x:v>
@@ -16352,10 +16352,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA177" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB177" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC177" s="21" t="str">
         <x:v>En cours</x:v>
@@ -16443,10 +16443,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA178" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB178" s="21" t="str">
-        <x:v>e03821783020a61aeaaa58d22886e2118781efaa</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC178" s="21" t="str">
         <x:v>En cours</x:v>
@@ -16534,10 +16534,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA179" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB179" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC179" s="21" t="str">
         <x:v>En cours</x:v>
@@ -16625,10 +16625,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA180" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB180" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC180" s="21" t="str">
         <x:v>En cours</x:v>
@@ -16716,10 +16716,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA181" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB181" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC181" s="21" t="str">
         <x:v>En cours</x:v>
@@ -16807,10 +16807,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA182" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB182" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC182" s="21" t="str">
         <x:v>En cours</x:v>
@@ -16898,10 +16898,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA183" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB183" s="21" t="str">
-        <x:v>e03821783020a61aeaaa58d22886e2118781efaa</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC183" s="21" t="str">
         <x:v>En cours</x:v>
@@ -16989,10 +16989,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA184" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB184" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC184" s="21" t="str">
         <x:v>En cours</x:v>
@@ -17023,7 +17023,7 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="H185" s="24" t="str">
-        <x:v>Réutilisé master #509</x:v>
+        <x:v>Archive Drive</x:v>
       </x:c>
       <x:c r="I185" s="24" t="str">
         <x:v>Présent</x:v>
@@ -17080,10 +17080,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA185" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB185" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC185" s="21" t="str">
         <x:v>En cours</x:v>
@@ -17171,10 +17171,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA186" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB186" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC186" s="21" t="str">
         <x:v>En cours</x:v>
@@ -17262,10 +17262,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA187" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB187" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC187" s="21" t="str">
         <x:v>En cours</x:v>
@@ -17353,10 +17353,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA188" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB188" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC188" s="21" t="str">
         <x:v>En cours</x:v>
@@ -17444,10 +17444,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA189" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB189" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC189" s="21" t="str">
         <x:v>En cours</x:v>
@@ -17535,10 +17535,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA190" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB190" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC190" s="21" t="str">
         <x:v>En cours</x:v>
@@ -17626,10 +17626,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA191" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB191" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC191" s="21" t="str">
         <x:v>En cours</x:v>
@@ -17717,10 +17717,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA192" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB192" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC192" s="21" t="str">
         <x:v>En cours</x:v>
@@ -17808,10 +17808,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA193" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB193" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC193" s="21" t="str">
         <x:v>En cours</x:v>
@@ -17899,10 +17899,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA194" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB194" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC194" s="21" t="str">
         <x:v>En cours</x:v>
@@ -17990,10 +17990,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA195" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB195" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC195" s="21" t="str">
         <x:v>En cours</x:v>
@@ -18081,10 +18081,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA196" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB196" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC196" s="21" t="str">
         <x:v>En cours</x:v>
@@ -18172,10 +18172,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA197" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB197" s="21" t="str">
-        <x:v>3eadba5f121c1017c032929534d269c330aa5abb</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC197" s="21" t="str">
         <x:v>En cours</x:v>
@@ -18263,10 +18263,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA198" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB198" s="21" t="str">
-        <x:v>b17117db72da867328bfee7e7b5ac7c17acc0aab</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC198" s="21" t="str">
         <x:v>En cours</x:v>
@@ -18354,10 +18354,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA199" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB199" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC199" s="21" t="str">
         <x:v>En cours</x:v>
@@ -18445,10 +18445,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA200" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB200" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC200" s="21" t="str">
         <x:v>En cours</x:v>
@@ -18536,10 +18536,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA201" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB201" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC201" s="21" t="str">
         <x:v>En cours</x:v>
@@ -18627,10 +18627,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA202" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB202" s="21" t="str">
-        <x:v>e03821783020a61aeaaa58d22886e2118781efaa</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC202" s="21" t="str">
         <x:v>En cours</x:v>
@@ -18718,10 +18718,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA203" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB203" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC203" s="21" t="str">
         <x:v>En cours</x:v>
@@ -18809,10 +18809,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA204" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB204" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC204" s="21" t="str">
         <x:v>En cours</x:v>
@@ -18900,10 +18900,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA205" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB205" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC205" s="21" t="str">
         <x:v>En cours</x:v>
@@ -18991,10 +18991,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA206" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB206" s="21" t="str">
-        <x:v>e03821783020a61aeaaa58d22886e2118781efaa</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC206" s="21" t="str">
         <x:v>En cours</x:v>
@@ -19082,10 +19082,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA207" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB207" s="21" t="str">
-        <x:v>e03821783020a61aeaaa58d22886e2118781efaa</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC207" s="21" t="str">
         <x:v>En cours</x:v>
@@ -19173,10 +19173,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA208" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB208" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC208" s="21" t="str">
         <x:v>En cours</x:v>
@@ -19264,10 +19264,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA209" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB209" s="21" t="str">
-        <x:v>b17117db72da867328bfee7e7b5ac7c17acc0aab</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC209" s="21" t="str">
         <x:v>En cours</x:v>
@@ -19355,10 +19355,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA210" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB210" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC210" s="21" t="str">
         <x:v>En cours</x:v>
@@ -19446,10 +19446,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA211" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB211" s="21" t="str">
-        <x:v>3eadba5f121c1017c032929534d269c330aa5abb</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC211" s="21" t="str">
         <x:v>En cours</x:v>
@@ -19537,10 +19537,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA212" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB212" s="21" t="str">
-        <x:v>3eadba5f121c1017c032929534d269c330aa5abb</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC212" s="21" t="str">
         <x:v>En cours</x:v>
@@ -19628,10 +19628,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA213" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB213" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC213" s="21" t="str">
         <x:v>En cours</x:v>
@@ -19719,10 +19719,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA214" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB214" s="21" t="str">
-        <x:v>e03821783020a61aeaaa58d22886e2118781efaa</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC214" s="21" t="str">
         <x:v>En cours</x:v>
@@ -19810,10 +19810,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA215" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB215" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC215" s="21" t="str">
         <x:v>En cours</x:v>
@@ -19901,10 +19901,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA216" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB216" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC216" s="21" t="str">
         <x:v>En cours</x:v>
@@ -19992,10 +19992,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA217" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB217" s="21" t="str">
-        <x:v>b17117db72da867328bfee7e7b5ac7c17acc0aab</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC217" s="21" t="str">
         <x:v>En cours</x:v>
@@ -20083,10 +20083,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA218" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB218" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC218" s="21" t="str">
         <x:v>En cours</x:v>
@@ -20174,10 +20174,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA219" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB219" s="21" t="str">
-        <x:v>b17117db72da867328bfee7e7b5ac7c17acc0aab</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC219" s="21" t="str">
         <x:v>En cours</x:v>
@@ -20265,10 +20265,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA220" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB220" s="21" t="str">
-        <x:v>b17117db72da867328bfee7e7b5ac7c17acc0aab</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC220" s="21" t="str">
         <x:v>En cours</x:v>
@@ -20356,10 +20356,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA221" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB221" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC221" s="21" t="str">
         <x:v>En cours</x:v>
@@ -20447,10 +20447,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA222" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB222" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC222" s="21" t="str">
         <x:v>En cours</x:v>
@@ -20538,10 +20538,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA223" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB223" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC223" s="21" t="str">
         <x:v>En cours</x:v>
@@ -20629,10 +20629,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA224" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB224" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC224" s="21" t="str">
         <x:v>En cours</x:v>
@@ -20720,10 +20720,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA225" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB225" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC225" s="21" t="str">
         <x:v>En cours</x:v>
@@ -20811,10 +20811,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA226" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB226" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC226" s="21" t="str">
         <x:v>En cours</x:v>
@@ -20902,10 +20902,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA227" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB227" s="21" t="str">
-        <x:v>e03821783020a61aeaaa58d22886e2118781efaa</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC227" s="21" t="str">
         <x:v>En cours</x:v>
@@ -20993,10 +20993,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA228" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB228" s="21" t="str">
-        <x:v>e03821783020a61aeaaa58d22886e2118781efaa</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC228" s="21" t="str">
         <x:v>En cours</x:v>
@@ -21084,10 +21084,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA229" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB229" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC229" s="21" t="str">
         <x:v>En cours</x:v>
@@ -21175,10 +21175,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA230" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB230" s="21" t="str">
-        <x:v>e03821783020a61aeaaa58d22886e2118781efaa</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC230" s="21" t="str">
         <x:v>En cours</x:v>
@@ -21266,10 +21266,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA231" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB231" s="21" t="str">
-        <x:v>e03821783020a61aeaaa58d22886e2118781efaa</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC231" s="21" t="str">
         <x:v>En cours</x:v>
@@ -21357,10 +21357,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA232" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB232" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC232" s="21" t="str">
         <x:v>En cours</x:v>
@@ -21448,10 +21448,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA233" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB233" s="21" t="str">
-        <x:v>3eadba5f121c1017c032929534d269c330aa5abb</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC233" s="21" t="str">
         <x:v>En cours</x:v>
@@ -21539,10 +21539,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA234" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB234" s="21" t="str">
-        <x:v>b17117db72da867328bfee7e7b5ac7c17acc0aab</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC234" s="21" t="str">
         <x:v>En cours</x:v>
@@ -21630,10 +21630,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA235" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB235" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC235" s="21" t="str">
         <x:v>En cours</x:v>
@@ -21721,10 +21721,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA236" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB236" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC236" s="21" t="str">
         <x:v>En cours</x:v>
@@ -21812,10 +21812,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA237" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB237" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC237" s="21" t="str">
         <x:v>En cours</x:v>
@@ -21903,10 +21903,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA238" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB238" s="21" t="str">
-        <x:v>e03821783020a61aeaaa58d22886e2118781efaa</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC238" s="21" t="str">
         <x:v>En cours</x:v>
@@ -21994,10 +21994,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA239" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB239" s="21" t="str">
-        <x:v>b17117db72da867328bfee7e7b5ac7c17acc0aab</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC239" s="21" t="str">
         <x:v>En cours</x:v>
@@ -22085,10 +22085,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA240" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB240" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC240" s="21" t="str">
         <x:v>En cours</x:v>
@@ -22176,10 +22176,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA241" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB241" s="21" t="str">
-        <x:v>e03821783020a61aeaaa58d22886e2118781efaa</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC241" s="21" t="str">
         <x:v>En cours</x:v>
@@ -22267,10 +22267,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA242" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB242" s="21" t="str">
-        <x:v>e03821783020a61aeaaa58d22886e2118781efaa</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC242" s="21" t="str">
         <x:v>En cours</x:v>
@@ -22358,10 +22358,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA243" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB243" s="21" t="str">
-        <x:v>b17117db72da867328bfee7e7b5ac7c17acc0aab</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC243" s="21" t="str">
         <x:v>En cours</x:v>
@@ -22449,10 +22449,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA244" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB244" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC244" s="21" t="str">
         <x:v>En cours</x:v>
@@ -22540,10 +22540,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA245" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB245" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC245" s="21" t="str">
         <x:v>En cours</x:v>
@@ -22631,10 +22631,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA246" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB246" s="21" t="str">
-        <x:v>b17117db72da867328bfee7e7b5ac7c17acc0aab</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC246" s="21" t="str">
         <x:v>En cours</x:v>
@@ -22665,7 +22665,7 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="H247" s="24" t="str">
-        <x:v>Réutilisé master #509</x:v>
+        <x:v>Archive Drive</x:v>
       </x:c>
       <x:c r="I247" s="24" t="str">
         <x:v>Présent</x:v>
@@ -22722,10 +22722,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA247" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB247" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC247" s="21" t="str">
         <x:v>En cours</x:v>
@@ -22813,10 +22813,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA248" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB248" s="21" t="str">
-        <x:v>e03821783020a61aeaaa58d22886e2118781efaa</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC248" s="21" t="str">
         <x:v>En cours</x:v>
@@ -22904,10 +22904,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA249" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB249" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC249" s="21" t="str">
         <x:v>En cours</x:v>
@@ -22995,10 +22995,10 @@
         <x:v>Périmée (0/6)</x:v>
       </x:c>
       <x:c r="AA250" s="23" t="str">
-        <x:v>QA actuelle. Accord non consigné ou périmé. Publication non consignée ou périmée.</x:v>
+        <x:v>Validation navigateur passée. Publication exacte en attente de Thanh.</x:v>
       </x:c>
       <x:c r="AB250" s="21" t="str">
-        <x:v>34209f968444db816f75779cd5b876df002ae9d3</x:v>
+        <x:v>674f752f62b3179c8a21300c7796024f5935efc1</x:v>
       </x:c>
       <x:c r="AC250" s="21" t="str">
         <x:v>En cours</x:v>
@@ -23094,7 +23094,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2543f6d651e84bc1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7f35598b33e1450e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>